<commit_message>
Safety backup in view of slob coding
</commit_message>
<xml_diff>
--- a/DegreeTests.xlsx
+++ b/DegreeTests.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Source\VS22\ProjExcel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7754A4F-2AC4-466D-A557-C73FB9A03364}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB4FB558-D1FD-4027-A410-D94FFDC86B72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38290" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -45976,10 +45976,10 @@
     <row r="128" spans="1:18" x14ac:dyDescent="0.35">
       <c r="M128"/>
     </row>
-    <row r="129" spans="3:13" x14ac:dyDescent="0.35">
+    <row r="129" spans="3:17" x14ac:dyDescent="0.35">
       <c r="M129"/>
     </row>
-    <row r="130" spans="3:13" x14ac:dyDescent="0.35">
+    <row r="130" spans="3:17" x14ac:dyDescent="0.35">
       <c r="C130" s="173" t="s">
         <v>136</v>
       </c>
@@ -45989,7 +45989,7 @@
       </c>
       <c r="M130"/>
     </row>
-    <row r="131" spans="3:13" x14ac:dyDescent="0.35">
+    <row r="131" spans="3:17" x14ac:dyDescent="0.35">
       <c r="C131" s="12" t="s">
         <v>137</v>
       </c>
@@ -45999,7 +45999,7 @@
       </c>
       <c r="M131"/>
     </row>
-    <row r="132" spans="3:13" x14ac:dyDescent="0.35">
+    <row r="132" spans="3:17" x14ac:dyDescent="0.35">
       <c r="C132" t="s">
         <v>138</v>
       </c>
@@ -46133,14 +46133,14 @@
       </c>
       <c r="M132"/>
     </row>
-    <row r="133" spans="3:13" x14ac:dyDescent="0.35">
+    <row r="133" spans="3:17" x14ac:dyDescent="0.35">
       <c r="D133" s="172" t="str" cm="1">
         <f t="array" ref="D133">_xll.PE.crs.AsProjString(D4)</f>
         <v>+proj=tmerc +lat_0=0 +lon_0=21 +k=1 +x_0=4500000 +y_0=0 +ellps=krass +units=m +no_defs +type=crs</v>
       </c>
       <c r="M133"/>
     </row>
-    <row r="134" spans="3:13" x14ac:dyDescent="0.35">
+    <row r="134" spans="3:17" x14ac:dyDescent="0.35">
       <c r="D134" s="172" t="str" cm="1">
         <f t="array" ref="D134">_xll.PE.crs.AsWktString(D4)</f>
         <v>PROJCRS["Albanian 1987 / Gauss-Kruger zone 4 (with axis order normalized for visualization)",
@@ -46187,33 +46187,50 @@
       </c>
       <c r="M134"/>
     </row>
-    <row r="135" spans="3:13" x14ac:dyDescent="0.35">
+    <row r="135" spans="3:17" x14ac:dyDescent="0.35">
       <c r="D135" s="174" t="str" cm="1">
         <f t="array" ref="D135">_xll.PE.crs.Axis.Abbreviation(D4,0,TRUE)</f>
         <v>Y</v>
       </c>
       <c r="M135"/>
     </row>
-    <row r="136" spans="3:13" x14ac:dyDescent="0.35">
+    <row r="136" spans="3:17" x14ac:dyDescent="0.35">
       <c r="D136" s="174" cm="1">
         <f t="array" ref="D136">_xll.PE.crs.Axis.Count(D4,TRUE)</f>
         <v>2</v>
       </c>
       <c r="M136"/>
     </row>
-    <row r="137" spans="3:13" x14ac:dyDescent="0.35">
+    <row r="137" spans="3:17" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="M137"/>
     </row>
-    <row r="138" spans="3:13" x14ac:dyDescent="0.35">
-      <c r="M138"/>
-    </row>
-    <row r="139" spans="3:13" x14ac:dyDescent="0.35">
+    <row r="138" spans="3:17" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="C138" s="182" t="str" cm="1">
+        <f t="array" ref="C138">_xll.PE.trf.Options2()</f>
+        <v>Authority=EPSG; Accuracy=; Area=; NoBallparkConversions=False; NoDiscardIfMissing=False; UsePrimaryGridNames=False; UseSuperseded=False; AllowDeprecatedCrs=False; StrictContains=False; IntermediateCrsUsage=Auto; CandidateIndex=0; BestOnly=False; ForceOver=False</v>
+      </c>
+      <c r="D138" s="183"/>
+      <c r="E138" s="183"/>
+      <c r="F138" s="183"/>
+      <c r="G138" s="183"/>
+      <c r="H138" s="183"/>
+      <c r="I138" s="183"/>
+      <c r="J138" s="183"/>
+      <c r="K138" s="183"/>
+      <c r="L138" s="183"/>
+      <c r="M138" s="183"/>
+      <c r="N138" s="183"/>
+      <c r="O138" s="205"/>
+      <c r="P138" s="183"/>
+      <c r="Q138" s="184"/>
+    </row>
+    <row r="139" spans="3:17" x14ac:dyDescent="0.35">
       <c r="M139"/>
     </row>
-    <row r="140" spans="3:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="140" spans="3:17" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="M140"/>
     </row>
-    <row r="141" spans="3:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="141" spans="3:17" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C141" s="182" t="str" cm="1">
         <f t="array" ref="C141:G143">_xll.PE.xfm.ListTransformPipelines($D$4,$D$5)</f>
         <v>PipelineID</v>
@@ -46236,7 +46253,7 @@
       <c r="K141" s="61"/>
       <c r="M141"/>
     </row>
-    <row r="142" spans="3:13" x14ac:dyDescent="0.35">
+    <row r="142" spans="3:17" x14ac:dyDescent="0.35">
       <c r="C142" s="199">
         <v>1</v>
       </c>
@@ -46255,7 +46272,7 @@
       <c r="K142" s="61"/>
       <c r="M142"/>
     </row>
-    <row r="143" spans="3:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="143" spans="3:17" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C143" s="201">
         <v>2</v>
       </c>
@@ -46274,7 +46291,7 @@
       <c r="K143" s="61"/>
       <c r="M143"/>
     </row>
-    <row r="144" spans="3:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="144" spans="3:17" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="K144" s="61"/>
       <c r="M144"/>
     </row>

</xml_diff>

<commit_message>
Safety push. You never know what your agent is upto.
</commit_message>
<xml_diff>
--- a/DegreeTests.xlsx
+++ b/DegreeTests.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Source\VS22\ProjExcel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB4FB558-D1FD-4027-A410-D94FFDC86B72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC8C95E4-1D27-45B0-96F1-0D90AFDD773D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38290" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -172,7 +172,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -194,7 +194,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="877" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="875" uniqueCount="142">
   <si>
     <t xml:space="preserve"> </t>
   </si>
@@ -618,12 +618,15 @@
   <si>
     <t>Transform options</t>
   </si>
+  <si>
+    <t xml:space="preserve"> CRS is deprecated</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="7">
+  <numFmts count="8">
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="#,##0.000000"/>
     <numFmt numFmtId="165" formatCode="#,##0.0000000"/>
@@ -631,6 +634,7 @@
     <numFmt numFmtId="167" formatCode="#,##0.0"/>
     <numFmt numFmtId="168" formatCode="0.000"/>
     <numFmt numFmtId="169" formatCode="0.0000"/>
+    <numFmt numFmtId="170" formatCode="0.0000E+00"/>
   </numFmts>
   <fonts count="14" x14ac:knownFonts="1">
     <font>
@@ -1199,7 +1203,7 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="13" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="210">
+  <cellXfs count="219">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1694,6 +1698,17 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="2" fontId="0" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="24" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="20" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="21" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="43" fontId="0" fillId="15" borderId="5" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="15" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="170" fontId="0" fillId="12" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="170" fontId="0" fillId="12" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Comma" xfId="3" builtinId="3"/>
@@ -1705,10 +1720,10 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FFCCFFFF"/>
+      <color rgb="FFFFFFCC"/>
       <color rgb="FF66FFFF"/>
       <color rgb="FF66CCFF"/>
-      <color rgb="FFCCFFFF"/>
-      <color rgb="FFFFFFCC"/>
       <color rgb="FFCCFFCC"/>
       <color rgb="FF0000FF"/>
     </mruColors>
@@ -39438,7 +39453,7 @@
     <col min="2" max="2" width="6.36328125" style="61" customWidth="1"/>
     <col min="3" max="3" width="25.7265625" customWidth="1"/>
     <col min="4" max="4" width="17.6328125" customWidth="1"/>
-    <col min="5" max="5" width="15" customWidth="1"/>
+    <col min="5" max="5" width="15.90625" customWidth="1"/>
     <col min="6" max="6" width="14.54296875" customWidth="1"/>
     <col min="7" max="7" width="13.36328125" customWidth="1"/>
     <col min="8" max="8" width="12.36328125" customWidth="1"/>
@@ -39463,19 +39478,18 @@
       <c r="D3" s="60" t="s">
         <v>27</v>
       </c>
-      <c r="E3" s="58" t="s">
+      <c r="E3" s="54" t="s">
+        <v>141</v>
+      </c>
+      <c r="F3" s="58" t="s">
         <v>28</v>
       </c>
-      <c r="F3" s="56"/>
       <c r="G3" s="56"/>
       <c r="H3" s="56"/>
       <c r="I3" s="56"/>
       <c r="J3" s="56"/>
       <c r="K3" s="56"/>
       <c r="L3" s="57"/>
-      <c r="M3" s="50" t="s">
-        <v>29</v>
-      </c>
     </row>
     <row r="4" spans="1:20" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C4" s="51" t="s">
@@ -39484,28 +39498,21 @@
       <c r="D4" s="49">
         <v>2462</v>
       </c>
-      <c r="E4" s="65" t="str" cm="1">
-        <f t="array" ref="E4">_xll.PE.crs.AsProjString(D4)</f>
+      <c r="E4" s="213" t="b" cm="1">
+        <f t="array" ref="E4">_xll.PE.crs.IsDeprecated(D4)</f>
+        <v>0</v>
+      </c>
+      <c r="F4" s="210" t="str" cm="1">
+        <f t="array" ref="F4">_xll.PE.crs.AsProjString(D4)</f>
         <v>+proj=tmerc +lat_0=0 +lon_0=21 +k=1 +x_0=4500000 +y_0=0 +ellps=krass +units=m +no_defs +type=crs</v>
       </c>
-      <c r="F4" s="66"/>
-      <c r="G4" s="66"/>
-      <c r="H4" s="66"/>
-      <c r="I4" s="66"/>
-      <c r="J4" s="66"/>
-      <c r="K4" s="66"/>
-      <c r="L4" s="67"/>
-      <c r="M4" s="50" t="s">
-        <v>17</v>
-      </c>
-      <c r="O4" s="166" cm="1">
-        <f t="array" ref="O4">_xll.PE.crs.UsageArea.Center.X(D4)</f>
-        <v>4426173.5325582689</v>
-      </c>
-      <c r="P4" s="167" cm="1">
-        <f t="array" ref="P4">_xll.PE.crs.UsageArea.Center.Y(D4)</f>
-        <v>4558658.032843451</v>
-      </c>
+      <c r="G4" s="211"/>
+      <c r="H4" s="211"/>
+      <c r="I4" s="211"/>
+      <c r="J4" s="211"/>
+      <c r="K4" s="211"/>
+      <c r="L4" s="212"/>
+      <c r="P4" s="167"/>
     </row>
     <row r="5" spans="1:20" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C5" s="52" t="s">
@@ -39514,20 +39521,20 @@
       <c r="D5" s="48">
         <v>4326</v>
       </c>
-      <c r="E5" s="62" t="str" cm="1">
-        <f t="array" ref="E5">_xll.PE.crs.AsProjString(D5)</f>
+      <c r="E5" s="213" t="b" cm="1">
+        <f t="array" ref="E5">_xll.PE.crs.IsDeprecated(D5)</f>
+        <v>0</v>
+      </c>
+      <c r="F5" s="182" t="str" cm="1">
+        <f t="array" ref="F5">_xll.PE.crs.AsProjString(D5)</f>
         <v>+proj=longlat +datum=WGS84 +no_defs +type=crs</v>
       </c>
-      <c r="F5" s="63"/>
-      <c r="G5" s="63"/>
-      <c r="H5" s="63"/>
-      <c r="I5" s="63"/>
-      <c r="J5" s="63"/>
-      <c r="K5" s="63"/>
-      <c r="L5" s="64"/>
-      <c r="M5" s="53" t="s">
-        <v>17</v>
-      </c>
+      <c r="G5" s="183"/>
+      <c r="H5" s="183"/>
+      <c r="I5" s="183"/>
+      <c r="J5" s="183"/>
+      <c r="K5" s="183"/>
+      <c r="L5" s="214"/>
     </row>
     <row r="6" spans="1:20" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="M6"/>
@@ -45538,36 +45545,36 @@
         <f>E119-$D$7*COS(RADIANS(O119))</f>
         <v>4452852.3097855086</v>
       </c>
-      <c r="F118" s="132" cm="1">
-        <f t="array" ref="F118:G118">_xll.PE.trf.FromEpsgNoToEpsgNo($D$4,$D$5,D118,E118)</f>
-        <v>20.155244386653319</v>
-      </c>
-      <c r="G118" s="134">
-        <v>40.205795085677487</v>
-      </c>
-      <c r="H118" s="132" t="str" cm="1">
+      <c r="F118" s="132" t="e" cm="1">
+        <f t="array" ref="F118:G118">_xll.PE.trf.ApplyForwardEx($D$4,$D$5,D118:E118,0,$C$127)</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="G118" s="134" t="e">
+        <v>#NUM!</v>
+      </c>
+      <c r="H118" s="132" t="e" cm="1">
         <f t="array" ref="H118">_xll.PE.deg.AsString(F118)</f>
-        <v>20 09 19</v>
-      </c>
-      <c r="I118" s="133" t="str" cm="1">
+        <v>#VALUE!</v>
+      </c>
+      <c r="I118" s="133" t="e" cm="1">
         <f t="array" ref="I118">_xll.PE.deg.AsString(G118)</f>
-        <v>40 12 21</v>
-      </c>
-      <c r="J118" s="132" cm="1">
+        <v>#VALUE!</v>
+      </c>
+      <c r="J118" s="132" t="e" cm="1">
         <f t="array" ref="J118">_xll.PE.deg.FromString(H118)</f>
-        <v>20.155277777777776</v>
-      </c>
-      <c r="K118" s="134" cm="1">
+        <v>#VALUE!</v>
+      </c>
+      <c r="K118" s="134" t="e" cm="1">
         <f t="array" ref="K118">_xll.PE.deg.FromString(I118)</f>
-        <v>40.205833333333338</v>
-      </c>
-      <c r="L118" s="83">
+        <v>#VALUE!</v>
+      </c>
+      <c r="L118" s="83" t="e">
         <f t="shared" ref="L118:M123" si="48">F118-J118</f>
-        <v>-3.3391124457438082E-5</v>
-      </c>
-      <c r="M118" s="79">
+        <v>#NUM!</v>
+      </c>
+      <c r="M118" s="79" t="e">
         <f t="shared" si="48"/>
-        <v>-3.824765585136447E-5</v>
+        <v>#NUM!</v>
       </c>
       <c r="N118" s="8">
         <f>SQRT((D119-D118)^2+(E119-E118)^2)</f>
@@ -45578,13 +45585,13 @@
         <v>54.497692329086064</v>
       </c>
       <c r="P118" s="94"/>
-      <c r="Q118" s="44" t="str">
+      <c r="Q118" s="44" t="e">
         <f t="shared" ref="Q118:Q123" si="49">CONCATENATE(TEXT(F118,"#.00000000"),",",TEXT(G118,"#.00000000"))</f>
-        <v>20.15524439,40.20579509</v>
-      </c>
-      <c r="R118" s="98" t="str">
+        <v>#NUM!</v>
+      </c>
+      <c r="R118" s="98" t="e">
         <f t="shared" ref="R118:R123" si="50">CONCATENATE("&lt;trkpt lon=""",TEXT(F118,"#.00000000"),""" lat=""",TEXT(G118,"#.00000000"),"""","&gt;&lt;name&gt;S",TEXT(B118,"00"),"&lt;/name&gt;&lt;/trkpt&gt;")</f>
-        <v>&lt;trkpt lon="20.15524439" lat="40.20579509"&gt;&lt;name&gt;S01&lt;/name&gt;&lt;/trkpt&gt;</v>
+        <v>#NUM!</v>
       </c>
     </row>
     <row r="119" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -45959,27 +45966,52 @@
         <v>19</v>
       </c>
     </row>
-    <row r="126" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="D126" s="198">
-        <f>AVERAGE(D16:D123)</f>
-        <v>4425866.9868022082</v>
-      </c>
-      <c r="E126" s="198">
-        <f>AVERAGE(E16:E123)</f>
-        <v>4471010.5922981566</v>
-      </c>
+    <row r="126" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="D126" s="198"/>
+      <c r="E126" s="198"/>
       <c r="M126"/>
     </row>
-    <row r="127" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="M127"/>
-    </row>
-    <row r="128" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="C127" s="182" t="str" cm="1">
+        <f t="array" ref="C127">_xll.PE.trf.Options(,,,,,1.01,,,,,,,,,1,)</f>
+        <v>Authority=EPSG; Area=; Accuracy=1.01; NoBallparkConversions=False; NoDiscardIfMissing=False; UsePrimaryGridNames=False; UseSuperseded=False; StrictContains=False; IntermediateCrsUsage=Auto; BestOnly=False; ForceOver=False; CandidateIndex=1; AllowDeprecatedCrs=False</v>
+      </c>
+      <c r="D127" s="183"/>
+      <c r="E127" s="183"/>
+      <c r="F127" s="183"/>
+      <c r="G127" s="183"/>
+      <c r="H127" s="183"/>
+      <c r="I127" s="183"/>
+      <c r="J127" s="183"/>
+      <c r="K127" s="183"/>
+      <c r="L127" s="183"/>
+      <c r="M127" s="183"/>
+      <c r="N127" s="183"/>
+      <c r="O127" s="205"/>
+      <c r="P127" s="183"/>
+      <c r="Q127" s="184"/>
+    </row>
+    <row r="128" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="M128"/>
     </row>
-    <row r="129" spans="3:17" x14ac:dyDescent="0.35">
+    <row r="129" spans="3:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="F129" s="182" cm="1">
+        <f t="array" ref="F129:G129">_xll.PE.trf.LatLongToWebMercatorEx(G123,F123,C127)</f>
+        <v>4488904.7260120427</v>
+      </c>
+      <c r="G129" s="184">
+        <v>2316761.8960968899</v>
+      </c>
+      <c r="I129" s="182" cm="1">
+        <f t="array" ref="I129:J129">_xll.PE.trf.LatLongToWebMercator(G123,F123)</f>
+        <v>2267435.056226131</v>
+      </c>
+      <c r="J129" s="184">
+        <v>4913212.9116666559</v>
+      </c>
       <c r="M129"/>
     </row>
-    <row r="130" spans="3:17" x14ac:dyDescent="0.35">
+    <row r="130" spans="3:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C130" s="173" t="s">
         <v>136</v>
       </c>
@@ -45987,9 +46019,21 @@
         <f t="array" ref="D130">_xll.PE.crs.GeodeticCRS.Name(D4)</f>
         <v>Albanian 1987</v>
       </c>
+      <c r="F130" s="215">
+        <v>2267435.056226131</v>
+      </c>
+      <c r="G130" s="216">
+        <v>4913212.9116666559</v>
+      </c>
+      <c r="I130" s="215">
+        <v>2267435.056226131</v>
+      </c>
+      <c r="J130" s="216">
+        <v>4913212.9116666559</v>
+      </c>
       <c r="M130"/>
     </row>
-    <row r="131" spans="3:17" x14ac:dyDescent="0.35">
+    <row r="131" spans="3:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C131" s="12" t="s">
         <v>137</v>
       </c>
@@ -45997,9 +46041,25 @@
         <f t="array" ref="D131">_xll.PE.crs.GeodeticCRS.Type(D4)</f>
         <v>Geographic2DCrs</v>
       </c>
+      <c r="F131" s="217">
+        <f>F129-F130</f>
+        <v>2221469.6697859117</v>
+      </c>
+      <c r="G131" s="218">
+        <f>G129-G130</f>
+        <v>-2596451.0155697661</v>
+      </c>
+      <c r="I131" s="217">
+        <f>I129-I130</f>
+        <v>0</v>
+      </c>
+      <c r="J131" s="218">
+        <f>J129-J130</f>
+        <v>0</v>
+      </c>
       <c r="M131"/>
     </row>
-    <row r="132" spans="3:17" x14ac:dyDescent="0.35">
+    <row r="132" spans="3:13" x14ac:dyDescent="0.35">
       <c r="C132" t="s">
         <v>138</v>
       </c>
@@ -46133,14 +46193,14 @@
       </c>
       <c r="M132"/>
     </row>
-    <row r="133" spans="3:17" x14ac:dyDescent="0.35">
+    <row r="133" spans="3:13" x14ac:dyDescent="0.35">
       <c r="D133" s="172" t="str" cm="1">
         <f t="array" ref="D133">_xll.PE.crs.AsProjString(D4)</f>
         <v>+proj=tmerc +lat_0=0 +lon_0=21 +k=1 +x_0=4500000 +y_0=0 +ellps=krass +units=m +no_defs +type=crs</v>
       </c>
       <c r="M133"/>
     </row>
-    <row r="134" spans="3:17" x14ac:dyDescent="0.35">
+    <row r="134" spans="3:13" x14ac:dyDescent="0.35">
       <c r="D134" s="172" t="str" cm="1">
         <f t="array" ref="D134">_xll.PE.crs.AsWktString(D4)</f>
         <v>PROJCRS["Albanian 1987 / Gauss-Kruger zone 4 (with axis order normalized for visualization)",
@@ -46187,50 +46247,30 @@
       </c>
       <c r="M134"/>
     </row>
-    <row r="135" spans="3:17" x14ac:dyDescent="0.35">
+    <row r="135" spans="3:13" x14ac:dyDescent="0.35">
       <c r="D135" s="174" t="str" cm="1">
         <f t="array" ref="D135">_xll.PE.crs.Axis.Abbreviation(D4,0,TRUE)</f>
         <v>Y</v>
       </c>
       <c r="M135"/>
     </row>
-    <row r="136" spans="3:17" x14ac:dyDescent="0.35">
+    <row r="136" spans="3:13" x14ac:dyDescent="0.35">
       <c r="D136" s="174" cm="1">
         <f t="array" ref="D136">_xll.PE.crs.Axis.Count(D4,TRUE)</f>
         <v>2</v>
       </c>
       <c r="M136"/>
     </row>
-    <row r="137" spans="3:17" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="137" spans="3:13" x14ac:dyDescent="0.35">
       <c r="M137"/>
     </row>
-    <row r="138" spans="3:17" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="C138" s="182" t="str" cm="1">
-        <f t="array" ref="C138">_xll.PE.trf.Options2()</f>
-        <v>Authority=EPSG; Accuracy=; Area=; NoBallparkConversions=False; NoDiscardIfMissing=False; UsePrimaryGridNames=False; UseSuperseded=False; AllowDeprecatedCrs=False; StrictContains=False; IntermediateCrsUsage=Auto; CandidateIndex=0; BestOnly=False; ForceOver=False</v>
-      </c>
-      <c r="D138" s="183"/>
-      <c r="E138" s="183"/>
-      <c r="F138" s="183"/>
-      <c r="G138" s="183"/>
-      <c r="H138" s="183"/>
-      <c r="I138" s="183"/>
-      <c r="J138" s="183"/>
-      <c r="K138" s="183"/>
-      <c r="L138" s="183"/>
-      <c r="M138" s="183"/>
-      <c r="N138" s="183"/>
-      <c r="O138" s="205"/>
-      <c r="P138" s="183"/>
-      <c r="Q138" s="184"/>
-    </row>
-    <row r="139" spans="3:17" x14ac:dyDescent="0.35">
+    <row r="139" spans="3:13" x14ac:dyDescent="0.35">
       <c r="M139"/>
     </row>
-    <row r="140" spans="3:17" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="140" spans="3:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="M140"/>
     </row>
-    <row r="141" spans="3:17" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="141" spans="3:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C141" s="182" t="str" cm="1">
         <f t="array" ref="C141:G143">_xll.PE.xfm.ListTransformPipelines($D$4,$D$5)</f>
         <v>PipelineID</v>
@@ -46253,7 +46293,7 @@
       <c r="K141" s="61"/>
       <c r="M141"/>
     </row>
-    <row r="142" spans="3:17" x14ac:dyDescent="0.35">
+    <row r="142" spans="3:13" x14ac:dyDescent="0.35">
       <c r="C142" s="199">
         <v>1</v>
       </c>
@@ -46272,7 +46312,7 @@
       <c r="K142" s="61"/>
       <c r="M142"/>
     </row>
-    <row r="143" spans="3:17" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="143" spans="3:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C143" s="201">
         <v>2</v>
       </c>
@@ -46291,7 +46331,7 @@
       <c r="K143" s="61"/>
       <c r="M143"/>
     </row>
-    <row r="144" spans="3:17" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="144" spans="3:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="K144" s="61"/>
       <c r="M144"/>
     </row>

</xml_diff>

<commit_message>
First reliable implementation of trf.Transform()
</commit_message>
<xml_diff>
--- a/DegreeTests.xlsx
+++ b/DegreeTests.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Source\VS22\ProjExcel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94F25A3F-A08A-4B5B-825D-2C1AA26364AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E954868-DF13-473D-9848-C4DD558A8D66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38290" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -194,7 +194,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="877" uniqueCount="144">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="880" uniqueCount="146">
   <si>
     <t xml:space="preserve"> </t>
   </si>
@@ -622,17 +622,23 @@
     <t xml:space="preserve"> CRS is deprecated</t>
   </si>
   <si>
-    <t>From</t>
+    <t>Source Crs</t>
   </si>
   <si>
-    <t>To</t>
+    <t>Target Crs</t>
+  </si>
+  <si>
+    <t>NAD27 / Alaska Albers</t>
+  </si>
+  <si>
+    <t>WGS 84</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="8">
+  <numFmts count="7">
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="#,##0.000000"/>
     <numFmt numFmtId="165" formatCode="#,##0.0000000"/>
@@ -640,9 +646,8 @@
     <numFmt numFmtId="167" formatCode="#,##0.0"/>
     <numFmt numFmtId="168" formatCode="0.000"/>
     <numFmt numFmtId="169" formatCode="0.0000"/>
-    <numFmt numFmtId="170" formatCode="0.0000E+00"/>
   </numFmts>
-  <fonts count="14" x14ac:knownFonts="1">
+  <fonts count="15" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -744,8 +749,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="7"/>
+      <color rgb="FFA31515"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
   </fonts>
-  <fills count="17">
+  <fills count="16">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -832,12 +843,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF66FFFF"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF66CCFF"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1209,7 +1214,7 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="13" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="220">
+  <cellXfs count="232">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1684,7 +1689,6 @@
     <xf numFmtId="4" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" indent="1"/>
     </xf>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
@@ -1696,8 +1700,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="2" fontId="0" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="15" borderId="24" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="15" borderId="20" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="15" borderId="21" xfId="0" applyFill="1" applyBorder="1"/>
@@ -1705,17 +1707,50 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="15" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="170" fontId="0" fillId="12" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="170" fontId="0" fillId="12" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="15" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="15" borderId="22" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="22" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="12" borderId="22" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Comma" xfId="3" builtinId="3"/>
@@ -1727,11 +1762,11 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
-      <color rgb="FF66CCFF"/>
+      <color rgb="FFCCFFFF"/>
       <color rgb="FF66FFFF"/>
       <color rgb="FFCCFFCC"/>
       <color rgb="FFFFFFCC"/>
-      <color rgb="FFCCFFFF"/>
+      <color rgb="FF66CCFF"/>
       <color rgb="FF0000FF"/>
     </mruColors>
   </colors>
@@ -39453,15 +39488,15 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E55C8259-B2F0-4599-98D4-024E12781605}">
-  <dimension ref="A2:T311"/>
+  <dimension ref="A2:T286"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="9" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="6.36328125" style="61" customWidth="1"/>
     <col min="3" max="3" width="32.7265625" customWidth="1"/>
     <col min="4" max="4" width="17.6328125" customWidth="1"/>
-    <col min="5" max="5" width="15.90625" customWidth="1"/>
-    <col min="6" max="6" width="14.54296875" customWidth="1"/>
+    <col min="5" max="5" width="16.1796875" customWidth="1"/>
+    <col min="6" max="6" width="15.54296875" customWidth="1"/>
     <col min="7" max="7" width="13.36328125" customWidth="1"/>
     <col min="8" max="8" width="12.36328125" customWidth="1"/>
     <col min="9" max="10" width="13.36328125" customWidth="1"/>
@@ -39505,20 +39540,20 @@
       <c r="D4" s="49">
         <v>2462</v>
       </c>
-      <c r="E4" s="211" t="b" cm="1">
+      <c r="E4" s="208" t="b" cm="1">
         <f t="array" ref="E4">_xll.PE.crs.IsDeprecated(D4)</f>
         <v>0</v>
       </c>
-      <c r="F4" s="208" t="str" cm="1">
+      <c r="F4" s="205" t="str" cm="1">
         <f t="array" ref="F4">_xll.PE.crs.AsProjString(D4)</f>
         <v>+proj=tmerc +lat_0=0 +lon_0=21 +k=1 +x_0=4500000 +y_0=0 +ellps=krass +units=m +no_defs +type=crs</v>
       </c>
-      <c r="G4" s="209"/>
-      <c r="H4" s="209"/>
-      <c r="I4" s="209"/>
-      <c r="J4" s="209"/>
-      <c r="K4" s="209"/>
-      <c r="L4" s="210"/>
+      <c r="G4" s="206"/>
+      <c r="H4" s="206"/>
+      <c r="I4" s="206"/>
+      <c r="J4" s="206"/>
+      <c r="K4" s="206"/>
+      <c r="L4" s="207"/>
       <c r="P4" s="167"/>
     </row>
     <row r="5" spans="1:20" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -39528,7 +39563,7 @@
       <c r="D5" s="48">
         <v>4326</v>
       </c>
-      <c r="E5" s="211" t="b" cm="1">
+      <c r="E5" s="208" t="b" cm="1">
         <f t="array" ref="E5">_xll.PE.crs.IsDeprecated(D5)</f>
         <v>0</v>
       </c>
@@ -39541,7 +39576,7 @@
       <c r="I5" s="183"/>
       <c r="J5" s="183"/>
       <c r="K5" s="183"/>
-      <c r="L5" s="212"/>
+      <c r="L5" s="209"/>
     </row>
     <row r="6" spans="1:20" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="M6"/>
@@ -39593,7 +39628,7 @@
         <v>File version</v>
       </c>
       <c r="E11" s="179" t="str">
-        <v>1.0.261016.1155</v>
+        <v>1.0.261019.1326</v>
       </c>
     </row>
     <row r="12" spans="1:20" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -39602,7 +39637,7 @@
         <v>Info version</v>
       </c>
       <c r="E12" s="181" t="str">
-        <v>1.0.261016.1155</v>
+        <v>1.0.261019.1326</v>
       </c>
       <c r="Q12" s="100" t="s">
         <v>44</v>
@@ -39612,13 +39647,13 @@
       </c>
     </row>
     <row r="13" spans="1:20" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="C13" s="43" t="s">
+      <c r="C13" s="55" t="s">
         <v>134</v>
       </c>
-      <c r="D13" s="180" t="str">
+      <c r="D13" s="178" t="str">
         <v>Proj version</v>
       </c>
-      <c r="E13" s="181" t="str">
+      <c r="E13" s="179" t="str">
         <v>9.5.1</v>
       </c>
       <c r="Q13" s="46" t="s">
@@ -39629,21 +39664,23 @@
       </c>
     </row>
     <row r="14" spans="1:20" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="C14" s="172" t="str" cm="1">
-        <f t="array" ref="C14">_xll.PE.trf.Options(0,0,0,0,0,0,"auto",0)</f>
+      <c r="C14" s="182" t="str" cm="1">
+        <f t="array" ref="C14">_xll.PE.trf.Options(0,0,0,0,0,0,"auto",0,,,,,,,,)</f>
         <v>Authority=0; Area=0,0,0,0; Accuracy=0; NoBallparkConversions=False; NoDiscardIfMissing=False; UsePrimaryGridNames=False; UseSuperseded=False; StrictContains=False; IntermediateCrsUsage=Auto; BestOnly=False; ForceOver=False; CandidateIndex=0; AllowDeprecatedCrs=False</v>
       </c>
-      <c r="D14" s="172"/>
-      <c r="E14" s="172"/>
-      <c r="F14" s="172"/>
-      <c r="G14" s="172"/>
-      <c r="H14" s="172"/>
-      <c r="I14" s="172"/>
-      <c r="J14" s="172"/>
-      <c r="K14" s="172"/>
-      <c r="L14" s="172"/>
-      <c r="M14" s="207"/>
-      <c r="N14" s="172"/>
+      <c r="D14" s="183"/>
+      <c r="E14" s="183"/>
+      <c r="F14" s="183"/>
+      <c r="G14" s="183"/>
+      <c r="H14" s="183"/>
+      <c r="I14" s="183"/>
+      <c r="J14" s="183"/>
+      <c r="K14" s="183"/>
+      <c r="L14" s="183"/>
+      <c r="M14" s="218"/>
+      <c r="N14" s="183"/>
+      <c r="O14" s="203"/>
+      <c r="P14" s="184"/>
       <c r="Q14" s="47" t="s">
         <v>20</v>
       </c>
@@ -39722,11 +39759,11 @@
         <f>E17-$D$7*COS(RADIANS(O17))</f>
         <v>4511477.2929155556</v>
       </c>
-      <c r="F16" s="132" cm="1">
-        <f t="array" ref="F16:G16">_xll.PE.trf.Transform($D$4,$D$5,D16,E16,C128)</f>
+      <c r="F16" s="135" cm="1">
+        <f t="array" ref="F16:G16">_xll.PE.trf.Transform($D$4,$D$5,D16,E16)</f>
         <v>19.627501288698802</v>
       </c>
-      <c r="G16" s="134">
+      <c r="G16" s="137">
         <v>40.728657406572829</v>
       </c>
       <c r="H16" s="135" t="str" cm="1">
@@ -39987,7 +40024,7 @@
         <v>4517571.1183339683</v>
       </c>
       <c r="F20" s="135" cm="1">
-        <f t="array" ref="F20:G20">_xll.PE.trf.FromEpsgNoToEpsgNo($D$4,$D$5,D20,E20)</f>
+        <f t="array" ref="F20:G20">_xll.PE.trf.Transform($D$4,$D$5,D20,E20)</f>
         <v>20.007599027220387</v>
       </c>
       <c r="G20" s="137">
@@ -40054,7 +40091,7 @@
         <v>4518129.2070844444</v>
       </c>
       <c r="F21" s="141" cm="1">
-        <f t="array" ref="F21:G21">_xll.PE.trf.FromEpsgNoToEpsgNo($D$4,$D$5,D21,E21)</f>
+        <f t="array" ref="F21:G21">_xll.PE.trf.Transform($D$4,$D$5,D21,E21)</f>
         <v>20.042444089865263</v>
       </c>
       <c r="G21" s="143">
@@ -40179,7 +40216,7 @@
         <v>4509248.2137425337</v>
       </c>
       <c r="F24" s="132" cm="1">
-        <f t="array" ref="F24:G24">_xll.PE.trf.FromEpsgNoToEpsgNo($D$4,$D$5,D24,E24)</f>
+        <f t="array" ref="F24:G24">_xll.PE.trf.Transform($D$4,$D$5,D24,E24)</f>
         <v>19.667912708680866</v>
       </c>
       <c r="G24" s="134">
@@ -40244,7 +40281,7 @@
         <v>4509971.1221385906</v>
       </c>
       <c r="F25" s="135" cm="1">
-        <f t="array" ref="F25:G25">_xll.PE.trf.FromEpsgNoToEpsgNo($D$4,$D$5,D25,E25)</f>
+        <f t="array" ref="F25:G25">_xll.PE.trf.Transform($D$4,$D$5,D25,E25)</f>
         <v>19.702232192676256</v>
       </c>
       <c r="G25" s="137">
@@ -40307,7 +40344,7 @@
         <v>4510935</v>
       </c>
       <c r="F26" s="138" cm="1">
-        <f t="array" ref="F26:G26">_xll.PE.trf.FromEpsgNoToEpsgNo($D$4,$D$5,D26,E26)</f>
+        <f t="array" ref="F26:G26">_xll.PE.trf.Transform($D$4,$D$5,D26,E26)</f>
         <v>19.748002911094968</v>
       </c>
       <c r="G26" s="140">
@@ -40372,7 +40409,7 @@
         <v>4513180</v>
       </c>
       <c r="F27" s="138" cm="1">
-        <f t="array" ref="F27:G27">_xll.PE.trf.FromEpsgNoToEpsgNo($D$4,$D$5,D27,E27)</f>
+        <f t="array" ref="F27:G27">_xll.PE.trf.Transform($D$4,$D$5,D27,E27)</f>
         <v>19.854659382414237</v>
       </c>
       <c r="G27" s="140">
@@ -40438,7 +40475,7 @@
         <v>4518740</v>
       </c>
       <c r="F28" s="138" cm="1">
-        <f t="array" ref="F28:G28">_xll.PE.trf.FromEpsgNoToEpsgNo($D$4,$D$5,D28,E28)</f>
+        <f t="array" ref="F28:G28">_xll.PE.trf.Transform($D$4,$D$5,D28,E28)</f>
         <v>20.099124970644958</v>
       </c>
       <c r="G28" s="140">
@@ -40506,7 +40543,7 @@
         <v>4519777.2910376322</v>
       </c>
       <c r="F29" s="135" cm="1">
-        <f t="array" ref="F29:G29">_xll.PE.trf.FromEpsgNoToEpsgNo($D$4,$D$5,D29,E29)</f>
+        <f t="array" ref="F29:G29">_xll.PE.trf.Transform($D$4,$D$5,D29,E29)</f>
         <v>20.144776595350073</v>
       </c>
       <c r="G29" s="137">
@@ -40573,7 +40610,7 @@
         <v>4520555.2593158567</v>
       </c>
       <c r="F30" s="141" cm="1">
-        <f t="array" ref="F30:G30">_xll.PE.trf.FromEpsgNoToEpsgNo($D$4,$D$5,D30,E30)</f>
+        <f t="array" ref="F30:G30">_xll.PE.trf.Transform($D$4,$D$5,D30,E30)</f>
         <v>20.17902421260742</v>
       </c>
       <c r="G30" s="143">
@@ -40698,7 +40735,7 @@
         <v>4525483.832561858</v>
       </c>
       <c r="F33" s="132" cm="1">
-        <f t="array" ref="F33:G33">_xll.PE.trf.FromEpsgNoToEpsgNo($D$4,$D$5,D33,E33)</f>
+        <f t="array" ref="F33:G33">_xll.PE.trf.Transform($D$4,$D$5,D33,E33)</f>
         <v>19.701095294756342</v>
       </c>
       <c r="G33" s="134">
@@ -40763,7 +40800,7 @@
         <v>4524196.0807782048</v>
       </c>
       <c r="F34" s="135" cm="1">
-        <f t="array" ref="F34:G34">_xll.PE.trf.FromEpsgNoToEpsgNo($D$4,$D$5,D34,E34)</f>
+        <f t="array" ref="F34:G34">_xll.PE.trf.Transform($D$4,$D$5,D34,E34)</f>
         <v>19.733442649612513</v>
       </c>
       <c r="G34" s="137">
@@ -40826,7 +40863,7 @@
         <v>4522479.0784</v>
       </c>
       <c r="F35" s="138" cm="1">
-        <f t="array" ref="F35:G35">_xll.PE.trf.FromEpsgNoToEpsgNo($D$4,$D$5,D35,E35)</f>
+        <f t="array" ref="F35:G35">_xll.PE.trf.Transform($D$4,$D$5,D35,E35)</f>
         <v>19.776555734991796</v>
       </c>
       <c r="G35" s="140">
@@ -40891,7 +40928,7 @@
         <v>4517866.0075000003</v>
       </c>
       <c r="F36" s="138" cm="1">
-        <f t="array" ref="F36:G36">_xll.PE.trf.FromEpsgNoToEpsgNo($D$4,$D$5,D36,E36)</f>
+        <f t="array" ref="F36:G36">_xll.PE.trf.Transform($D$4,$D$5,D36,E36)</f>
         <v>19.892292936682402</v>
       </c>
       <c r="G36" s="140">
@@ -40957,7 +40994,7 @@
         <v>4514669.1546</v>
       </c>
       <c r="F37" s="138" cm="1">
-        <f t="array" ref="F37:G37">_xll.PE.trf.FromEpsgNoToEpsgNo($D$4,$D$5,D37,E37)</f>
+        <f t="array" ref="F37:G37">_xll.PE.trf.Transform($D$4,$D$5,D37,E37)</f>
         <v>19.965689392996619</v>
       </c>
       <c r="G37" s="140">
@@ -41025,7 +41062,7 @@
         <v>4512826.2181084193</v>
       </c>
       <c r="F38" s="135" cm="1">
-        <f t="array" ref="F38:G38">_xll.PE.trf.FromEpsgNoToEpsgNo($D$4,$D$5,D38,E38)</f>
+        <f t="array" ref="F38:G38">_xll.PE.trf.Transform($D$4,$D$5,D38,E38)</f>
         <v>20.007973540197661</v>
       </c>
       <c r="G38" s="137">
@@ -41092,7 +41129,7 @@
         <v>4511444.0157397343</v>
       </c>
       <c r="F39" s="141" cm="1">
-        <f t="array" ref="F39:G39">_xll.PE.trf.FromEpsgNoToEpsgNo($D$4,$D$5,D39,E39)</f>
+        <f t="array" ref="F39:G39">_xll.PE.trf.Transform($D$4,$D$5,D39,E39)</f>
         <v>20.039673311207402</v>
       </c>
       <c r="G39" s="143">
@@ -41217,7 +41254,7 @@
         <v>4466849.4596596127</v>
       </c>
       <c r="F42" s="132" cm="1">
-        <f t="array" ref="F42:G42">_xll.PE.trf.FromEpsgNoToEpsgNo($D$4,$D$5,D42,E42)</f>
+        <f t="array" ref="F42:G42">_xll.PE.trf.Transform($D$4,$D$5,D42,E42)</f>
         <v>19.873652457410753</v>
       </c>
       <c r="G42" s="134">
@@ -41282,7 +41319,7 @@
         <v>4467896.6912340643</v>
       </c>
       <c r="F43" s="135" cm="1">
-        <f t="array" ref="F43:G43">_xll.PE.trf.FromEpsgNoToEpsgNo($D$4,$D$5,D43,E43)</f>
+        <f t="array" ref="F43:G43">_xll.PE.trf.Transform($D$4,$D$5,D43,E43)</f>
         <v>19.906574728018438</v>
       </c>
       <c r="G43" s="137">
@@ -41347,7 +41384,7 @@
         <v>4469293</v>
       </c>
       <c r="F44" s="138" cm="1">
-        <f t="array" ref="F44:G44">_xll.PE.trf.FromEpsgNoToEpsgNo($D$4,$D$5,D44,E44)</f>
+        <f t="array" ref="F44:G44">_xll.PE.trf.Transform($D$4,$D$5,D44,E44)</f>
         <v>19.950486102913491</v>
       </c>
       <c r="G44" s="140">
@@ -41413,7 +41450,7 @@
         <v>4479111.9987000003</v>
       </c>
       <c r="F45" s="138" cm="1">
-        <f t="array" ref="F45:G45">_xll.PE.trf.FromEpsgNoToEpsgNo($D$4,$D$5,D45,E45)</f>
+        <f t="array" ref="F45:G45">_xll.PE.trf.Transform($D$4,$D$5,D45,E45)</f>
         <v>20.259758719416958</v>
       </c>
       <c r="G45" s="140">
@@ -41481,7 +41518,7 @@
         <v>4480508.3074659361</v>
       </c>
       <c r="F46" s="135" cm="1">
-        <f t="array" ref="F46:G46">_xll.PE.trf.FromEpsgNoToEpsgNo($D$4,$D$5,D46,E46)</f>
+        <f t="array" ref="F46:G46">_xll.PE.trf.Transform($D$4,$D$5,D46,E46)</f>
         <v>20.303807202490884</v>
       </c>
       <c r="G46" s="137">
@@ -41548,7 +41585,7 @@
         <v>4481555.5390403876</v>
       </c>
       <c r="F47" s="141" cm="1">
-        <f t="array" ref="F47:G47">_xll.PE.trf.FromEpsgNoToEpsgNo($D$4,$D$5,D47,E47)</f>
+        <f t="array" ref="F47:G47">_xll.PE.trf.Transform($D$4,$D$5,D47,E47)</f>
         <v>20.336854707752281</v>
       </c>
       <c r="G47" s="143">
@@ -41673,7 +41710,7 @@
         <v>4464929.1109348536</v>
       </c>
       <c r="F50" s="132" cm="1">
-        <f t="array" ref="F50:G50">_xll.PE.trf.FromEpsgNoToEpsgNo($D$4,$D$5,D50,E50)</f>
+        <f t="array" ref="F50:G50">_xll.PE.trf.Transform($D$4,$D$5,D50,E50)</f>
         <v>19.900207757522892</v>
       </c>
       <c r="G50" s="134">
@@ -41738,7 +41775,7 @@
         <v>4465879.6348627731</v>
       </c>
       <c r="F51" s="135" cm="1">
-        <f t="array" ref="F51:G51">_xll.PE.trf.FromEpsgNoToEpsgNo($D$4,$D$5,D51,E51)</f>
+        <f t="array" ref="F51:G51">_xll.PE.trf.Transform($D$4,$D$5,D51,E51)</f>
         <v>19.933541273379543</v>
       </c>
       <c r="G51" s="137">
@@ -41803,7 +41840,7 @@
         <v>4467147.0000999998</v>
       </c>
       <c r="F52" s="138" cm="1">
-        <f t="array" ref="F52:G52">_xll.PE.trf.FromEpsgNoToEpsgNo($D$4,$D$5,D52,E52)</f>
+        <f t="array" ref="F52:G52">_xll.PE.trf.Transform($D$4,$D$5,D52,E52)</f>
         <v>19.97799981976652</v>
       </c>
       <c r="G52" s="140">
@@ -41869,7 +41906,7 @@
         <v>4475048.0003000004</v>
       </c>
       <c r="F53" s="138" cm="1">
-        <f t="array" ref="F53:G53">_xll.PE.trf.FromEpsgNoToEpsgNo($D$4,$D$5,D53,E53)</f>
+        <f t="array" ref="F53:G53">_xll.PE.trf.Transform($D$4,$D$5,D53,E53)</f>
         <v>20.255518710888996</v>
       </c>
       <c r="G53" s="140">
@@ -41937,7 +41974,7 @@
         <v>4476315.3655372271</v>
       </c>
       <c r="F54" s="135" cm="1">
-        <f t="array" ref="F54:G54">_xll.PE.trf.FromEpsgNoToEpsgNo($D$4,$D$5,D54,E54)</f>
+        <f t="array" ref="F54:G54">_xll.PE.trf.Transform($D$4,$D$5,D54,E54)</f>
         <v>20.300091131624491</v>
       </c>
       <c r="G54" s="137">
@@ -42004,7 +42041,7 @@
         <v>4477265.8894651467</v>
       </c>
       <c r="F55" s="141" cm="1">
-        <f t="array" ref="F55:G55">_xll.PE.trf.FromEpsgNoToEpsgNo($D$4,$D$5,D55,E55)</f>
+        <f t="array" ref="F55:G55">_xll.PE.trf.Transform($D$4,$D$5,D55,E55)</f>
         <v>20.333530712767278</v>
       </c>
       <c r="G55" s="143">
@@ -42129,7 +42166,7 @@
         <v>4463055.1312818611</v>
       </c>
       <c r="F58" s="132" cm="1">
-        <f t="array" ref="F58:G58">_xll.PE.trf.FromEpsgNoToEpsgNo($D$4,$D$5,D58,E58)</f>
+        <f t="array" ref="F58:G58">_xll.PE.trf.Transform($D$4,$D$5,D58,E58)</f>
         <v>19.925860955743484</v>
       </c>
       <c r="G58" s="134">
@@ -42194,7 +42231,7 @@
         <v>4463865.0748896347</v>
       </c>
       <c r="F59" s="135" cm="1">
-        <f t="array" ref="F59:G59">_xll.PE.trf.FromEpsgNoToEpsgNo($D$4,$D$5,D59,E59)</f>
+        <f t="array" ref="F59:G59">_xll.PE.trf.Transform($D$4,$D$5,D59,E59)</f>
         <v>19.959716888540239</v>
       </c>
       <c r="G59" s="137">
@@ -42259,7 +42296,7 @@
         <v>4464944.9996999996</v>
       </c>
       <c r="F60" s="138" cm="1">
-        <f t="array" ref="F60:G60">_xll.PE.trf.FromEpsgNoToEpsgNo($D$4,$D$5,D60,E60)</f>
+        <f t="array" ref="F60:G60">_xll.PE.trf.Transform($D$4,$D$5,D60,E60)</f>
         <v>20.00487023617189</v>
       </c>
       <c r="G60" s="140">
@@ -42325,7 +42362,7 @@
         <v>4470817.0005000001</v>
       </c>
       <c r="F61" s="138" cm="1">
-        <f t="array" ref="F61:G61">_xll.PE.trf.FromEpsgNoToEpsgNo($D$4,$D$5,D61,E61)</f>
+        <f t="array" ref="F61:G61">_xll.PE.trf.Transform($D$4,$D$5,D61,E61)</f>
         <v>20.250628652514411</v>
       </c>
       <c r="G61" s="140">
@@ -42393,7 +42430,7 @@
         <v>4471896.9253103649</v>
       </c>
       <c r="F62" s="135" cm="1">
-        <f t="array" ref="F62:G62">_xll.PE.trf.FromEpsgNoToEpsgNo($D$4,$D$5,D62,E62)</f>
+        <f t="array" ref="F62:G62">_xll.PE.trf.Transform($D$4,$D$5,D62,E62)</f>
         <v>20.295870360336661</v>
       </c>
       <c r="G62" s="137">
@@ -42460,7 +42497,7 @@
         <v>4472706.8689181386</v>
       </c>
       <c r="F63" s="141" cm="1">
-        <f t="array" ref="F63:G63">_xll.PE.trf.FromEpsgNoToEpsgNo($D$4,$D$5,D63,E63)</f>
+        <f t="array" ref="F63:G63">_xll.PE.trf.Transform($D$4,$D$5,D63,E63)</f>
         <v>20.32981057815698</v>
       </c>
       <c r="G63" s="143">
@@ -42581,7 +42618,7 @@
         <v>4450574.3227219004</v>
       </c>
       <c r="F66" s="132" cm="1">
-        <f t="array" ref="F66:G66">_xll.PE.trf.FromEpsgNoToEpsgNo($D$4,$D$5,D66,E66)</f>
+        <f t="array" ref="F66:G66">_xll.PE.trf.Transform($D$4,$D$5,D66,E66)</f>
         <v>19.99171711359562</v>
       </c>
       <c r="G66" s="134">
@@ -42646,7 +42683,7 @@
         <v>4452180.0220553717</v>
       </c>
       <c r="F67" s="135" cm="1">
-        <f t="array" ref="F67:G67">_xll.PE.trf.FromEpsgNoToEpsgNo($D$4,$D$5,D67,E67)</f>
+        <f t="array" ref="F67:G67">_xll.PE.trf.Transform($D$4,$D$5,D67,E67)</f>
         <v>20.021260198241439</v>
       </c>
       <c r="G67" s="137">
@@ -42709,7 +42746,7 @@
         <v>4454320.9545</v>
       </c>
       <c r="F68" s="138" cm="1">
-        <f t="array" ref="F68:G68">_xll.PE.trf.FromEpsgNoToEpsgNo($D$4,$D$5,D68,E68)</f>
+        <f t="array" ref="F68:G68">_xll.PE.trf.Transform($D$4,$D$5,D68,E68)</f>
         <v>20.06067098541865</v>
       </c>
       <c r="G68" s="140">
@@ -42774,7 +42811,7 @@
         <v>4459903.6739999996</v>
       </c>
       <c r="F69" s="138" cm="1">
-        <f t="array" ref="F69:G69">_xll.PE.trf.FromEpsgNoToEpsgNo($D$4,$D$5,D69,E69)</f>
+        <f t="array" ref="F69:G69">_xll.PE.trf.Transform($D$4,$D$5,D69,E69)</f>
         <v>20.163546599470713</v>
       </c>
       <c r="G69" s="140">
@@ -42840,7 +42877,7 @@
         <v>4465830.3525</v>
       </c>
       <c r="F70" s="138" cm="1">
-        <f t="array" ref="F70:G70">_xll.PE.trf.FromEpsgNoToEpsgNo($D$4,$D$5,D70,E70)</f>
+        <f t="array" ref="F70:G70">_xll.PE.trf.Transform($D$4,$D$5,D70,E70)</f>
         <v>20.236972394273813</v>
       </c>
       <c r="G70" s="140">
@@ -42908,7 +42945,7 @@
         <v>4468571.8112974633</v>
       </c>
       <c r="F71" s="135" cm="1">
-        <f t="array" ref="F71:G71">_xll.PE.trf.FromEpsgNoToEpsgNo($D$4,$D$5,D71,E71)</f>
+        <f t="array" ref="F71:G71">_xll.PE.trf.Transform($D$4,$D$5,D71,E71)</f>
         <v>20.270975922742149</v>
       </c>
       <c r="G71" s="137">
@@ -42975,7 +43012,7 @@
         <v>4470627.9053955609</v>
       </c>
       <c r="F72" s="141" cm="1">
-        <f t="array" ref="F72:G72">_xll.PE.trf.FromEpsgNoToEpsgNo($D$4,$D$5,D72,E72)</f>
+        <f t="array" ref="F72:G72">_xll.PE.trf.Transform($D$4,$D$5,D72,E72)</f>
         <v>20.296494997345555</v>
       </c>
       <c r="G72" s="143">
@@ -43100,7 +43137,7 @@
         <v>4441250.3036329644</v>
       </c>
       <c r="F75" s="132" cm="1">
-        <f t="array" ref="F75:G75">_xll.PE.trf.FromEpsgNoToEpsgNo($D$4,$D$5,D75,E75)</f>
+        <f t="array" ref="F75:G75">_xll.PE.trf.Transform($D$4,$D$5,D75,E75)</f>
         <v>20.009021806680682</v>
       </c>
       <c r="G75" s="134">
@@ -43165,7 +43202,7 @@
         <v>4442758.5208331225</v>
       </c>
       <c r="F76" s="135" cm="1">
-        <f t="array" ref="F76:G76">_xll.PE.trf.FromEpsgNoToEpsgNo($D$4,$D$5,D76,E76)</f>
+        <f t="array" ref="F76:G76">_xll.PE.trf.Transform($D$4,$D$5,D76,E76)</f>
         <v>20.039239468543986</v>
       </c>
       <c r="G76" s="137">
@@ -43228,7 +43265,7 @@
         <v>4444769.4770999998</v>
       </c>
       <c r="F77" s="138" cm="1">
-        <f t="array" ref="F77:G77">_xll.PE.trf.FromEpsgNoToEpsgNo($D$4,$D$5,D77,E77)</f>
+        <f t="array" ref="F77:G77">_xll.PE.trf.Transform($D$4,$D$5,D77,E77)</f>
         <v>20.079548896305266</v>
       </c>
       <c r="G77" s="140">
@@ -43293,7 +43330,7 @@
         <v>4450616.7803999996</v>
       </c>
       <c r="F78" s="138" cm="1">
-        <f t="array" ref="F78:G78">_xll.PE.trf.FromEpsgNoToEpsgNo($D$4,$D$5,D78,E78)</f>
+        <f t="array" ref="F78:G78">_xll.PE.trf.Transform($D$4,$D$5,D78,E78)</f>
         <v>20.196882297215772</v>
       </c>
       <c r="G78" s="140">
@@ -43359,7 +43396,7 @@
         <v>4459612.6317999996</v>
       </c>
       <c r="F79" s="138" cm="1">
-        <f t="array" ref="F79:G79">_xll.PE.trf.FromEpsgNoToEpsgNo($D$4,$D$5,D79,E79)</f>
+        <f t="array" ref="F79:G79">_xll.PE.trf.Transform($D$4,$D$5,D79,E79)</f>
         <v>20.333399268047305</v>
       </c>
       <c r="G79" s="140">
@@ -43427,7 +43464,7 @@
         <v>4462051.4748460185</v>
       </c>
       <c r="F80" s="135" cm="1">
-        <f t="array" ref="F80:G80">_xll.PE.trf.FromEpsgNoToEpsgNo($D$4,$D$5,D80,E80)</f>
+        <f t="array" ref="F80:G80">_xll.PE.trf.Transform($D$4,$D$5,D80,E80)</f>
         <v>20.370466902167522</v>
       </c>
       <c r="G80" s="137">
@@ -43494,7 +43531,7 @@
         <v>4463880.6071305331</v>
       </c>
       <c r="F81" s="141" cm="1">
-        <f t="array" ref="F81:G81">_xll.PE.trf.FromEpsgNoToEpsgNo($D$4,$D$5,D81,E81)</f>
+        <f t="array" ref="F81:G81">_xll.PE.trf.Transform($D$4,$D$5,D81,E81)</f>
         <v>20.398283565718462</v>
       </c>
       <c r="G81" s="143">
@@ -43619,7 +43656,7 @@
         <v>4429507.8151147934</v>
       </c>
       <c r="F84" s="132" cm="1">
-        <f t="array" ref="F84:G84">_xll.PE.trf.FromEpsgNoToEpsgNo($D$4,$D$5,D84,E84)</f>
+        <f t="array" ref="F84:G84">_xll.PE.trf.Transform($D$4,$D$5,D84,E84)</f>
         <v>20.069993444467798</v>
       </c>
       <c r="G84" s="134">
@@ -43684,7 +43721,7 @@
         <v>4431013.8744655959</v>
       </c>
       <c r="F85" s="135" cm="1">
-        <f t="array" ref="F85:G85">_xll.PE.trf.FromEpsgNoToEpsgNo($D$4,$D$5,D85,E85)</f>
+        <f t="array" ref="F85:G85">_xll.PE.trf.Transform($D$4,$D$5,D85,E85)</f>
         <v>20.100192626928944</v>
       </c>
       <c r="G85" s="137">
@@ -43747,7 +43784,7 @@
         <v>4433021.9535999997</v>
       </c>
       <c r="F86" s="138" cm="1">
-        <f t="array" ref="F86:G86">_xll.PE.trf.FromEpsgNoToEpsgNo($D$4,$D$5,D86,E86)</f>
+        <f t="array" ref="F86:G86">_xll.PE.trf.Transform($D$4,$D$5,D86,E86)</f>
         <v>20.140477274654241</v>
       </c>
       <c r="G86" s="140">
@@ -43812,7 +43849,7 @@
         <v>4439871.5713</v>
       </c>
       <c r="F87" s="138" cm="1">
-        <f t="array" ref="F87:G87">_xll.PE.trf.FromEpsgNoToEpsgNo($D$4,$D$5,D87,E87)</f>
+        <f t="array" ref="F87:G87">_xll.PE.trf.Transform($D$4,$D$5,D87,E87)</f>
         <v>20.278053401830466</v>
       </c>
       <c r="G87" s="140">
@@ -43878,7 +43915,7 @@
         <v>4450775.5307999998</v>
       </c>
       <c r="F88" s="138" cm="1">
-        <f t="array" ref="F88:G88">_xll.PE.trf.FromEpsgNoToEpsgNo($D$4,$D$5,D88,E88)</f>
+        <f t="array" ref="F88:G88">_xll.PE.trf.Transform($D$4,$D$5,D88,E88)</f>
         <v>20.472740821899968</v>
       </c>
       <c r="G88" s="140">
@@ -43946,7 +43983,7 @@
         <v>4452965.229134731</v>
       </c>
       <c r="F89" s="135" cm="1">
-        <f t="array" ref="F89:G89">_xll.PE.trf.FromEpsgNoToEpsgNo($D$4,$D$5,D89,E89)</f>
+        <f t="array" ref="F89:G89">_xll.PE.trf.Transform($D$4,$D$5,D89,E89)</f>
         <v>20.511905954708112</v>
       </c>
       <c r="G89" s="137">
@@ -44013,7 +44050,7 @@
         <v>4454607.5028857794</v>
       </c>
       <c r="F90" s="141" cm="1">
-        <f t="array" ref="F90:G90">_xll.PE.trf.FromEpsgNoToEpsgNo($D$4,$D$5,D90,E90)</f>
+        <f t="array" ref="F90:G90">_xll.PE.trf.Transform($D$4,$D$5,D90,E90)</f>
         <v>20.541294879939993</v>
       </c>
       <c r="G90" s="143">
@@ -44138,7 +44175,7 @@
         <v>4468581.3680245327</v>
       </c>
       <c r="F93" s="132" cm="1">
-        <f t="array" ref="F93:G93">_xll.PE.trf.FromEpsgNoToEpsgNo($D$4,$D$5,D93,E93)</f>
+        <f t="array" ref="F93:G93">_xll.PE.trf.Transform($D$4,$D$5,D93,E93)</f>
         <v>20.041822842787745</v>
       </c>
       <c r="G93" s="134">
@@ -44203,7 +44240,7 @@
         <v>4466546.5277140187</v>
       </c>
       <c r="F94" s="135" cm="1">
-        <f t="array" ref="F94:G94">_xll.PE.trf.FromEpsgNoToEpsgNo($D$4,$D$5,D94,E94)</f>
+        <f t="array" ref="F94:G94">_xll.PE.trf.Transform($D$4,$D$5,D94,E94)</f>
         <v>20.068017585449915</v>
       </c>
       <c r="G94" s="137">
@@ -44266,7 +44303,7 @@
         <v>4463833.4073000001</v>
       </c>
       <c r="F95" s="138" cm="1">
-        <f t="array" ref="F95:G95">_xll.PE.trf.FromEpsgNoToEpsgNo($D$4,$D$5,D95,E95)</f>
+        <f t="array" ref="F95:G95">_xll.PE.trf.Transform($D$4,$D$5,D95,E95)</f>
         <v>20.102922159653534</v>
       </c>
       <c r="G95" s="140">
@@ -44331,7 +44368,7 @@
         <v>4452879.6354</v>
       </c>
       <c r="F96" s="138" cm="1">
-        <f t="array" ref="F96:G96">_xll.PE.trf.FromEpsgNoToEpsgNo($D$4,$D$5,D96,E96)</f>
+        <f t="array" ref="F96:G96">_xll.PE.trf.Transform($D$4,$D$5,D96,E96)</f>
         <v>20.243591327481912</v>
       </c>
       <c r="G96" s="140">
@@ -44397,7 +44434,7 @@
         <v>4437480.8546000002</v>
       </c>
       <c r="F97" s="138" cm="1">
-        <f t="array" ref="F97:G97">_xll.PE.trf.FromEpsgNoToEpsgNo($D$4,$D$5,D97,E97)</f>
+        <f t="array" ref="F97:G97">_xll.PE.trf.Transform($D$4,$D$5,D97,E97)</f>
         <v>20.435390220595277</v>
       </c>
       <c r="G97" s="140">
@@ -44465,7 +44502,7 @@
         <v>4434727.9086254323</v>
       </c>
       <c r="F98" s="135" cm="1">
-        <f t="array" ref="F98:G98">_xll.PE.trf.FromEpsgNoToEpsgNo($D$4,$D$5,D98,E98)</f>
+        <f t="array" ref="F98:G98">_xll.PE.trf.Transform($D$4,$D$5,D98,E98)</f>
         <v>20.469598076487333</v>
       </c>
       <c r="G98" s="137">
@@ -44532,7 +44569,7 @@
         <v>4432663.1991445068</v>
       </c>
       <c r="F99" s="141" cm="1">
-        <f t="array" ref="F99:G99">_xll.PE.trf.FromEpsgNoToEpsgNo($D$4,$D$5,D99,E99)</f>
+        <f t="array" ref="F99:G99">_xll.PE.trf.Transform($D$4,$D$5,D99,E99)</f>
         <v>20.495237819768231</v>
       </c>
       <c r="G99" s="143">
@@ -44657,7 +44694,7 @@
         <v>4468437.1458815532</v>
       </c>
       <c r="F102" s="132" cm="1">
-        <f t="array" ref="F102:G102">_xll.PE.trf.FromEpsgNoToEpsgNo($D$4,$D$5,D102,E102)</f>
+        <f t="array" ref="F102:G102">_xll.PE.trf.Transform($D$4,$D$5,D102,E102)</f>
         <v>20.122614090696832</v>
       </c>
       <c r="G102" s="134">
@@ -44722,7 +44759,7 @@
         <v>4466599.7976466017</v>
       </c>
       <c r="F103" s="135" cm="1">
-        <f t="array" ref="F103:G103">_xll.PE.trf.FromEpsgNoToEpsgNo($D$4,$D$5,D103,E103)</f>
+        <f t="array" ref="F103:G103">_xll.PE.trf.Transform($D$4,$D$5,D103,E103)</f>
         <v>20.150731246325268</v>
       </c>
       <c r="G103" s="137">
@@ -44787,7 +44824,7 @@
         <v>4464150</v>
       </c>
       <c r="F104" s="138" cm="1">
-        <f t="array" ref="F104:G104">_xll.PE.trf.FromEpsgNoToEpsgNo($D$4,$D$5,D104,E104)</f>
+        <f t="array" ref="F104:G104">_xll.PE.trf.Transform($D$4,$D$5,D104,E104)</f>
         <v>20.188199773372965</v>
       </c>
       <c r="G104" s="140">
@@ -44853,7 +44890,7 @@
         <v>4445370</v>
       </c>
       <c r="F105" s="138" cm="1">
-        <f t="array" ref="F105:G105">_xll.PE.trf.FromEpsgNoToEpsgNo($D$4,$D$5,D105,E105)</f>
+        <f t="array" ref="F105:G105">_xll.PE.trf.Transform($D$4,$D$5,D105,E105)</f>
         <v>20.474635225434131</v>
       </c>
       <c r="G105" s="140">
@@ -44921,7 +44958,7 @@
         <v>4442920.2023533983</v>
       </c>
       <c r="F106" s="135" cm="1">
-        <f t="array" ref="F106:G106">_xll.PE.trf.FromEpsgNoToEpsgNo($D$4,$D$5,D106,E106)</f>
+        <f t="array" ref="F106:G106">_xll.PE.trf.Transform($D$4,$D$5,D106,E106)</f>
         <v>20.511896311461349</v>
       </c>
       <c r="G106" s="137">
@@ -44988,7 +45025,7 @@
         <v>4441082.8541184468</v>
       </c>
       <c r="F107" s="141" cm="1">
-        <f t="array" ref="F107:G107">_xll.PE.trf.FromEpsgNoToEpsgNo($D$4,$D$5,D107,E107)</f>
+        <f t="array" ref="F107:G107">_xll.PE.trf.Transform($D$4,$D$5,D107,E107)</f>
         <v>20.53982646884727</v>
       </c>
       <c r="G107" s="143">
@@ -45113,7 +45150,7 @@
         <v>4456901.3573793834</v>
       </c>
       <c r="F110" s="132" cm="1">
-        <f t="array" ref="F110:G110">_xll.PE.trf.FromEpsgNoToEpsgNo($D$4,$D$5,D110,E110)</f>
+        <f t="array" ref="F110:G110">_xll.PE.trf.Transform($D$4,$D$5,D110,E110)</f>
         <v>19.980295097411723</v>
       </c>
       <c r="G110" s="134">
@@ -45178,7 +45215,7 @@
         <v>4454655.0613596477</v>
       </c>
       <c r="F111" s="135" cm="1">
-        <f t="array" ref="F111:G111">_xll.PE.trf.FromEpsgNoToEpsgNo($D$4,$D$5,D111,E111)</f>
+        <f t="array" ref="F111:G111">_xll.PE.trf.Transform($D$4,$D$5,D111,E111)</f>
         <v>20.003956316830397</v>
       </c>
       <c r="G111" s="137">
@@ -45243,7 +45280,7 @@
         <v>4451660</v>
       </c>
       <c r="F112" s="138" cm="1">
-        <f t="array" ref="F112:G112">_xll.PE.trf.FromEpsgNoToEpsgNo($D$4,$D$5,D112,E112)</f>
+        <f t="array" ref="F112:G112">_xll.PE.trf.Transform($D$4,$D$5,D112,E112)</f>
         <v>20.035482907483946</v>
       </c>
       <c r="G112" s="140">
@@ -45309,7 +45346,7 @@
         <v>4430146</v>
       </c>
       <c r="F113" s="138" cm="1">
-        <f t="array" ref="F113:G113">_xll.PE.trf.FromEpsgNoToEpsgNo($D$4,$D$5,D113,E113)</f>
+        <f t="array" ref="F113:G113">_xll.PE.trf.Transform($D$4,$D$5,D113,E113)</f>
         <v>20.261217584877354</v>
       </c>
       <c r="G113" s="140">
@@ -45377,7 +45414,7 @@
         <v>4427150.9386403523</v>
       </c>
       <c r="F114" s="135" cm="1">
-        <f t="array" ref="F114:G114">_xll.PE.trf.FromEpsgNoToEpsgNo($D$4,$D$5,D114,E114)</f>
+        <f t="array" ref="F114:G114">_xll.PE.trf.Transform($D$4,$D$5,D114,E114)</f>
         <v>20.292542535155217</v>
       </c>
       <c r="G114" s="137">
@@ -45444,7 +45481,7 @@
         <v>4424904.6426206166</v>
       </c>
       <c r="F115" s="141" cm="1">
-        <f t="array" ref="F115:G115">_xll.PE.trf.FromEpsgNoToEpsgNo($D$4,$D$5,D115,E115)</f>
+        <f t="array" ref="F115:G115">_xll.PE.trf.Transform($D$4,$D$5,D115,E115)</f>
         <v>20.316020182948577</v>
       </c>
       <c r="G115" s="143">
@@ -45568,11 +45605,11 @@
         <f>E119-$D$7*COS(RADIANS(O119))</f>
         <v>4452852.3097855086</v>
       </c>
-      <c r="F118" s="132" cm="1">
-        <f t="array" ref="F118:G118">_xll.PE.trf.Transform($D$4,$D$5,D118,E118,$C$128)</f>
+      <c r="F118" s="135" cm="1">
+        <f t="array" ref="F118:G118">_xll.PE.trf.Transform($D$4,$D$5,D118,E118)</f>
         <v>20.155244386653319</v>
       </c>
-      <c r="G118" s="134">
+      <c r="G118" s="137">
         <v>40.205795085677487</v>
       </c>
       <c r="H118" s="132" t="str" cm="1">
@@ -45634,7 +45671,7 @@
         <v>4454594.5170202907</v>
       </c>
       <c r="F119" s="135" cm="1">
-        <f t="array" ref="F119:G119">_xll.PE.trf.FromEpsgNoToEpsgNo($D$4,$D$5,D119,E119)</f>
+        <f t="array" ref="F119:G119">_xll.PE.trf.Transform($D$4,$D$5,D119,E119)</f>
         <v>20.183739389448178</v>
       </c>
       <c r="G119" s="137">
@@ -45699,7 +45736,7 @@
         <v>4456917.46</v>
       </c>
       <c r="F120" s="138" cm="1">
-        <f t="array" ref="F120:G120">_xll.PE.trf.FromEpsgNoToEpsgNo($D$4,$D$5,D120,E120)</f>
+        <f t="array" ref="F120:G120">_xll.PE.trf.Transform($D$4,$D$5,D120,E120)</f>
         <v>20.22175353346173</v>
       </c>
       <c r="G120" s="140">
@@ -45765,7 +45802,7 @@
         <v>4461819.1283</v>
       </c>
       <c r="F121" s="138" cm="1">
-        <f t="array" ref="F121:G121">_xll.PE.trf.FromEpsgNoToEpsgNo($D$4,$D$5,D121,E121)</f>
+        <f t="array" ref="F121:G121">_xll.PE.trf.Transform($D$4,$D$5,D121,E121)</f>
         <v>20.302045697642804</v>
       </c>
       <c r="G121" s="140">
@@ -45833,7 +45870,7 @@
         <v>4464142.0712797092</v>
       </c>
       <c r="F122" s="135" cm="1">
-        <f t="array" ref="F122:G122">_xll.PE.trf.FromEpsgNoToEpsgNo($D$4,$D$5,D122,E122)</f>
+        <f t="array" ref="F122:G122">_xll.PE.trf.Transform($D$4,$D$5,D122,E122)</f>
         <v>20.340133885134307</v>
       </c>
       <c r="G122" s="137">
@@ -45900,7 +45937,7 @@
         <v>4465884.2785144914</v>
       </c>
       <c r="F123" s="141" cm="1">
-        <f t="array" ref="F123:G123">_xll.PE.trf.FromEpsgNoToEpsgNo($D$4,$D$5,D123,E123)</f>
+        <f t="array" ref="F123:G123">_xll.PE.trf.Transform($D$4,$D$5,D123,E123)</f>
         <v>20.3687156675634</v>
       </c>
       <c r="G123" s="143">
@@ -45990,1729 +46027,2144 @@
       </c>
     </row>
     <row r="126" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="D126" s="198"/>
-      <c r="E126" s="198"/>
+      <c r="K126" s="61"/>
       <c r="M126"/>
     </row>
-    <row r="127" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="C127" s="182" t="str" cm="1">
-        <f t="array" ref="C127">_xll.PE.trf.Options(,,,,,1,,,,,,,,,1,)</f>
-        <v>Authority=EPSG; Area=; Accuracy=1; NoBallparkConversions=False; NoDiscardIfMissing=False; UsePrimaryGridNames=False; UseSuperseded=False; StrictContains=False; IntermediateCrsUsage=Auto; BestOnly=False; ForceOver=False; CandidateIndex=1; AllowDeprecatedCrs=False</v>
-      </c>
-      <c r="D127" s="183"/>
-      <c r="E127" s="183"/>
-      <c r="F127" s="183"/>
-      <c r="G127" s="183"/>
-      <c r="H127" s="183"/>
-      <c r="I127" s="183"/>
-      <c r="J127" s="183"/>
-      <c r="K127" s="183"/>
-      <c r="L127" s="183"/>
-      <c r="M127" s="183"/>
-      <c r="N127" s="183"/>
-      <c r="O127" s="204"/>
-      <c r="P127" s="183"/>
-      <c r="Q127" s="184"/>
+    <row r="127" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="C127" s="41" t="s">
+        <v>142</v>
+      </c>
+      <c r="D127" s="224">
+        <f>D4</f>
+        <v>2462</v>
+      </c>
     </row>
     <row r="128" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="C128" s="182" t="str" cm="1">
-        <f t="array" ref="C128">_xll.PE.trf.Options(,,,,,,,,,,,,,,0,)</f>
+      <c r="C128" s="12" t="s">
+        <v>143</v>
+      </c>
+      <c r="D128" s="225">
+        <f>D5</f>
+        <v>4326</v>
+      </c>
+    </row>
+    <row r="129" spans="3:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="C129" s="227" t="str">
+        <f>C14</f>
+        <v>Authority=0; Area=0,0,0,0; Accuracy=0; NoBallparkConversions=False; NoDiscardIfMissing=False; UsePrimaryGridNames=False; UseSuperseded=False; StrictContains=False; IntermediateCrsUsage=Auto; BestOnly=False; ForceOver=False; CandidateIndex=0; AllowDeprecatedCrs=False</v>
+      </c>
+      <c r="D129" s="228"/>
+      <c r="E129" s="228"/>
+      <c r="F129" s="228"/>
+      <c r="G129" s="228"/>
+      <c r="H129" s="228"/>
+      <c r="I129" s="228"/>
+      <c r="J129" s="228"/>
+      <c r="K129" s="228"/>
+      <c r="L129" s="228"/>
+      <c r="M129" s="229"/>
+      <c r="N129" s="228"/>
+      <c r="O129" s="230"/>
+      <c r="P129" s="231"/>
+    </row>
+    <row r="130" spans="3:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="C130" s="226" t="str" cm="1">
+        <f t="array" ref="C130:D153">_xll.PE.trf.TransformList(D127,D128,C129,"nil")</f>
+        <v>Transform Number</v>
+      </c>
+      <c r="D130" s="103">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="131" spans="3:16" x14ac:dyDescent="0.35">
+      <c r="C131" s="12" t="str">
+        <v>Transform Name</v>
+      </c>
+      <c r="D131" s="216" t="str">
+        <v>Inverse of 6-degree Gauss-Kruger zone 4 + Ballpark geographic offset from Albanian 1987 to WGS 84 (with axis order normalized for visualization)</v>
+      </c>
+    </row>
+    <row r="132" spans="3:16" x14ac:dyDescent="0.35">
+      <c r="C132" s="12" t="str">
+        <v>Transform Type</v>
+      </c>
+      <c r="D132" s="216" t="str">
+        <v>ConcatenatedOperation</v>
+      </c>
+    </row>
+    <row r="133" spans="3:16" x14ac:dyDescent="0.35">
+      <c r="C133" s="12" t="str">
+        <v>Identifier</v>
+      </c>
+      <c r="D133" s="216" t="str">
+        <v>nil</v>
+      </c>
+    </row>
+    <row r="134" spans="3:16" x14ac:dyDescent="0.35">
+      <c r="C134" s="12" t="str">
+        <v>Identifiers</v>
+      </c>
+      <c r="D134" s="216" t="str">
+        <v>nil</v>
+      </c>
+    </row>
+    <row r="135" spans="3:16" x14ac:dyDescent="0.35">
+      <c r="C135" s="12" t="str">
+        <v>Accuracy</v>
+      </c>
+      <c r="D135" s="216" t="str">
+        <v>nil</v>
+      </c>
+    </row>
+    <row r="136" spans="3:16" x14ac:dyDescent="0.35">
+      <c r="C136" s="12" t="str">
+        <v>IsAvailable</v>
+      </c>
+      <c r="D136" s="216" t="str">
+        <v>True</v>
+      </c>
+    </row>
+    <row r="137" spans="3:16" x14ac:dyDescent="0.35">
+      <c r="C137" s="12" t="str">
+        <v>HasBallParkTransformation</v>
+      </c>
+      <c r="D137" s="216" t="str">
+        <v>True</v>
+      </c>
+    </row>
+    <row r="138" spans="3:16" x14ac:dyDescent="0.35">
+      <c r="C138" s="12" t="str">
+        <v>HasInverse</v>
+      </c>
+      <c r="D138" s="216" t="str">
+        <v>True</v>
+      </c>
+    </row>
+    <row r="139" spans="3:16" x14ac:dyDescent="0.35">
+      <c r="C139" s="12" t="str">
+        <v>MethodName</v>
+      </c>
+      <c r="D139" s="216" t="str">
+        <v>nil</v>
+      </c>
+    </row>
+    <row r="140" spans="3:16" x14ac:dyDescent="0.35">
+      <c r="C140" s="12" t="str">
+        <v>Scope</v>
+      </c>
+      <c r="D140" s="216" t="str">
+        <v>nil</v>
+      </c>
+    </row>
+    <row r="141" spans="3:16" x14ac:dyDescent="0.35">
+      <c r="C141" s="12" t="str">
+        <v>Remarks</v>
+      </c>
+      <c r="D141" s="216" t="str">
+        <v>nil</v>
+      </c>
+    </row>
+    <row r="142" spans="3:16" x14ac:dyDescent="0.35">
+      <c r="C142" s="12" t="str">
+        <v>GridUsages</v>
+      </c>
+      <c r="D142" s="216" t="str">
+        <v>nil</v>
+      </c>
+    </row>
+    <row r="143" spans="3:16" x14ac:dyDescent="0.35">
+      <c r="C143" s="12" t="str">
+        <v>Parameters</v>
+      </c>
+      <c r="D143" s="216" t="str">
+        <v>nil</v>
+      </c>
+    </row>
+    <row r="144" spans="3:16" x14ac:dyDescent="0.35">
+      <c r="C144" s="12" t="str">
+        <v>SourceCRS</v>
+      </c>
+      <c r="D144" s="216" t="str">
+        <v>Albanian 1987 / Gauss-Kruger zone 4 (with axis order normalized for visualization)</v>
+      </c>
+    </row>
+    <row r="145" spans="3:16" x14ac:dyDescent="0.35">
+      <c r="C145" s="12" t="str">
+        <v>TargetCRS</v>
+      </c>
+      <c r="D145" s="216" t="str">
+        <v>WGS 84 (with axis order normalized for visualization)</v>
+      </c>
+    </row>
+    <row r="146" spans="3:16" x14ac:dyDescent="0.35">
+      <c r="C146" s="12" t="str">
+        <v>Context</v>
+      </c>
+      <c r="D146" s="216" t="str">
+        <v>LogLevel=Error; EndpointUrl=https://cdn.proj.org; EnableNetworkConnections=True</v>
+      </c>
+    </row>
+    <row r="147" spans="3:16" x14ac:dyDescent="0.35">
+      <c r="C147" s="12" t="str">
+        <v>UsageArea</v>
+      </c>
+      <c r="D147" s="216" t="str">
+        <v>UsageArea</v>
+      </c>
+    </row>
+    <row r="148" spans="3:16" x14ac:dyDescent="0.35">
+      <c r="C148" s="12" t="str">
+        <v>UsageArea.Name</v>
+      </c>
+      <c r="D148" s="216" t="str">
+        <v>World</v>
+      </c>
+    </row>
+    <row r="149" spans="3:16" x14ac:dyDescent="0.35">
+      <c r="C149" s="12" t="str">
+        <v>UsageArea.WestLongitude</v>
+      </c>
+      <c r="D149" s="216" t="str">
+        <v>-180</v>
+      </c>
+    </row>
+    <row r="150" spans="3:16" x14ac:dyDescent="0.35">
+      <c r="C150" s="12" t="str">
+        <v>UsageArea.SouthLatitude</v>
+      </c>
+      <c r="D150" s="216" t="str">
+        <v>-90</v>
+      </c>
+    </row>
+    <row r="151" spans="3:16" x14ac:dyDescent="0.35">
+      <c r="C151" s="12" t="str">
+        <v>UsageArea.EastLongitude</v>
+      </c>
+      <c r="D151" s="216" t="str">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="152" spans="3:16" x14ac:dyDescent="0.35">
+      <c r="C152" s="12" t="str">
+        <v>UsageArea.NorthLatitude</v>
+      </c>
+      <c r="D152" s="216" t="str">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="153" spans="3:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="C153" s="13" t="str">
+        <v>UsageArea.Center</v>
+      </c>
+      <c r="D153" s="217" t="str">
+        <v>X=5696153.94925188, Y=484326.958550755</v>
+      </c>
+    </row>
+    <row r="154" spans="3:16" x14ac:dyDescent="0.35">
+      <c r="M154"/>
+    </row>
+    <row r="155" spans="3:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="M155"/>
+    </row>
+    <row r="156" spans="3:16" x14ac:dyDescent="0.35">
+      <c r="C156" s="41" t="s">
+        <v>142</v>
+      </c>
+      <c r="D156" s="210">
+        <v>3857</v>
+      </c>
+      <c r="K156" s="61"/>
+      <c r="M156"/>
+    </row>
+    <row r="157" spans="3:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="C157" s="13" t="s">
+        <v>143</v>
+      </c>
+      <c r="D157" s="211">
+        <v>23095</v>
+      </c>
+      <c r="K157" s="61"/>
+      <c r="M157"/>
+    </row>
+    <row r="158" spans="3:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="C158" s="182" t="str" cm="1">
+        <f t="array" ref="C158">_xll.PE.trf.Options(,,,,,55,,,,,,"Never",,,,1)</f>
+        <v>Authority=EPSG; Area=; Accuracy=55; NoBallparkConversions=False; NoDiscardIfMissing=False; UsePrimaryGridNames=False; UseSuperseded=False; StrictContains=False; IntermediateCrsUsage=Never; BestOnly=False; ForceOver=False; CandidateIndex=0; AllowDeprecatedCrs=True</v>
+      </c>
+      <c r="D158" s="183"/>
+      <c r="E158" s="183"/>
+      <c r="F158" s="183"/>
+      <c r="G158" s="183"/>
+      <c r="H158" s="183"/>
+      <c r="I158" s="183"/>
+      <c r="J158" s="183"/>
+      <c r="K158" s="183"/>
+      <c r="L158" s="183"/>
+      <c r="M158" s="183"/>
+      <c r="N158" s="183"/>
+      <c r="O158" s="184"/>
+      <c r="P158" s="184"/>
+    </row>
+    <row r="159" spans="3:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="C159" s="223" t="str" cm="1">
+        <f t="array" ref="C159:I182">_xll.PE.trf.TransformList(D156,D157,C158,"")</f>
+        <v>Transform Number</v>
+      </c>
+      <c r="D159" s="215">
+        <v>0</v>
+      </c>
+      <c r="E159" s="215">
+        <v>1</v>
+      </c>
+      <c r="F159" s="215">
+        <v>2</v>
+      </c>
+      <c r="G159" s="215">
+        <v>3</v>
+      </c>
+      <c r="H159" s="215">
+        <v>4</v>
+      </c>
+      <c r="I159" s="5">
+        <v>5</v>
+      </c>
+      <c r="M159"/>
+    </row>
+    <row r="160" spans="3:16" x14ac:dyDescent="0.35">
+      <c r="C160" s="12" t="str">
+        <v>Transform Name</v>
+      </c>
+      <c r="D160" s="212" t="str">
+        <v>Inverse of Popular Visualisation Pseudo-Mercator + Inverse of ED50 to WGS 84 (18) + TM 5 NE</v>
+      </c>
+      <c r="E160" s="212" t="str">
+        <v>Inverse of Popular Visualisation Pseudo-Mercator + Inverse of ED50 to WGS 84 (32) + TM 5 NE</v>
+      </c>
+      <c r="F160" s="212" t="str">
+        <v>Inverse of Popular Visualisation Pseudo-Mercator + Inverse of ED50 to WGS 84 (2) + TM 5 NE</v>
+      </c>
+      <c r="G160" s="172" t="str">
+        <v>Inverse of Popular Visualisation Pseudo-Mercator + Inverse of ED50 to WGS 84 (1) + TM 5 NE</v>
+      </c>
+      <c r="H160" s="172" t="str">
+        <v>Inverse of Popular Visualisation Pseudo-Mercator + Inverse of ED50 to WGS 84 (36) + TM 5 NE</v>
+      </c>
+      <c r="I160" s="179" t="str">
+        <v>Inverse of Popular Visualisation Pseudo-Mercator + Inverse of ED50 to WGS 84 (17) + TM 5 NE</v>
+      </c>
+      <c r="M160"/>
+    </row>
+    <row r="161" spans="3:13" x14ac:dyDescent="0.35">
+      <c r="C161" s="12" t="str">
+        <v>Transform Type</v>
+      </c>
+      <c r="D161" s="212" t="str">
+        <v>ConcatenatedOperation</v>
+      </c>
+      <c r="E161" s="212" t="str">
+        <v>ConcatenatedOperation</v>
+      </c>
+      <c r="F161" s="212" t="str">
+        <v>ConcatenatedOperation</v>
+      </c>
+      <c r="G161" s="172" t="str">
+        <v>ConcatenatedOperation</v>
+      </c>
+      <c r="H161" s="172" t="str">
+        <v>ConcatenatedOperation</v>
+      </c>
+      <c r="I161" s="179" t="str">
+        <v>ConcatenatedOperation</v>
+      </c>
+      <c r="M161"/>
+    </row>
+    <row r="162" spans="3:13" x14ac:dyDescent="0.35">
+      <c r="C162" s="12" t="str">
+        <v>Identifier</v>
+      </c>
+      <c r="D162" s="212" t="str">
+        <v/>
+      </c>
+      <c r="E162" s="212" t="str">
+        <v/>
+      </c>
+      <c r="F162" s="212" t="str">
+        <v/>
+      </c>
+      <c r="G162" s="172" t="str">
+        <v/>
+      </c>
+      <c r="H162" s="172" t="str">
+        <v/>
+      </c>
+      <c r="I162" s="179" t="str">
+        <v/>
+      </c>
+      <c r="M162"/>
+    </row>
+    <row r="163" spans="3:13" x14ac:dyDescent="0.35">
+      <c r="C163" s="12" t="str">
+        <v>Identifiers</v>
+      </c>
+      <c r="D163" s="212" t="str">
+        <v/>
+      </c>
+      <c r="E163" s="212" t="str">
+        <v/>
+      </c>
+      <c r="F163" s="212" t="str">
+        <v/>
+      </c>
+      <c r="G163" s="172" t="str">
+        <v/>
+      </c>
+      <c r="H163" s="172" t="str">
+        <v/>
+      </c>
+      <c r="I163" s="179" t="str">
+        <v/>
+      </c>
+      <c r="M163"/>
+    </row>
+    <row r="164" spans="3:13" x14ac:dyDescent="0.35">
+      <c r="C164" s="12" t="str">
+        <v>Accuracy</v>
+      </c>
+      <c r="D164" s="212" t="str">
+        <v>1</v>
+      </c>
+      <c r="E164" s="212" t="str">
+        <v>5</v>
+      </c>
+      <c r="F164" s="212" t="str">
+        <v>6</v>
+      </c>
+      <c r="G164" s="172" t="str">
+        <v>10</v>
+      </c>
+      <c r="H164" s="172" t="str">
+        <v>1</v>
+      </c>
+      <c r="I164" s="179" t="str">
+        <v>2</v>
+      </c>
+      <c r="M164"/>
+    </row>
+    <row r="165" spans="3:13" x14ac:dyDescent="0.35">
+      <c r="C165" s="12" t="str">
+        <v>IsAvailable</v>
+      </c>
+      <c r="D165" s="212" t="str">
+        <v>True</v>
+      </c>
+      <c r="E165" s="212" t="str">
+        <v>True</v>
+      </c>
+      <c r="F165" s="212" t="str">
+        <v>True</v>
+      </c>
+      <c r="G165" s="172" t="str">
+        <v>True</v>
+      </c>
+      <c r="H165" s="172" t="str">
+        <v>True</v>
+      </c>
+      <c r="I165" s="179" t="str">
+        <v>True</v>
+      </c>
+      <c r="M165"/>
+    </row>
+    <row r="166" spans="3:13" x14ac:dyDescent="0.35">
+      <c r="C166" s="12" t="str">
+        <v>HasBallParkTransformation</v>
+      </c>
+      <c r="D166" s="212" t="str">
+        <v>False</v>
+      </c>
+      <c r="E166" s="212" t="str">
+        <v>False</v>
+      </c>
+      <c r="F166" s="212" t="str">
+        <v>False</v>
+      </c>
+      <c r="G166" s="172" t="str">
+        <v>False</v>
+      </c>
+      <c r="H166" s="172" t="str">
+        <v>False</v>
+      </c>
+      <c r="I166" s="179" t="str">
+        <v>False</v>
+      </c>
+      <c r="M166"/>
+    </row>
+    <row r="167" spans="3:13" x14ac:dyDescent="0.35">
+      <c r="C167" s="12" t="str">
+        <v>HasInverse</v>
+      </c>
+      <c r="D167" s="212" t="str">
+        <v>True</v>
+      </c>
+      <c r="E167" s="212" t="str">
+        <v>True</v>
+      </c>
+      <c r="F167" s="212" t="str">
+        <v>True</v>
+      </c>
+      <c r="G167" s="172" t="str">
+        <v>True</v>
+      </c>
+      <c r="H167" s="172" t="str">
+        <v>True</v>
+      </c>
+      <c r="I167" s="179" t="str">
+        <v>True</v>
+      </c>
+      <c r="M167"/>
+    </row>
+    <row r="168" spans="3:13" x14ac:dyDescent="0.35">
+      <c r="C168" s="12" t="str">
+        <v>MethodName</v>
+      </c>
+      <c r="D168" s="212" t="str">
+        <v/>
+      </c>
+      <c r="E168" s="212" t="str">
+        <v/>
+      </c>
+      <c r="F168" s="212" t="str">
+        <v/>
+      </c>
+      <c r="G168" s="172" t="str">
+        <v/>
+      </c>
+      <c r="H168" s="172" t="str">
+        <v/>
+      </c>
+      <c r="I168" s="179" t="str">
+        <v/>
+      </c>
+      <c r="M168"/>
+    </row>
+    <row r="169" spans="3:13" x14ac:dyDescent="0.35">
+      <c r="C169" s="12" t="str">
+        <v>Scope</v>
+      </c>
+      <c r="D169" s="212" t="str">
+        <v/>
+      </c>
+      <c r="E169" s="212" t="str">
+        <v/>
+      </c>
+      <c r="F169" s="212" t="str">
+        <v/>
+      </c>
+      <c r="G169" s="172" t="str">
+        <v/>
+      </c>
+      <c r="H169" s="172" t="str">
+        <v/>
+      </c>
+      <c r="I169" s="179" t="str">
+        <v/>
+      </c>
+      <c r="M169"/>
+    </row>
+    <row r="170" spans="3:13" x14ac:dyDescent="0.35">
+      <c r="C170" s="12" t="str">
+        <v>Remarks</v>
+      </c>
+      <c r="D170" s="212" t="str">
+        <v/>
+      </c>
+      <c r="E170" s="212" t="str">
+        <v/>
+      </c>
+      <c r="F170" s="212" t="str">
+        <v/>
+      </c>
+      <c r="G170" s="172" t="str">
+        <v/>
+      </c>
+      <c r="H170" s="172" t="str">
+        <v/>
+      </c>
+      <c r="I170" s="179" t="str">
+        <v/>
+      </c>
+      <c r="M170"/>
+    </row>
+    <row r="171" spans="3:13" x14ac:dyDescent="0.35">
+      <c r="C171" s="12" t="str">
+        <v>GridUsages</v>
+      </c>
+      <c r="D171" s="212" t="str">
+        <v/>
+      </c>
+      <c r="E171" s="212" t="str">
+        <v/>
+      </c>
+      <c r="F171" s="212" t="str">
+        <v/>
+      </c>
+      <c r="G171" s="172" t="str">
+        <v/>
+      </c>
+      <c r="H171" s="172" t="str">
+        <v/>
+      </c>
+      <c r="I171" s="179" t="str">
+        <v/>
+      </c>
+      <c r="M171"/>
+    </row>
+    <row r="172" spans="3:13" x14ac:dyDescent="0.35">
+      <c r="C172" s="12" t="str">
+        <v>Parameters</v>
+      </c>
+      <c r="D172" s="212" t="str">
+        <v/>
+      </c>
+      <c r="E172" s="212" t="str">
+        <v/>
+      </c>
+      <c r="F172" s="212" t="str">
+        <v/>
+      </c>
+      <c r="G172" s="172" t="str">
+        <v/>
+      </c>
+      <c r="H172" s="172" t="str">
+        <v/>
+      </c>
+      <c r="I172" s="179" t="str">
+        <v/>
+      </c>
+      <c r="M172"/>
+    </row>
+    <row r="173" spans="3:13" x14ac:dyDescent="0.35">
+      <c r="C173" s="12" t="str">
+        <v>SourceCRS</v>
+      </c>
+      <c r="D173" s="212" t="str">
+        <v>WGS 84 / Pseudo-Mercator</v>
+      </c>
+      <c r="E173" s="212" t="str">
+        <v>WGS 84 / Pseudo-Mercator</v>
+      </c>
+      <c r="F173" s="212" t="str">
+        <v>WGS 84 / Pseudo-Mercator</v>
+      </c>
+      <c r="G173" s="172" t="str">
+        <v>WGS 84 / Pseudo-Mercator</v>
+      </c>
+      <c r="H173" s="172" t="str">
+        <v>WGS 84 / Pseudo-Mercator</v>
+      </c>
+      <c r="I173" s="179" t="str">
+        <v>WGS 84 / Pseudo-Mercator</v>
+      </c>
+      <c r="M173"/>
+    </row>
+    <row r="174" spans="3:13" x14ac:dyDescent="0.35">
+      <c r="C174" s="12" t="str">
+        <v>TargetCRS</v>
+      </c>
+      <c r="D174" s="212" t="str">
+        <v>ED50 / TM 5 NE</v>
+      </c>
+      <c r="E174" s="212" t="str">
+        <v>ED50 / TM 5 NE</v>
+      </c>
+      <c r="F174" s="212" t="str">
+        <v>ED50 / TM 5 NE</v>
+      </c>
+      <c r="G174" s="172" t="str">
+        <v>ED50 / TM 5 NE</v>
+      </c>
+      <c r="H174" s="172" t="str">
+        <v>ED50 / TM 5 NE</v>
+      </c>
+      <c r="I174" s="179" t="str">
+        <v>ED50 / TM 5 NE</v>
+      </c>
+      <c r="M174"/>
+    </row>
+    <row r="175" spans="3:13" x14ac:dyDescent="0.35">
+      <c r="C175" s="12" t="str">
+        <v>Context</v>
+      </c>
+      <c r="D175" s="212" t="str">
+        <v>LogLevel=Error; EndpointUrl=https://cdn.proj.org; EnableNetworkConnections=True</v>
+      </c>
+      <c r="E175" s="212" t="str">
+        <v>LogLevel=Error; EndpointUrl=https://cdn.proj.org; EnableNetworkConnections=True</v>
+      </c>
+      <c r="F175" s="212" t="str">
+        <v>LogLevel=Error; EndpointUrl=https://cdn.proj.org; EnableNetworkConnections=True</v>
+      </c>
+      <c r="G175" s="172" t="str">
+        <v>LogLevel=Error; EndpointUrl=https://cdn.proj.org; EnableNetworkConnections=True</v>
+      </c>
+      <c r="H175" s="172" t="str">
+        <v>LogLevel=Error; EndpointUrl=https://cdn.proj.org; EnableNetworkConnections=True</v>
+      </c>
+      <c r="I175" s="179" t="str">
+        <v>LogLevel=Error; EndpointUrl=https://cdn.proj.org; EnableNetworkConnections=True</v>
+      </c>
+      <c r="M175"/>
+    </row>
+    <row r="176" spans="3:13" x14ac:dyDescent="0.35">
+      <c r="C176" s="12" t="str">
+        <v>UsageArea</v>
+      </c>
+      <c r="D176" s="212" t="str">
+        <v>UsageArea</v>
+      </c>
+      <c r="E176" s="212" t="str">
+        <v>UsageArea</v>
+      </c>
+      <c r="F176" s="212" t="str">
+        <v>UsageArea</v>
+      </c>
+      <c r="G176" s="172" t="str">
+        <v>UsageArea</v>
+      </c>
+      <c r="H176" s="172" t="str">
+        <v>UsageArea</v>
+      </c>
+      <c r="I176" s="179" t="str">
+        <v>UsageArea</v>
+      </c>
+      <c r="M176"/>
+    </row>
+    <row r="177" spans="2:16" x14ac:dyDescent="0.35">
+      <c r="C177" s="12" t="str">
+        <v>UsageArea.Name</v>
+      </c>
+      <c r="D177" s="212" t="str">
+        <v>Denmark - offshore North Sea; Ireland - offshore; Netherlands - offshore; United Kingdom - UKCS offshore.</v>
+      </c>
+      <c r="E177" s="212" t="str">
+        <v>Netherlands - offshore North Sea.</v>
+      </c>
+      <c r="F177" s="212" t="str">
+        <v>Austria; Denmark; France; Germany (west); Netherlands; Switzerland.</v>
+      </c>
+      <c r="G177" s="172" t="str">
+        <v>Austria; Belgium; Denmark; Finland; Faroe islands; France; Germany (west); Gibraltar; Greece; Italy; Luxembourg; Netherlands; Norway; Portugal; Spain; Sweden; Switzerland.</v>
+      </c>
+      <c r="H177" s="172" t="str">
+        <v>Germany - offshore North Sea.</v>
+      </c>
+      <c r="I177" s="179" t="str">
+        <v>France - onshore and offshore, mainland and Corsica (France métropolitaine including Corsica).</v>
+      </c>
+      <c r="M177"/>
+    </row>
+    <row r="178" spans="2:16" x14ac:dyDescent="0.35">
+      <c r="C178" s="12" t="str">
+        <v>UsageArea.WestLongitude</v>
+      </c>
+      <c r="D178" s="212" t="str">
+        <v>-16.1</v>
+      </c>
+      <c r="E178" s="212" t="str">
+        <v>2.53</v>
+      </c>
+      <c r="F178" s="212" t="str">
+        <v>-4.87</v>
+      </c>
+      <c r="G178" s="172" t="str">
+        <v>-9.56</v>
+      </c>
+      <c r="H178" s="172" t="str">
+        <v>3.34</v>
+      </c>
+      <c r="I178" s="179" t="str">
+        <v>-9.86</v>
+      </c>
+      <c r="M178"/>
+    </row>
+    <row r="179" spans="2:16" x14ac:dyDescent="0.35">
+      <c r="C179" s="12" t="str">
+        <v>UsageArea.SouthLatitude</v>
+      </c>
+      <c r="D179" s="212" t="str">
+        <v>47.42</v>
+      </c>
+      <c r="E179" s="212" t="str">
+        <v>51.44</v>
+      </c>
+      <c r="F179" s="212" t="str">
+        <v>42.33</v>
+      </c>
+      <c r="G179" s="172" t="str">
+        <v>34.88</v>
+      </c>
+      <c r="H179" s="172" t="str">
+        <v>53.58</v>
+      </c>
+      <c r="I179" s="179" t="str">
+        <v>41.15</v>
+      </c>
+      <c r="M179"/>
+    </row>
+    <row r="180" spans="2:16" x14ac:dyDescent="0.35">
+      <c r="C180" s="12" t="str">
+        <v>UsageArea.EastLongitude</v>
+      </c>
+      <c r="D180" s="212" t="str">
+        <v>10.86</v>
+      </c>
+      <c r="E180" s="212" t="str">
+        <v>6.37</v>
+      </c>
+      <c r="F180" s="212" t="str">
+        <v>17.17</v>
+      </c>
+      <c r="G180" s="172" t="str">
+        <v>31.59</v>
+      </c>
+      <c r="H180" s="172" t="str">
+        <v>8.88</v>
+      </c>
+      <c r="I180" s="179" t="str">
+        <v>10.38</v>
+      </c>
+      <c r="M180"/>
+    </row>
+    <row r="181" spans="2:16" x14ac:dyDescent="0.35">
+      <c r="C181" s="12" t="str">
+        <v>UsageArea.NorthLatitude</v>
+      </c>
+      <c r="D181" s="212" t="str">
+        <v>63.89</v>
+      </c>
+      <c r="E181" s="212" t="str">
+        <v>55.77</v>
+      </c>
+      <c r="F181" s="212" t="str">
+        <v>57.8</v>
+      </c>
+      <c r="G181" s="172" t="str">
+        <v>71.24</v>
+      </c>
+      <c r="H181" s="172" t="str">
+        <v>55.92</v>
+      </c>
+      <c r="I181" s="179" t="str">
+        <v>51.56</v>
+      </c>
+      <c r="M181"/>
+    </row>
+    <row r="182" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="C182" s="13" t="str">
+        <v>UsageArea.Center</v>
+      </c>
+      <c r="D182" s="213" t="str">
+        <v>X=-291657.065878377, Y=7666392.98144475</v>
+      </c>
+      <c r="E182" s="213" t="str">
+        <v>X=495371.734030067, Y=7106130.774072</v>
+      </c>
+      <c r="F182" s="213" t="str">
+        <v>X=684614.868378632, Y=6567980.67490485</v>
+      </c>
+      <c r="G182" s="214" t="str">
+        <v>X=1226184.19108791, Y=7816211.44812981</v>
+      </c>
+      <c r="H182" s="214" t="str">
+        <v>X=680162.088746901, Y=7316758.79219274</v>
+      </c>
+      <c r="I182" s="181" t="str">
+        <v>X=28943.0676062511, Y=5877723.68014364</v>
+      </c>
+      <c r="M182"/>
+    </row>
+    <row r="183" spans="2:16" x14ac:dyDescent="0.35">
+      <c r="M183"/>
+    </row>
+    <row r="184" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="M184"/>
+    </row>
+    <row r="185" spans="2:16" x14ac:dyDescent="0.35">
+      <c r="C185" s="41" t="s">
+        <v>142</v>
+      </c>
+      <c r="D185" s="210">
+        <v>2964</v>
+      </c>
+      <c r="E185" s="222" t="s">
+        <v>144</v>
+      </c>
+      <c r="M185"/>
+    </row>
+    <row r="186" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="C186" s="12" t="s">
+        <v>143</v>
+      </c>
+      <c r="D186" s="221">
+        <v>4326</v>
+      </c>
+      <c r="E186" s="222" t="s">
+        <v>145</v>
+      </c>
+      <c r="M186"/>
+    </row>
+    <row r="187" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="C187" s="182" t="str" cm="1">
+        <f t="array" ref="C187">_xll.PE.trf.Options(,,,,,,,,,,,,0,,,)</f>
         <v>Authority=EPSG; Area=; Accuracy=; NoBallparkConversions=False; NoDiscardIfMissing=False; UsePrimaryGridNames=False; UseSuperseded=False; StrictContains=False; IntermediateCrsUsage=Auto; BestOnly=False; ForceOver=False; CandidateIndex=0; AllowDeprecatedCrs=False</v>
       </c>
-      <c r="D128" s="183"/>
-      <c r="E128" s="183"/>
-      <c r="F128" s="183"/>
-      <c r="G128" s="183"/>
-      <c r="H128" s="183"/>
-      <c r="I128" s="183"/>
-      <c r="J128" s="183"/>
-      <c r="K128" s="183"/>
-      <c r="L128" s="183"/>
-      <c r="M128" s="183"/>
-      <c r="N128" s="183"/>
-      <c r="O128" s="204"/>
-      <c r="P128" s="183"/>
-      <c r="Q128" s="184"/>
-    </row>
-    <row r="129" spans="3:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="F129" s="180" cm="1">
-        <f t="array" ref="F129:G129">_xll.PE.trf.LatLongToWebMercatorEx(G123,F123,C127)</f>
-        <v>4488904.7260120427</v>
-      </c>
-      <c r="G129" s="181">
-        <v>2316761.8960968899</v>
-      </c>
-      <c r="I129" s="180" cm="1">
-        <f t="array" ref="I129:J129">_xll.PE.trf.LatLongToWebMercator(G123,F123)</f>
-        <v>2267435.056226131</v>
-      </c>
-      <c r="J129" s="181">
-        <v>4913212.9116666559</v>
-      </c>
-      <c r="M129"/>
-    </row>
-    <row r="130" spans="3:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="C130" s="173" t="s">
-        <v>136</v>
-      </c>
-      <c r="D130" s="172" t="str" cm="1">
-        <f t="array" ref="D130">_xll.PE.crs.GeodeticCRS.Name(D4)</f>
-        <v>Albanian 1987</v>
-      </c>
-      <c r="F130" s="213">
-        <v>2267435.0562261301</v>
-      </c>
-      <c r="G130" s="214">
-        <v>4913212.9116666559</v>
-      </c>
-      <c r="I130" s="213">
-        <v>2267435.056226131</v>
-      </c>
-      <c r="J130" s="214">
-        <v>4913212.9116666559</v>
-      </c>
-      <c r="M130"/>
-    </row>
-    <row r="131" spans="3:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="C131" s="12" t="s">
-        <v>137</v>
-      </c>
-      <c r="D131" s="172" t="str" cm="1">
-        <f t="array" ref="D131">_xll.PE.crs.GeodeticCRS.Type(D4)</f>
-        <v>Geographic2DCrs</v>
-      </c>
-      <c r="F131" s="215">
-        <f>F129-F130</f>
-        <v>2221469.6697859126</v>
-      </c>
-      <c r="G131" s="216">
-        <f>G129-G130</f>
-        <v>-2596451.0155697661</v>
-      </c>
-      <c r="I131" s="215">
-        <f>I129-I130</f>
+      <c r="D187" s="183"/>
+      <c r="E187" s="183"/>
+      <c r="F187" s="183"/>
+      <c r="G187" s="183"/>
+      <c r="H187" s="183"/>
+      <c r="I187" s="183"/>
+      <c r="J187" s="183"/>
+      <c r="K187" s="183"/>
+      <c r="L187" s="183"/>
+      <c r="M187" s="183"/>
+      <c r="N187" s="183"/>
+      <c r="O187" s="184"/>
+      <c r="P187" s="184"/>
+    </row>
+    <row r="188" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B188"/>
+      <c r="C188" s="223" t="str" cm="1">
+        <f t="array" ref="C188:M211">_xll.PE.trf.TransformList(D185,D186,C187, "")</f>
+        <v>Transform Number</v>
+      </c>
+      <c r="D188" s="215">
         <v>0</v>
       </c>
-      <c r="J131" s="216">
-        <f>J129-J130</f>
+      <c r="E188" s="215">
+        <v>1</v>
+      </c>
+      <c r="F188" s="215">
+        <v>2</v>
+      </c>
+      <c r="G188" s="215">
+        <v>3</v>
+      </c>
+      <c r="H188" s="215">
+        <v>4</v>
+      </c>
+      <c r="I188" s="215">
+        <v>5</v>
+      </c>
+      <c r="J188" s="215">
+        <v>6</v>
+      </c>
+      <c r="K188" s="215">
+        <v>7</v>
+      </c>
+      <c r="L188" s="215">
+        <v>8</v>
+      </c>
+      <c r="M188" s="5">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="189" spans="2:16" x14ac:dyDescent="0.35">
+      <c r="B189"/>
+      <c r="C189" s="12" t="str">
+        <v>Transform Name</v>
+      </c>
+      <c r="D189" s="212" t="str">
+        <v>Inverse of Alaska Albers + NAD27 to WGS 84 (85) + axis order change (2D)</v>
+      </c>
+      <c r="E189" s="212" t="str">
+        <v>Inverse of Alaska Albers + NAD27 to WGS 84 (7) + axis order change (2D)</v>
+      </c>
+      <c r="F189" s="212" t="str">
+        <v>Inverse of Alaska Albers + NAD27 to WGS 84 (33) + axis order change (2D)</v>
+      </c>
+      <c r="G189" s="212" t="str">
+        <v>Inverse of Alaska Albers + NAD27 to WGS 84 (3) + axis order change (2D)</v>
+      </c>
+      <c r="H189" s="212" t="str">
+        <v>Inverse of Alaska Albers + NAD27 to WGS 84 (13) + axis order change (2D)</v>
+      </c>
+      <c r="I189" s="212" t="str">
+        <v>Inverse of Alaska Albers + NAD27 to WGS 84 (14) + axis order change (2D)</v>
+      </c>
+      <c r="J189" s="212" t="str">
+        <v>Inverse of Alaska Albers + NAD27 to WGS 84 (10) + axis order change (2D)</v>
+      </c>
+      <c r="K189" s="212" t="str">
+        <v>Inverse of Alaska Albers + NAD27 to WGS 84 (21) + axis order change (2D)</v>
+      </c>
+      <c r="L189" s="212" t="str">
+        <v>Inverse of Alaska Albers + NAD27 to WGS 84 (22) + axis order change (2D)</v>
+      </c>
+      <c r="M189" s="219" t="str">
+        <v>Inverse of Alaska Albers + Ballpark geographic offset from NAD27 to WGS 84 (with axis order normalized for visualization)</v>
+      </c>
+    </row>
+    <row r="190" spans="2:16" x14ac:dyDescent="0.35">
+      <c r="B190"/>
+      <c r="C190" s="12" t="str">
+        <v>Transform Type</v>
+      </c>
+      <c r="D190" s="212" t="str">
+        <v>ConcatenatedOperation</v>
+      </c>
+      <c r="E190" s="212" t="str">
+        <v>ConcatenatedOperation</v>
+      </c>
+      <c r="F190" s="212" t="str">
+        <v>ConcatenatedOperation</v>
+      </c>
+      <c r="G190" s="212" t="str">
+        <v>ConcatenatedOperation</v>
+      </c>
+      <c r="H190" s="212" t="str">
+        <v>ConcatenatedOperation</v>
+      </c>
+      <c r="I190" s="212" t="str">
+        <v>ConcatenatedOperation</v>
+      </c>
+      <c r="J190" s="212" t="str">
+        <v>ConcatenatedOperation</v>
+      </c>
+      <c r="K190" s="212" t="str">
+        <v>ConcatenatedOperation</v>
+      </c>
+      <c r="L190" s="212" t="str">
+        <v>ConcatenatedOperation</v>
+      </c>
+      <c r="M190" s="219" t="str">
+        <v>ConcatenatedOperation</v>
+      </c>
+    </row>
+    <row r="191" spans="2:16" x14ac:dyDescent="0.35">
+      <c r="B191"/>
+      <c r="C191" s="12" t="str">
+        <v>Identifier</v>
+      </c>
+      <c r="D191" s="212" t="str">
+        <v/>
+      </c>
+      <c r="E191" s="212" t="str">
+        <v/>
+      </c>
+      <c r="F191" s="212" t="str">
+        <v/>
+      </c>
+      <c r="G191" s="212" t="str">
+        <v/>
+      </c>
+      <c r="H191" s="212" t="str">
+        <v/>
+      </c>
+      <c r="I191" s="212" t="str">
+        <v/>
+      </c>
+      <c r="J191" s="212" t="str">
+        <v/>
+      </c>
+      <c r="K191" s="212" t="str">
+        <v/>
+      </c>
+      <c r="L191" s="212" t="str">
+        <v/>
+      </c>
+      <c r="M191" s="219" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="192" spans="2:16" x14ac:dyDescent="0.35">
+      <c r="B192"/>
+      <c r="C192" s="12" t="str">
+        <v>Identifiers</v>
+      </c>
+      <c r="D192" s="212" t="str">
+        <v/>
+      </c>
+      <c r="E192" s="212" t="str">
+        <v/>
+      </c>
+      <c r="F192" s="212" t="str">
+        <v/>
+      </c>
+      <c r="G192" s="212" t="str">
+        <v/>
+      </c>
+      <c r="H192" s="212" t="str">
+        <v/>
+      </c>
+      <c r="I192" s="212" t="str">
+        <v/>
+      </c>
+      <c r="J192" s="212" t="str">
+        <v/>
+      </c>
+      <c r="K192" s="212" t="str">
+        <v/>
+      </c>
+      <c r="L192" s="212" t="str">
+        <v/>
+      </c>
+      <c r="M192" s="219" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="193" spans="2:15" x14ac:dyDescent="0.35">
+      <c r="B193"/>
+      <c r="C193" s="12" t="str">
+        <v>Accuracy</v>
+      </c>
+      <c r="D193" s="212" t="str">
+        <v>5</v>
+      </c>
+      <c r="E193" s="212" t="str">
+        <v>12</v>
+      </c>
+      <c r="F193" s="212" t="str">
+        <v>2</v>
+      </c>
+      <c r="G193" s="212" t="str">
+        <v>20</v>
+      </c>
+      <c r="H193" s="212" t="str">
+        <v>8</v>
+      </c>
+      <c r="I193" s="212" t="str">
+        <v>10</v>
+      </c>
+      <c r="J193" s="212" t="str">
+        <v>13</v>
+      </c>
+      <c r="K193" s="212" t="str">
+        <v>15</v>
+      </c>
+      <c r="L193" s="212" t="str">
+        <v>18</v>
+      </c>
+      <c r="M193" s="219" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="194" spans="2:15" x14ac:dyDescent="0.35">
+      <c r="B194"/>
+      <c r="C194" s="12" t="str">
+        <v>IsAvailable</v>
+      </c>
+      <c r="D194" s="212" t="str">
+        <v>True</v>
+      </c>
+      <c r="E194" s="212" t="str">
+        <v>True</v>
+      </c>
+      <c r="F194" s="212" t="str">
+        <v>True</v>
+      </c>
+      <c r="G194" s="212" t="str">
+        <v>True</v>
+      </c>
+      <c r="H194" s="212" t="str">
+        <v>True</v>
+      </c>
+      <c r="I194" s="212" t="str">
+        <v>True</v>
+      </c>
+      <c r="J194" s="212" t="str">
+        <v>True</v>
+      </c>
+      <c r="K194" s="212" t="str">
+        <v>True</v>
+      </c>
+      <c r="L194" s="212" t="str">
+        <v>True</v>
+      </c>
+      <c r="M194" s="219" t="str">
+        <v>True</v>
+      </c>
+    </row>
+    <row r="195" spans="2:15" x14ac:dyDescent="0.35">
+      <c r="B195"/>
+      <c r="C195" s="12" t="str">
+        <v>HasBallParkTransformation</v>
+      </c>
+      <c r="D195" s="212" t="str">
+        <v>False</v>
+      </c>
+      <c r="E195" s="212" t="str">
+        <v>False</v>
+      </c>
+      <c r="F195" s="212" t="str">
+        <v>False</v>
+      </c>
+      <c r="G195" s="212" t="str">
+        <v>False</v>
+      </c>
+      <c r="H195" s="212" t="str">
+        <v>False</v>
+      </c>
+      <c r="I195" s="212" t="str">
+        <v>False</v>
+      </c>
+      <c r="J195" s="212" t="str">
+        <v>False</v>
+      </c>
+      <c r="K195" s="212" t="str">
+        <v>False</v>
+      </c>
+      <c r="L195" s="212" t="str">
+        <v>False</v>
+      </c>
+      <c r="M195" s="219" t="str">
+        <v>True</v>
+      </c>
+    </row>
+    <row r="196" spans="2:15" x14ac:dyDescent="0.35">
+      <c r="B196"/>
+      <c r="C196" s="12" t="str">
+        <v>HasInverse</v>
+      </c>
+      <c r="D196" s="212" t="str">
+        <v>True</v>
+      </c>
+      <c r="E196" s="212" t="str">
+        <v>True</v>
+      </c>
+      <c r="F196" s="212" t="str">
+        <v>True</v>
+      </c>
+      <c r="G196" s="212" t="str">
+        <v>True</v>
+      </c>
+      <c r="H196" s="212" t="str">
+        <v>True</v>
+      </c>
+      <c r="I196" s="212" t="str">
+        <v>True</v>
+      </c>
+      <c r="J196" s="212" t="str">
+        <v>True</v>
+      </c>
+      <c r="K196" s="212" t="str">
+        <v>True</v>
+      </c>
+      <c r="L196" s="212" t="str">
+        <v>True</v>
+      </c>
+      <c r="M196" s="219" t="str">
+        <v>True</v>
+      </c>
+    </row>
+    <row r="197" spans="2:15" x14ac:dyDescent="0.35">
+      <c r="B197"/>
+      <c r="C197" s="12" t="str">
+        <v>MethodName</v>
+      </c>
+      <c r="D197" s="212" t="str">
+        <v/>
+      </c>
+      <c r="E197" s="212" t="str">
+        <v/>
+      </c>
+      <c r="F197" s="212" t="str">
+        <v/>
+      </c>
+      <c r="G197" s="212" t="str">
+        <v/>
+      </c>
+      <c r="H197" s="212" t="str">
+        <v/>
+      </c>
+      <c r="I197" s="212" t="str">
+        <v/>
+      </c>
+      <c r="J197" s="212" t="str">
+        <v/>
+      </c>
+      <c r="K197" s="212" t="str">
+        <v/>
+      </c>
+      <c r="L197" s="212" t="str">
+        <v/>
+      </c>
+      <c r="M197" s="219" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="198" spans="2:15" x14ac:dyDescent="0.35">
+      <c r="B198"/>
+      <c r="C198" s="12" t="str">
+        <v>Scope</v>
+      </c>
+      <c r="D198" s="212" t="str">
+        <v/>
+      </c>
+      <c r="E198" s="212" t="str">
+        <v/>
+      </c>
+      <c r="F198" s="212" t="str">
+        <v/>
+      </c>
+      <c r="G198" s="212" t="str">
+        <v/>
+      </c>
+      <c r="H198" s="212" t="str">
+        <v/>
+      </c>
+      <c r="I198" s="212" t="str">
+        <v/>
+      </c>
+      <c r="J198" s="212" t="str">
+        <v/>
+      </c>
+      <c r="K198" s="212" t="str">
+        <v/>
+      </c>
+      <c r="L198" s="212" t="str">
+        <v/>
+      </c>
+      <c r="M198" s="219" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="199" spans="2:15" x14ac:dyDescent="0.35">
+      <c r="B199"/>
+      <c r="C199" s="12" t="str">
+        <v>Remarks</v>
+      </c>
+      <c r="D199" s="212" t="str">
+        <v/>
+      </c>
+      <c r="E199" s="212" t="str">
+        <v/>
+      </c>
+      <c r="F199" s="212" t="str">
+        <v/>
+      </c>
+      <c r="G199" s="212" t="str">
+        <v/>
+      </c>
+      <c r="H199" s="212" t="str">
+        <v/>
+      </c>
+      <c r="I199" s="212" t="str">
+        <v/>
+      </c>
+      <c r="J199" s="212" t="str">
+        <v/>
+      </c>
+      <c r="K199" s="212" t="str">
+        <v/>
+      </c>
+      <c r="L199" s="212" t="str">
+        <v/>
+      </c>
+      <c r="M199" s="219" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="200" spans="2:15" x14ac:dyDescent="0.35">
+      <c r="B200"/>
+      <c r="C200" s="12" t="str">
+        <v>GridUsages</v>
+      </c>
+      <c r="D200" s="212" t="str">
+        <v/>
+      </c>
+      <c r="E200" s="212" t="str">
+        <v/>
+      </c>
+      <c r="F200" s="212" t="str">
+        <v/>
+      </c>
+      <c r="G200" s="212" t="str">
+        <v/>
+      </c>
+      <c r="H200" s="212" t="str">
+        <v/>
+      </c>
+      <c r="I200" s="212" t="str">
+        <v/>
+      </c>
+      <c r="J200" s="212" t="str">
+        <v/>
+      </c>
+      <c r="K200" s="212" t="str">
+        <v/>
+      </c>
+      <c r="L200" s="212" t="str">
+        <v/>
+      </c>
+      <c r="M200" s="219" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="201" spans="2:15" x14ac:dyDescent="0.35">
+      <c r="B201"/>
+      <c r="C201" s="12" t="str">
+        <v>Parameters</v>
+      </c>
+      <c r="D201" s="212" t="str">
+        <v/>
+      </c>
+      <c r="E201" s="212" t="str">
+        <v/>
+      </c>
+      <c r="F201" s="212" t="str">
+        <v/>
+      </c>
+      <c r="G201" s="212" t="str">
+        <v/>
+      </c>
+      <c r="H201" s="212" t="str">
+        <v/>
+      </c>
+      <c r="I201" s="212" t="str">
+        <v/>
+      </c>
+      <c r="J201" s="212" t="str">
+        <v/>
+      </c>
+      <c r="K201" s="212" t="str">
+        <v/>
+      </c>
+      <c r="L201" s="212" t="str">
+        <v/>
+      </c>
+      <c r="M201" s="219" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="202" spans="2:15" x14ac:dyDescent="0.35">
+      <c r="B202"/>
+      <c r="C202" s="12" t="str">
+        <v>SourceCRS</v>
+      </c>
+      <c r="D202" s="212" t="str">
+        <v>NAD27 / Alaska Albers</v>
+      </c>
+      <c r="E202" s="212" t="str">
+        <v>NAD27 / Alaska Albers</v>
+      </c>
+      <c r="F202" s="212" t="str">
+        <v>NAD27 / Alaska Albers</v>
+      </c>
+      <c r="G202" s="212" t="str">
+        <v>NAD27 / Alaska Albers</v>
+      </c>
+      <c r="H202" s="212" t="str">
+        <v>NAD27 / Alaska Albers</v>
+      </c>
+      <c r="I202" s="212" t="str">
+        <v>NAD27 / Alaska Albers</v>
+      </c>
+      <c r="J202" s="212" t="str">
+        <v>NAD27 / Alaska Albers</v>
+      </c>
+      <c r="K202" s="212" t="str">
+        <v>NAD27 / Alaska Albers</v>
+      </c>
+      <c r="L202" s="212" t="str">
+        <v>NAD27 / Alaska Albers</v>
+      </c>
+      <c r="M202" s="219" t="str">
+        <v>NAD27 / Alaska Albers</v>
+      </c>
+    </row>
+    <row r="203" spans="2:15" x14ac:dyDescent="0.35">
+      <c r="B203"/>
+      <c r="C203" s="12" t="str">
+        <v>TargetCRS</v>
+      </c>
+      <c r="D203" s="212" t="str">
+        <v>WGS 84 (with axis order normalized for visualization)</v>
+      </c>
+      <c r="E203" s="212" t="str">
+        <v>WGS 84 (with axis order normalized for visualization)</v>
+      </c>
+      <c r="F203" s="212" t="str">
+        <v>WGS 84 (with axis order normalized for visualization)</v>
+      </c>
+      <c r="G203" s="212" t="str">
+        <v>WGS 84 (with axis order normalized for visualization)</v>
+      </c>
+      <c r="H203" s="212" t="str">
+        <v>WGS 84 (with axis order normalized for visualization)</v>
+      </c>
+      <c r="I203" s="212" t="str">
+        <v>WGS 84 (with axis order normalized for visualization)</v>
+      </c>
+      <c r="J203" s="212" t="str">
+        <v>WGS 84 (with axis order normalized for visualization)</v>
+      </c>
+      <c r="K203" s="212" t="str">
+        <v>WGS 84 (with axis order normalized for visualization)</v>
+      </c>
+      <c r="L203" s="212" t="str">
+        <v>WGS 84 (with axis order normalized for visualization)</v>
+      </c>
+      <c r="M203" s="219" t="str">
+        <v>WGS 84 (with axis order normalized for visualization)</v>
+      </c>
+    </row>
+    <row r="204" spans="2:15" x14ac:dyDescent="0.35">
+      <c r="B204"/>
+      <c r="C204" s="12" t="str">
+        <v>Context</v>
+      </c>
+      <c r="D204" s="212" t="str">
+        <v>LogLevel=Error; EndpointUrl=https://cdn.proj.org; EnableNetworkConnections=True</v>
+      </c>
+      <c r="E204" s="212" t="str">
+        <v>LogLevel=Error; EndpointUrl=https://cdn.proj.org; EnableNetworkConnections=True</v>
+      </c>
+      <c r="F204" s="212" t="str">
+        <v>LogLevel=Error; EndpointUrl=https://cdn.proj.org; EnableNetworkConnections=True</v>
+      </c>
+      <c r="G204" s="212" t="str">
+        <v>LogLevel=Error; EndpointUrl=https://cdn.proj.org; EnableNetworkConnections=True</v>
+      </c>
+      <c r="H204" s="212" t="str">
+        <v>LogLevel=Error; EndpointUrl=https://cdn.proj.org; EnableNetworkConnections=True</v>
+      </c>
+      <c r="I204" s="212" t="str">
+        <v>LogLevel=Error; EndpointUrl=https://cdn.proj.org; EnableNetworkConnections=True</v>
+      </c>
+      <c r="J204" s="212" t="str">
+        <v>LogLevel=Error; EndpointUrl=https://cdn.proj.org; EnableNetworkConnections=True</v>
+      </c>
+      <c r="K204" s="212" t="str">
+        <v>LogLevel=Error; EndpointUrl=https://cdn.proj.org; EnableNetworkConnections=True</v>
+      </c>
+      <c r="L204" s="212" t="str">
+        <v>LogLevel=Error; EndpointUrl=https://cdn.proj.org; EnableNetworkConnections=True</v>
+      </c>
+      <c r="M204" s="219" t="str">
+        <v>LogLevel=Error; EndpointUrl=https://cdn.proj.org; EnableNetworkConnections=True</v>
+      </c>
+    </row>
+    <row r="205" spans="2:15" x14ac:dyDescent="0.35">
+      <c r="B205"/>
+      <c r="C205" s="12" t="str">
+        <v>UsageArea</v>
+      </c>
+      <c r="D205" s="212" t="str">
+        <v>UsageArea</v>
+      </c>
+      <c r="E205" s="212" t="str">
+        <v>UsageArea</v>
+      </c>
+      <c r="F205" s="212" t="str">
+        <v>UsageArea</v>
+      </c>
+      <c r="G205" s="212" t="str">
+        <v>UsageArea</v>
+      </c>
+      <c r="H205" s="212" t="str">
+        <v>UsageArea</v>
+      </c>
+      <c r="I205" s="212" t="str">
+        <v>UsageArea</v>
+      </c>
+      <c r="J205" s="212" t="str">
+        <v>UsageArea</v>
+      </c>
+      <c r="K205" s="212" t="str">
+        <v>UsageArea</v>
+      </c>
+      <c r="L205" s="212" t="str">
+        <v>UsageArea</v>
+      </c>
+      <c r="M205" s="219" t="str">
+        <v>UsageArea</v>
+      </c>
+      <c r="O205"/>
+    </row>
+    <row r="206" spans="2:15" x14ac:dyDescent="0.35">
+      <c r="B206"/>
+      <c r="C206" s="12" t="str">
+        <v>UsageArea.Name</v>
+      </c>
+      <c r="D206" s="212" t="str">
+        <v>United States (USA) - Alaska including EEZ.</v>
+      </c>
+      <c r="E206" s="212" t="str">
+        <v>United States (USA) - Alaska mainland.</v>
+      </c>
+      <c r="F206" s="212" t="str">
+        <v>Canada - onshore - Alberta; British Columbia; Manitoba; New Brunswick; Newfoundland and Labrador; Northwest Territories; Nova Scotia; Nunavut; Ontario; Prince Edward Island; Quebec; Saskatchewan; Yukon; offshore east coast west of 44°W and north of 40°N.</v>
+      </c>
+      <c r="G206" s="212" t="str">
+        <v>Canada - onshore - Alberta; British Columbia; Manitoba; New Brunswick; Newfoundland and Labrador; Northwest Territories; Nova Scotia; Nunavut; Ontario; Prince Edward Island; Quebec; Saskatchewan; Yukon; offshore east coast west of 44°W and north of 40°N.</v>
+      </c>
+      <c r="H206" s="212" t="str">
+        <v>Canada - Northwest Territories; Nunavut; Saskatchewan.</v>
+      </c>
+      <c r="I206" s="212" t="str">
+        <v>Canada - Yukon.</v>
+      </c>
+      <c r="J206" s="212" t="str">
+        <v>Canada - Alberta; British Columbia.</v>
+      </c>
+      <c r="K206" s="212" t="str">
+        <v>United States (USA) - Alaska - Aleutian Islands onshore east of 180°E.</v>
+      </c>
+      <c r="L206" s="212" t="str">
+        <v>United States (USA) - Alaska - Aleutian Islands onshore west of 180°W.</v>
+      </c>
+      <c r="M206" s="219" t="str">
+        <v>World</v>
+      </c>
+      <c r="O206"/>
+    </row>
+    <row r="207" spans="2:15" x14ac:dyDescent="0.35">
+      <c r="B207"/>
+      <c r="C207" s="12" t="str">
+        <v>UsageArea.WestLongitude</v>
+      </c>
+      <c r="D207" s="212" t="str">
+        <v>167.65</v>
+      </c>
+      <c r="E207" s="212" t="str">
+        <v>-168.26</v>
+      </c>
+      <c r="F207" s="212" t="str">
+        <v>-141.01</v>
+      </c>
+      <c r="G207" s="212" t="str">
+        <v>-141.01</v>
+      </c>
+      <c r="H207" s="212" t="str">
+        <v>-136.46</v>
+      </c>
+      <c r="I207" s="212" t="str">
+        <v>-141.01</v>
+      </c>
+      <c r="J207" s="212" t="str">
+        <v>-139.04</v>
+      </c>
+      <c r="K207" s="212" t="str">
+        <v>-178.3</v>
+      </c>
+      <c r="L207" s="212" t="str">
+        <v>172.42</v>
+      </c>
+      <c r="M207" s="219" t="str">
+        <v>-180</v>
+      </c>
+      <c r="O207"/>
+    </row>
+    <row r="208" spans="2:15" x14ac:dyDescent="0.35">
+      <c r="B208"/>
+      <c r="C208" s="12" t="str">
+        <v>UsageArea.SouthLatitude</v>
+      </c>
+      <c r="D208" s="212" t="str">
+        <v>47.88</v>
+      </c>
+      <c r="E208" s="212" t="str">
+        <v>54.34</v>
+      </c>
+      <c r="F208" s="212" t="str">
+        <v>40</v>
+      </c>
+      <c r="G208" s="212" t="str">
+        <v>40</v>
+      </c>
+      <c r="H208" s="212" t="str">
+        <v>49</v>
+      </c>
+      <c r="I208" s="212" t="str">
+        <v>59.99</v>
+      </c>
+      <c r="J208" s="212" t="str">
+        <v>48.25</v>
+      </c>
+      <c r="K208" s="212" t="str">
+        <v>51.54</v>
+      </c>
+      <c r="L208" s="212" t="str">
+        <v>51.3</v>
+      </c>
+      <c r="M208" s="219" t="str">
+        <v>-90</v>
+      </c>
+      <c r="O208"/>
+    </row>
+    <row r="209" spans="2:15" x14ac:dyDescent="0.35">
+      <c r="B209"/>
+      <c r="C209" s="12" t="str">
+        <v>UsageArea.EastLongitude</v>
+      </c>
+      <c r="D209" s="212" t="str">
+        <v>-129.99</v>
+      </c>
+      <c r="E209" s="212" t="str">
+        <v>-129.99</v>
+      </c>
+      <c r="F209" s="212" t="str">
+        <v>-44</v>
+      </c>
+      <c r="G209" s="212" t="str">
+        <v>-44</v>
+      </c>
+      <c r="H209" s="212" t="str">
+        <v>-60.72</v>
+      </c>
+      <c r="I209" s="212" t="str">
+        <v>-123.91</v>
+      </c>
+      <c r="J209" s="212" t="str">
+        <v>-109.98</v>
+      </c>
+      <c r="K209" s="212" t="str">
+        <v>-164.84</v>
+      </c>
+      <c r="L209" s="212" t="str">
+        <v>179.86</v>
+      </c>
+      <c r="M209" s="219" t="str">
+        <v>180</v>
+      </c>
+      <c r="O209"/>
+    </row>
+    <row r="210" spans="2:15" x14ac:dyDescent="0.35">
+      <c r="B210"/>
+      <c r="C210" s="12" t="str">
+        <v>UsageArea.NorthLatitude</v>
+      </c>
+      <c r="D210" s="212" t="str">
+        <v>74.71</v>
+      </c>
+      <c r="E210" s="212" t="str">
+        <v>71.4</v>
+      </c>
+      <c r="F210" s="212" t="str">
+        <v>83.17</v>
+      </c>
+      <c r="G210" s="212" t="str">
+        <v>83.17</v>
+      </c>
+      <c r="H210" s="212" t="str">
+        <v>83.17</v>
+      </c>
+      <c r="I210" s="212" t="str">
+        <v>69.7</v>
+      </c>
+      <c r="J210" s="212" t="str">
+        <v>60.01</v>
+      </c>
+      <c r="K210" s="212" t="str">
+        <v>54.34</v>
+      </c>
+      <c r="L210" s="212" t="str">
+        <v>53.07</v>
+      </c>
+      <c r="M210" s="219" t="str">
+        <v>90</v>
+      </c>
+      <c r="O210"/>
+    </row>
+    <row r="211" spans="2:15" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B211"/>
+      <c r="C211" s="13" t="str">
+        <v>UsageArea.Center</v>
+      </c>
+      <c r="D211" s="213" t="str">
+        <v>X=-1588108.78400993, Y=4653218.0046065</v>
+      </c>
+      <c r="E211" s="213" t="str">
+        <v>X=997429.291647658, Y=4946549.42959731</v>
+      </c>
+      <c r="F211" s="213" t="str">
+        <v>X=10065812.5662102, Y=7108107.30892012</v>
+      </c>
+      <c r="G211" s="213" t="str">
+        <v>X=10065812.5662102, Y=7108107.30892012</v>
+      </c>
+      <c r="H211" s="213" t="str">
+        <v>X=8492926.6648403, Y=7635942.58187141</v>
+      </c>
+      <c r="I211" s="213" t="str">
+        <v>X=3484722.01098932, Y=5966394.92755121</v>
+      </c>
+      <c r="J211" s="213" t="str">
+        <v>X=6396219.97160481, Y=2999807.81964541</v>
+      </c>
+      <c r="K211" s="213" t="str">
+        <v>X=-3872417.46753571, Y=1638056.1329905</v>
+      </c>
+      <c r="L211" s="213" t="str">
+        <v>X=-6512034.35982648, Y=2293627.08879407</v>
+      </c>
+      <c r="M211" s="220" t="str">
+        <v>X=30428.2699143998, Y=12753882.6489658</v>
+      </c>
+      <c r="O211"/>
+    </row>
+    <row r="212" spans="2:15" x14ac:dyDescent="0.35">
+      <c r="B212"/>
+      <c r="M212"/>
+      <c r="O212"/>
+    </row>
+    <row r="213" spans="2:15" x14ac:dyDescent="0.35">
+      <c r="B213"/>
+      <c r="M213"/>
+      <c r="O213"/>
+    </row>
+    <row r="214" spans="2:15" x14ac:dyDescent="0.35">
+      <c r="B214"/>
+      <c r="M214"/>
+      <c r="O214"/>
+    </row>
+    <row r="215" spans="2:15" x14ac:dyDescent="0.35">
+      <c r="B215"/>
+      <c r="M215"/>
+      <c r="O215"/>
+    </row>
+    <row r="216" spans="2:15" x14ac:dyDescent="0.35">
+      <c r="B216"/>
+      <c r="M216"/>
+      <c r="O216"/>
+    </row>
+    <row r="217" spans="2:15" x14ac:dyDescent="0.35">
+      <c r="B217"/>
+      <c r="M217"/>
+      <c r="O217"/>
+    </row>
+    <row r="218" spans="2:15" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B218"/>
+      <c r="M218"/>
+      <c r="O218"/>
+    </row>
+    <row r="219" spans="2:15" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B219"/>
+      <c r="C219" s="182" t="str" cm="1">
+        <f t="array" ref="C219:G221">_xll.PE.xfm.ListTransformPipelines($D$4,$D$5)</f>
+        <v>PipelineID</v>
+      </c>
+      <c r="D219" s="183" t="str">
+        <v>Name</v>
+      </c>
+      <c r="E219" s="183" t="str">
+        <v>Accuracy(m)</v>
+      </c>
+      <c r="F219" s="183" t="str">
+        <v>Grids</v>
+      </c>
+      <c r="G219" s="184" t="str">
+        <v>IsAvailable</v>
+      </c>
+      <c r="J219" t="s">
         <v>0</v>
       </c>
-      <c r="M131"/>
-    </row>
-    <row r="132" spans="3:13" x14ac:dyDescent="0.35">
-      <c r="C132" t="s">
-        <v>138</v>
-      </c>
-      <c r="D132" s="172" t="str" cm="1">
-        <f t="array" ref="D132">_xll.PE.crs.AsJsonString(D4)</f>
-        <v>{
-  "$schema": "https://proj.org/schemas/v0.7/projjson.schema.json",
-  "type": "ProjectedCRS",
-  "name": "Albanian 1987 / Gauss-Kruger zone 4 (with axis order normalized for visualization)",
-  "base_crs": {
-    "name": "Albanian 1987",
-    "datum": {
-      "type": "GeodeticReferenceFrame",
-      "name": "Albanian 1987",
-      "ellipsoid": {
-        "name": "Krassowsky 1940",
-        "semi_major_axis": 6378245,
-        "inverse_flattening": 298.3
-      }
-    },
-    "coordinate_system": {
-      "subtype": "ellipsoidal",
-      "axis": [
-        {
-          "name": "Geodetic latitude",
-          "abbreviation": "Lat",
-          "direction": "north",
-          "unit": "degree"
-        },
-        {
-          "name": "Geodetic longitude",
-          "abbreviation": "Lon",
-          "direction": "east",
-          "unit": "degree"
-        }
-      ]
-    },
-    "id": {
-      "authority": "EPSG",
-      "code": 4191
-    }
-  },
-  "conversion": {
-    "name": "6-degree Gauss-Kruger zone 4",
-    "method": {
-      "name": "Transverse Mercator",
-      "id": {
-        "authority": "EPSG",
-        "code": 9807
-      }
-    },
-    "parameters": [
-      {
-        "name": "Latitude of natural origin",
-        "value": 0,
-        "unit": "degree",
-        "id": {
-          "authority": "EPSG",
-          "code": 8801
-        }
-      },
-      {
-        "name": "Longitude of natural origin",
-        "value": 21,
-        "unit": "degree",
-        "id": {
-          "authority": "EPSG",
-          "code": 8802
-        }
-      },
-      {
-        "name": "Scale factor at natural origin",
-        "value": 1,
-        "unit": "unity",
-        "id": {
-          "authority": "EPSG",
-          "code": 8805
-        }
-      },
-      {
-        "name": "False easting",
-        "value": 4500000,
-        "unit": "metre",
-        "id": {
-          "authority": "EPSG",
-          "code": 8806
-        }
-      },
-      {
-        "name": "False northing",
-        "value": 0,
-        "unit": "metre",
-        "id": {
-          "authority": "EPSG",
-          "code": 8807
-        }
-      }
-    ],
-    "id": {
-      "authority": "EPSG",
-      "code": 16204
-    }
-  },
-  "coordinate_system": {
-    "subtype": "Cartesian",
-    "axis": [
-      {
-        "name": "Easting",
-        "abbreviation": "Y",
-        "direction": "east",
-        "unit": "metre"
-      },
-      {
-        "name": "Northing",
-        "abbreviation": "X",
-        "direction": "north",
-        "unit": "metre"
-      }
-    ]
-  },
-  "scope": "Cadastre, engineering survey, topographic mapping.",
-  "area": "Albania - onshore.",
-  "bbox": {
-    "south_latitude": 39.64,
-    "west_longitude": 19.22,
-    "north_latitude": 42.67,
-    "east_longitude": 21.06
-  },
-  "remarks": "Axis order reversed compared to EPSG:2462"
-}</v>
-      </c>
-      <c r="M132"/>
-    </row>
-    <row r="133" spans="3:13" x14ac:dyDescent="0.35">
-      <c r="D133" s="172" t="str" cm="1">
-        <f t="array" ref="D133">_xll.PE.crs.AsProjString(D4)</f>
-        <v>+proj=tmerc +lat_0=0 +lon_0=21 +k=1 +x_0=4500000 +y_0=0 +ellps=krass +units=m +no_defs +type=crs</v>
-      </c>
-      <c r="M133"/>
-    </row>
-    <row r="134" spans="3:13" x14ac:dyDescent="0.35">
-      <c r="D134" s="172" t="str" cm="1">
-        <f t="array" ref="D134">_xll.PE.crs.AsWktString(D4)</f>
-        <v>PROJCRS["Albanian 1987 / Gauss-Kruger zone 4 (with axis order normalized for visualization)",
-    BASEGEOGCRS["Albanian 1987",
-        DATUM["Albanian 1987",
-            ELLIPSOID["Krassowsky 1940",6378245,298.3,
-                LENGTHUNIT["metre",1]]],
-        PRIMEM["Greenwich",0,
-            ANGLEUNIT["degree",0.0174532925199433]],
-        ID["EPSG",4191]],
-    CONVERSION["6-degree Gauss-Kruger zone 4",
-        METHOD["Transverse Mercator",
-            ID["EPSG",9807]],
-        PARAMETER["Latitude of natural origin",0,
-            ANGLEUNIT["degree",0.0174532925199433],
-            ID["EPSG",8801]],
-        PARAMETER["Longitude of natural origin",21,
-            ANGLEUNIT["degree",0.0174532925199433],
-            ID["EPSG",8802]],
-        PARAMETER["Scale factor at natural origin",1,
-            SCALEUNIT["unity",1],
-            ID["EPSG",8805]],
-        PARAMETER["False easting",4500000,
-            LENGTHUNIT["metre",1],
-            ID["EPSG",8806]],
-        PARAMETER["False northing",0,
-            LENGTHUNIT["metre",1],
-            ID["EPSG",8807]],
-        ID["EPSG",16204]],
-    CS[Cartesian,2],
-        AXIS["easting (Y)",east,
-            ORDER[1],
-            LENGTHUNIT["metre",1,
-                ID["EPSG",9001]]],
-        AXIS["northing (X)",north,
-            ORDER[2],
-            LENGTHUNIT["metre",1,
-                ID["EPSG",9001]]],
-    USAGE[
-        SCOPE["Cadastre, engineering survey, topographic mapping."],
-        AREA["Albania - onshore."],
-        BBOX[39.64,19.22,42.67,21.06]],
-    REMARK["Axis order reversed compared to EPSG:2462"]]</v>
-      </c>
-      <c r="M134"/>
-    </row>
-    <row r="135" spans="3:13" x14ac:dyDescent="0.35">
-      <c r="D135" s="174" t="str" cm="1">
-        <f t="array" ref="D135">_xll.PE.crs.Axis.Abbreviation(D4,0,TRUE)</f>
-        <v>Y</v>
-      </c>
-      <c r="M135"/>
-    </row>
-    <row r="136" spans="3:13" x14ac:dyDescent="0.35">
-      <c r="D136" s="174" cm="1">
-        <f t="array" ref="D136">_xll.PE.crs.Axis.Count(D4,TRUE)</f>
+      <c r="K219" s="61"/>
+      <c r="M219"/>
+      <c r="O219"/>
+    </row>
+    <row r="220" spans="2:15" x14ac:dyDescent="0.35">
+      <c r="B220"/>
+      <c r="C220" s="198">
+        <v>1</v>
+      </c>
+      <c r="D220" t="str">
+        <v>Inverse of 6-degree Gauss-Kruger zone 4</v>
+      </c>
+      <c r="E220" t="str">
+        <v/>
+      </c>
+      <c r="F220" t="str">
+        <v/>
+      </c>
+      <c r="G220" s="199" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="K220" s="61"/>
+      <c r="M220"/>
+      <c r="O220"/>
+    </row>
+    <row r="221" spans="2:15" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B221"/>
+      <c r="C221" s="200">
         <v>2</v>
       </c>
-      <c r="M136"/>
-    </row>
-    <row r="137" spans="3:13" x14ac:dyDescent="0.35">
-      <c r="M137"/>
-    </row>
-    <row r="139" spans="3:13" x14ac:dyDescent="0.35">
-      <c r="M139"/>
-    </row>
-    <row r="140" spans="3:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="M140"/>
-    </row>
-    <row r="141" spans="3:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="C141" s="182" t="str" cm="1">
-        <f t="array" ref="C141:G143">_xll.PE.xfm.ListTransformPipelines($D$4,$D$5)</f>
-        <v>PipelineID</v>
-      </c>
-      <c r="D141" s="183" t="str">
+      <c r="D221" s="201" t="str">
+        <v>Albanian 1987 to WGS 84 (1)</v>
+      </c>
+      <c r="E221" s="201">
+        <v>1</v>
+      </c>
+      <c r="F221" s="201" t="str">
+        <v/>
+      </c>
+      <c r="G221" s="202" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="K221" s="61"/>
+      <c r="M221"/>
+      <c r="O221"/>
+    </row>
+    <row r="222" spans="2:15" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B222"/>
+      <c r="K222" s="61"/>
+      <c r="M222"/>
+      <c r="O222"/>
+    </row>
+    <row r="223" spans="2:15" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="C223" s="182" t="str" cm="1">
+        <f t="array" ref="C223:L226">_xll.PE.trf.ListTransformOptions($D$4,$D$5)</f>
+        <v>CandidateIndex</v>
+      </c>
+      <c r="D223" s="183" t="str">
+        <v>DefaultSelection</v>
+      </c>
+      <c r="E223" s="183" t="str">
         <v>Name</v>
       </c>
-      <c r="E141" s="183" t="str">
-        <v>Accuracy(m)</v>
-      </c>
-      <c r="F141" s="183" t="str">
-        <v>Grids</v>
-      </c>
-      <c r="G141" s="184" t="str">
+      <c r="F223" s="183" t="str">
+        <v>Type</v>
+      </c>
+      <c r="G223" s="183" t="str">
+        <v>Accuracy</v>
+      </c>
+      <c r="H223" s="183" t="str">
         <v>IsAvailable</v>
       </c>
-      <c r="J141" t="s">
+      <c r="I223" s="183" t="str">
+        <v>HasBallPark</v>
+      </c>
+      <c r="J223" s="183" t="str">
+        <v>UsageArea</v>
+      </c>
+      <c r="K223" s="203" t="str">
+        <v>Pros</v>
+      </c>
+      <c r="L223" s="184" t="str">
+        <v>Cons</v>
+      </c>
+      <c r="M223"/>
+      <c r="O223"/>
+    </row>
+    <row r="224" spans="2:15" x14ac:dyDescent="0.35">
+      <c r="C224" s="198">
         <v>0</v>
       </c>
-      <c r="K141" s="61"/>
-      <c r="M141"/>
-    </row>
-    <row r="142" spans="3:13" x14ac:dyDescent="0.35">
-      <c r="C142" s="199">
+      <c r="D224" t="str">
+        <v>Only</v>
+      </c>
+      <c r="E224" t="str">
+        <v>Albanian 1987 to WGS 84 (1)</v>
+      </c>
+      <c r="F224" t="str">
+        <v>Transformation</v>
+      </c>
+      <c r="G224">
         <v>1</v>
       </c>
-      <c r="D142" t="str">
+      <c r="H224" t="b">
+        <v>1</v>
+      </c>
+      <c r="I224" t="b">
+        <v>0</v>
+      </c>
+      <c r="J224" t="str">
+        <v>Albania - onshore.</v>
+      </c>
+      <c r="K224" s="61" t="str">
+        <v>Available; Non-ballpark; Accuracy=1; Has usage area; Default selection</v>
+      </c>
+      <c r="L224" s="199" t="str">
+        <v/>
+      </c>
+      <c r="M224"/>
+      <c r="O224"/>
+    </row>
+    <row r="225" spans="3:15" x14ac:dyDescent="0.35">
+      <c r="C225" s="198">
+        <v>1</v>
+      </c>
+      <c r="D225" t="str">
+        <v>Only</v>
+      </c>
+      <c r="E225" t="str">
         <v>Inverse of 6-degree Gauss-Kruger zone 4</v>
       </c>
-      <c r="E142" t="str">
+      <c r="F225" t="str">
+        <v>Conversion</v>
+      </c>
+      <c r="G225">
+        <v>0</v>
+      </c>
+      <c r="H225" t="b">
+        <v>1</v>
+      </c>
+      <c r="I225" t="b">
+        <v>0</v>
+      </c>
+      <c r="J225" t="str">
+        <v>Between 18°E and 24°E.</v>
+      </c>
+      <c r="K225" s="61" t="str">
+        <v>Available; Non-ballpark; Has usage area; Default selection</v>
+      </c>
+      <c r="L225" s="199" t="str">
+        <v>No reported accuracy</v>
+      </c>
+      <c r="M225"/>
+      <c r="O225"/>
+    </row>
+    <row r="226" spans="3:15" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="C226" s="200">
+        <v>2</v>
+      </c>
+      <c r="D226" s="201" t="str">
+        <v>Only</v>
+      </c>
+      <c r="E226" s="201" t="str">
+        <v>axis order change (2D)</v>
+      </c>
+      <c r="F226" s="201" t="str">
+        <v>Conversion</v>
+      </c>
+      <c r="G226" s="201">
+        <v>0</v>
+      </c>
+      <c r="H226" s="201" t="b">
+        <v>1</v>
+      </c>
+      <c r="I226" s="201" t="b">
+        <v>0</v>
+      </c>
+      <c r="J226" s="201" t="str">
         <v/>
       </c>
-      <c r="F142" t="str">
-        <v/>
-      </c>
-      <c r="G142" s="200" t="str">
-        <v>TRUE</v>
-      </c>
-      <c r="K142" s="61"/>
-      <c r="M142"/>
-    </row>
-    <row r="143" spans="3:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="C143" s="201">
-        <v>2</v>
-      </c>
-      <c r="D143" s="202" t="str">
-        <v>Albanian 1987 to WGS 84 (1)</v>
-      </c>
-      <c r="E143" s="202">
-        <v>1</v>
-      </c>
-      <c r="F143" s="202" t="str">
-        <v/>
-      </c>
-      <c r="G143" s="203" t="str">
-        <v>TRUE</v>
-      </c>
-      <c r="K143" s="61"/>
-      <c r="M143"/>
-    </row>
-    <row r="144" spans="3:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="K144" s="61"/>
-      <c r="M144"/>
-    </row>
-    <row r="145" spans="3:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="C145" s="182" t="str" cm="1">
-        <f t="array" ref="C145:L148">_xll.PE.trf.ListTransformOptions($D$4,$D$5)</f>
-        <v>CandidateIndex</v>
-      </c>
-      <c r="D145" s="183" t="str">
-        <v>DefaultSelection</v>
-      </c>
-      <c r="E145" s="183" t="str">
-        <v>Name</v>
-      </c>
-      <c r="F145" s="183" t="str">
-        <v>Type</v>
-      </c>
-      <c r="G145" s="183" t="str">
-        <v>Accuracy</v>
-      </c>
-      <c r="H145" s="183" t="str">
-        <v>IsAvailable</v>
-      </c>
-      <c r="I145" s="183" t="str">
-        <v>HasBallPark</v>
-      </c>
-      <c r="J145" s="183" t="str">
-        <v>UsageArea</v>
-      </c>
-      <c r="K145" s="204" t="str">
-        <v>Pros</v>
-      </c>
-      <c r="L145" s="184" t="str">
-        <v>Cons</v>
-      </c>
-      <c r="M145"/>
-    </row>
-    <row r="146" spans="3:13" x14ac:dyDescent="0.35">
-      <c r="C146" s="199">
-        <v>0</v>
-      </c>
-      <c r="D146" t="str">
-        <v>Only</v>
-      </c>
-      <c r="E146" t="str">
-        <v>Albanian 1987 to WGS 84 (1)</v>
-      </c>
-      <c r="F146" t="str">
-        <v>Transformation</v>
-      </c>
-      <c r="G146">
-        <v>1</v>
-      </c>
-      <c r="H146" t="b">
-        <v>1</v>
-      </c>
-      <c r="I146" t="b">
-        <v>0</v>
-      </c>
-      <c r="J146" t="str">
-        <v>Albania - onshore.</v>
-      </c>
-      <c r="K146" s="61" t="str">
-        <v>Available; Non-ballpark; Accuracy=1; Has usage area; Default selection</v>
-      </c>
-      <c r="L146" s="200" t="str">
-        <v/>
-      </c>
-      <c r="M146"/>
-    </row>
-    <row r="147" spans="3:13" x14ac:dyDescent="0.35">
-      <c r="C147" s="199">
-        <v>1</v>
-      </c>
-      <c r="D147" t="str">
-        <v>Only</v>
-      </c>
-      <c r="E147" t="str">
-        <v>Inverse of 6-degree Gauss-Kruger zone 4</v>
-      </c>
-      <c r="F147" t="str">
-        <v>Conversion</v>
-      </c>
-      <c r="G147">
-        <v>0</v>
-      </c>
-      <c r="H147" t="b">
-        <v>1</v>
-      </c>
-      <c r="I147" t="b">
-        <v>0</v>
-      </c>
-      <c r="J147" t="str">
-        <v>Between 18°E and 24°E.</v>
-      </c>
-      <c r="K147" s="61" t="str">
-        <v>Available; Non-ballpark; Has usage area; Default selection</v>
-      </c>
-      <c r="L147" s="200" t="str">
+      <c r="K226" s="204" t="str">
+        <v>Available; Non-ballpark; Default selection</v>
+      </c>
+      <c r="L226" s="202" t="str">
         <v>No reported accuracy</v>
       </c>
-      <c r="M147"/>
-    </row>
-    <row r="148" spans="3:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="C148" s="201">
-        <v>2</v>
-      </c>
-      <c r="D148" s="202" t="str">
-        <v>Only</v>
-      </c>
-      <c r="E148" s="202" t="str">
-        <v>axis order change (2D)</v>
-      </c>
-      <c r="F148" s="202" t="str">
-        <v>Conversion</v>
-      </c>
-      <c r="G148" s="202">
-        <v>0</v>
-      </c>
-      <c r="H148" s="202" t="b">
-        <v>1</v>
-      </c>
-      <c r="I148" s="202" t="b">
-        <v>0</v>
-      </c>
-      <c r="J148" s="202" t="str">
-        <v/>
-      </c>
-      <c r="K148" s="205" t="str">
-        <v>Available; Non-ballpark; Default selection</v>
-      </c>
-      <c r="L148" s="203" t="str">
-        <v>No reported accuracy</v>
-      </c>
-      <c r="M148"/>
-    </row>
-    <row r="149" spans="3:13" x14ac:dyDescent="0.35">
-      <c r="K149" s="61"/>
-      <c r="M149"/>
-    </row>
-    <row r="150" spans="3:13" x14ac:dyDescent="0.35">
-      <c r="K150" s="61"/>
-      <c r="M150"/>
-    </row>
-    <row r="151" spans="3:13" x14ac:dyDescent="0.35">
-      <c r="C151">
-        <v>2462</v>
-      </c>
-      <c r="K151" s="61"/>
-      <c r="M151"/>
-    </row>
-    <row r="152" spans="3:13" x14ac:dyDescent="0.35">
-      <c r="C152" s="217">
-        <v>4326</v>
-      </c>
-      <c r="D152" t="s">
-        <v>142</v>
-      </c>
-      <c r="K152" s="61"/>
-      <c r="M152"/>
-    </row>
-    <row r="153" spans="3:13" x14ac:dyDescent="0.35">
-      <c r="C153" s="217">
-        <v>3857</v>
-      </c>
-      <c r="D153" t="s">
-        <v>143</v>
-      </c>
-      <c r="K153" s="61"/>
-      <c r="M153"/>
-    </row>
-    <row r="154" spans="3:13" x14ac:dyDescent="0.35">
-      <c r="K154" s="61"/>
-      <c r="M154"/>
-    </row>
-    <row r="155" spans="3:13" x14ac:dyDescent="0.35">
-      <c r="M155"/>
-    </row>
-    <row r="156" spans="3:13" x14ac:dyDescent="0.35">
-      <c r="C156" s="172" t="str" cm="1">
-        <f t="array" ref="C156:D246">_xll.PE.trf.ListTransformInfo(C151,C152)</f>
-        <v>SourceCrs</v>
-      </c>
-      <c r="D156" t="str">
-        <v>2462</v>
-      </c>
-      <c r="M156"/>
-    </row>
-    <row r="157" spans="3:13" x14ac:dyDescent="0.35">
-      <c r="C157" s="172" t="str">
-        <v>DestinationCrs</v>
-      </c>
-      <c r="D157" t="str">
-        <v>4326</v>
-      </c>
-      <c r="M157"/>
-    </row>
-    <row r="158" spans="3:13" x14ac:dyDescent="0.35">
-      <c r="C158" s="172" t="str">
-        <v>Transform.Name</v>
-      </c>
-      <c r="D158" t="str">
-        <v>Inverse of 6-degree Gauss-Kruger zone 4 + Albanian 1987 to WGS 84 (1) + axis order change (2D)</v>
-      </c>
-      <c r="M158"/>
-    </row>
-    <row r="159" spans="3:13" x14ac:dyDescent="0.35">
-      <c r="C159" s="172" t="str">
-        <v>Transform.Type</v>
-      </c>
-      <c r="D159" t="str">
-        <v>ConcatenatedOperation</v>
-      </c>
-      <c r="M159"/>
-    </row>
-    <row r="160" spans="3:13" x14ac:dyDescent="0.35">
-      <c r="C160" s="172" t="str">
-        <v>Transform.Identifier</v>
-      </c>
-      <c r="D160" t="str">
-        <v/>
-      </c>
-      <c r="M160"/>
-    </row>
-    <row r="161" spans="3:13" x14ac:dyDescent="0.35">
-      <c r="C161" s="172" t="str">
-        <v>Transform.Identifiers</v>
-      </c>
-      <c r="D161" t="str">
-        <v/>
-      </c>
-      <c r="M161"/>
-    </row>
-    <row r="162" spans="3:13" x14ac:dyDescent="0.35">
-      <c r="C162" s="172" t="str">
-        <v>Transform.Accuracy</v>
-      </c>
-      <c r="D162" t="str">
-        <v>1</v>
-      </c>
-      <c r="M162"/>
-    </row>
-    <row r="163" spans="3:13" x14ac:dyDescent="0.35">
-      <c r="C163" s="172" t="str">
-        <v>Transform.Count</v>
-      </c>
-      <c r="D163" t="str">
-        <v>3</v>
-      </c>
-      <c r="M163"/>
-    </row>
-    <row r="164" spans="3:13" x14ac:dyDescent="0.35">
-      <c r="C164" s="172" t="str">
-        <v>Transform.IsAvailable</v>
-      </c>
-      <c r="D164" t="str">
-        <v>True</v>
-      </c>
-      <c r="M164"/>
-    </row>
-    <row r="165" spans="3:13" x14ac:dyDescent="0.35">
-      <c r="C165" s="172" t="str">
-        <v>Transform.HasBallParkTransformation</v>
-      </c>
-      <c r="D165" t="str">
-        <v>False</v>
-      </c>
-      <c r="M165"/>
-    </row>
-    <row r="166" spans="3:13" x14ac:dyDescent="0.35">
-      <c r="C166" s="172" t="str">
-        <v>Transform.HasInverse</v>
-      </c>
-      <c r="D166" t="str">
-        <v>True</v>
-      </c>
-      <c r="M166"/>
-    </row>
-    <row r="167" spans="3:13" x14ac:dyDescent="0.35">
-      <c r="C167" s="172" t="str">
-        <v>Transform.MethodName</v>
-      </c>
-      <c r="D167" t="str">
-        <v/>
-      </c>
-      <c r="M167"/>
-    </row>
-    <row r="168" spans="3:13" x14ac:dyDescent="0.35">
-      <c r="C168" s="172" t="str">
-        <v>Transform.Scope</v>
-      </c>
-      <c r="D168" t="str">
-        <v/>
-      </c>
-      <c r="M168"/>
-    </row>
-    <row r="169" spans="3:13" x14ac:dyDescent="0.35">
-      <c r="C169" s="172" t="str">
-        <v>Transform.Remarks</v>
-      </c>
-      <c r="D169" t="str">
-        <v/>
-      </c>
-      <c r="M169"/>
-    </row>
-    <row r="170" spans="3:13" x14ac:dyDescent="0.35">
-      <c r="C170" s="172" t="str">
-        <v>Transform.GridUsages</v>
-      </c>
-      <c r="D170" t="str">
-        <v/>
-      </c>
-      <c r="M170"/>
-    </row>
-    <row r="171" spans="3:13" x14ac:dyDescent="0.35">
-      <c r="C171" s="172" t="str">
-        <v>Transform.Parameters</v>
-      </c>
-      <c r="D171" t="str">
-        <v/>
-      </c>
-      <c r="M171"/>
-    </row>
-    <row r="172" spans="3:13" x14ac:dyDescent="0.35">
-      <c r="C172" s="172" t="str">
-        <v>Transform.SourceCRS</v>
-      </c>
-      <c r="D172" t="str">
-        <v>Albanian 1987 / Gauss-Kruger zone 4 (with axis order normalized for visualization)</v>
-      </c>
-      <c r="M172"/>
-    </row>
-    <row r="173" spans="3:13" x14ac:dyDescent="0.35">
-      <c r="C173" s="172" t="str">
-        <v>Transform.TargetCRS</v>
-      </c>
-      <c r="D173" t="str">
-        <v>WGS 84 (with axis order normalized for visualization)</v>
-      </c>
-      <c r="M173"/>
-    </row>
-    <row r="174" spans="3:13" x14ac:dyDescent="0.35">
-      <c r="C174" s="172" t="str">
-        <v>Transform.Context</v>
-      </c>
-      <c r="D174" t="str">
-        <v>LogLevel=Error; EndpointUrl=https://cdn.proj.org; EnableNetworkConnections=True</v>
-      </c>
-      <c r="M174"/>
-    </row>
-    <row r="175" spans="3:13" x14ac:dyDescent="0.35">
-      <c r="C175" s="172" t="str">
-        <v>Transform.UsageArea</v>
-      </c>
-      <c r="D175" t="str">
-        <v>SharpProj.Proj.UsageArea</v>
-      </c>
-      <c r="M175"/>
-    </row>
-    <row r="176" spans="3:13" x14ac:dyDescent="0.35">
-      <c r="C176" s="172" t="str">
-        <v>Transform.UsageArea.Name</v>
-      </c>
-      <c r="D176" t="str">
-        <v>Albania - onshore.</v>
-      </c>
-      <c r="M176"/>
-    </row>
-    <row r="177" spans="3:13" x14ac:dyDescent="0.35">
-      <c r="C177" s="172" t="str">
-        <v>Transform.UsageArea.WestLongitude</v>
-      </c>
-      <c r="D177" t="str">
-        <v>19.22</v>
-      </c>
-      <c r="M177"/>
-    </row>
-    <row r="178" spans="3:13" x14ac:dyDescent="0.35">
-      <c r="C178" s="172" t="str">
-        <v>Transform.UsageArea.SouthLatitude</v>
-      </c>
-      <c r="D178" t="str">
-        <v>39.64</v>
-      </c>
-      <c r="M178"/>
-    </row>
-    <row r="179" spans="3:13" x14ac:dyDescent="0.35">
-      <c r="C179" s="172" t="str">
-        <v>Transform.UsageArea.EastLongitude</v>
-      </c>
-      <c r="D179" t="str">
-        <v>21.06</v>
-      </c>
-      <c r="M179"/>
-    </row>
-    <row r="180" spans="3:13" x14ac:dyDescent="0.35">
-      <c r="C180" s="172" t="str">
-        <v>Transform.UsageArea.NorthLatitude</v>
-      </c>
-      <c r="D180" t="str">
-        <v>42.67</v>
-      </c>
-      <c r="M180"/>
-    </row>
-    <row r="181" spans="3:13" x14ac:dyDescent="0.35">
-      <c r="C181" s="172" t="str">
-        <v>Transform.UsageArea.Center</v>
-      </c>
-      <c r="D181" t="str">
-        <v>X=4426173.53255827, Y=4558658.03284345</v>
-      </c>
-      <c r="M181"/>
-    </row>
-    <row r="182" spans="3:13" x14ac:dyDescent="0.35">
-      <c r="C182" s="172" t="str">
-        <v>Transform.EnumerableCount</v>
-      </c>
-      <c r="D182" t="str">
-        <v>3</v>
-      </c>
-      <c r="M182"/>
-    </row>
-    <row r="183" spans="3:13" x14ac:dyDescent="0.35">
-      <c r="C183" s="172" t="str">
-        <v>Transform.EnumerableItems</v>
-      </c>
-      <c r="D183" t="str">
-        <v>Inverse of 6-degree Gauss-Kruger zone 4 | Albanian 1987 to WGS 84 (1) | axis order change (2D)</v>
-      </c>
-      <c r="H183" s="173" t="str" cm="1">
-        <f t="array" ref="H183:K206">_xll.PE.trf.TransformList(C151,C152)</f>
-        <v>TransformNo.</v>
-      </c>
-      <c r="I183" s="219">
-        <v>0</v>
-      </c>
-      <c r="J183" s="219">
-        <v>1</v>
-      </c>
-      <c r="K183" s="219">
-        <v>2</v>
-      </c>
-      <c r="M183"/>
-    </row>
-    <row r="184" spans="3:13" x14ac:dyDescent="0.35">
-      <c r="C184" s="206" t="str">
-        <v>Candidate[0].Name</v>
-      </c>
-      <c r="D184" t="str">
-        <v>Albanian 1987 to WGS 84 (1)</v>
-      </c>
-      <c r="H184" s="173" t="str">
-        <v>Name</v>
-      </c>
-      <c r="I184" s="218" t="str">
-        <v>Inverse of 6-degree Gauss-Kruger zone 4</v>
-      </c>
-      <c r="J184" s="218" t="str">
-        <v>Albanian 1987 to WGS 84 (1)</v>
-      </c>
-      <c r="K184" s="218" t="str">
-        <v>axis order change (2D)</v>
-      </c>
-      <c r="M184"/>
-    </row>
-    <row r="185" spans="3:13" x14ac:dyDescent="0.35">
-      <c r="C185" s="206" t="str">
-        <v>Candidate[0].Type</v>
-      </c>
-      <c r="D185" t="str">
-        <v>Transformation</v>
-      </c>
-      <c r="H185" s="173" t="str">
-        <v>Type</v>
-      </c>
-      <c r="I185" s="218" t="str">
-        <v>Conversion</v>
-      </c>
-      <c r="J185" s="218" t="str">
-        <v>Transformation</v>
-      </c>
-      <c r="K185" s="218" t="str">
-        <v>Conversion</v>
-      </c>
-      <c r="M185"/>
-    </row>
-    <row r="186" spans="3:13" x14ac:dyDescent="0.35">
-      <c r="C186" s="206" t="str">
-        <v>Candidate[0].Identifier</v>
-      </c>
-      <c r="D186" t="str">
-        <v>DERIVED_FROM(EPSG):7834</v>
-      </c>
-      <c r="H186" s="173" t="str">
-        <v>Identifier</v>
-      </c>
-      <c r="I186" s="218" t="str">
-        <v>INVERSE(EPSG):16204</v>
-      </c>
-      <c r="J186" s="218" t="str">
-        <v>DERIVED_FROM(EPSG):7834</v>
-      </c>
-      <c r="K186" s="218" t="str">
-        <v>EPSG:15498</v>
-      </c>
-      <c r="M186"/>
-    </row>
-    <row r="187" spans="3:13" x14ac:dyDescent="0.35">
-      <c r="C187" s="206" t="str">
-        <v>Candidate[0].Identifiers</v>
-      </c>
-      <c r="D187" t="str">
-        <v>DERIVED_FROM(EPSG):7834</v>
-      </c>
-      <c r="H187" s="173" t="str">
-        <v>Identifiers</v>
-      </c>
-      <c r="I187" s="218" t="str">
-        <v>&lt;null&gt;</v>
-      </c>
-      <c r="J187" s="218" t="str">
-        <v>&lt;null&gt;</v>
-      </c>
-      <c r="K187" s="218" t="str">
-        <v>&lt;null&gt;</v>
-      </c>
-      <c r="M187"/>
-    </row>
-    <row r="188" spans="3:13" x14ac:dyDescent="0.35">
-      <c r="C188" s="206" t="str">
-        <v>Candidate[0].Accuracy</v>
-      </c>
-      <c r="D188" t="str">
-        <v>1</v>
-      </c>
-      <c r="H188" s="173" t="str">
-        <v>Accuracy</v>
-      </c>
-      <c r="I188" s="218" t="str">
-        <v>&lt;null&gt;</v>
-      </c>
-      <c r="J188" s="218" t="str">
-        <v>1</v>
-      </c>
-      <c r="K188" s="218" t="str">
-        <v>&lt;null&gt;</v>
-      </c>
-      <c r="M188"/>
-    </row>
-    <row r="189" spans="3:13" x14ac:dyDescent="0.35">
-      <c r="C189" s="206" t="str">
-        <v>Candidate[0].IsAvailable</v>
-      </c>
-      <c r="D189" t="str">
-        <v>True</v>
-      </c>
-      <c r="H189" s="173" t="str">
-        <v>IsAvailable</v>
-      </c>
-      <c r="I189" s="218" t="str">
-        <v>True</v>
-      </c>
-      <c r="J189" s="218" t="str">
-        <v>True</v>
-      </c>
-      <c r="K189" s="218" t="str">
-        <v>True</v>
-      </c>
-      <c r="M189"/>
-    </row>
-    <row r="190" spans="3:13" x14ac:dyDescent="0.35">
-      <c r="C190" s="206" t="str">
-        <v>Candidate[0].HasBallParkTransformation</v>
-      </c>
-      <c r="D190" t="str">
-        <v>False</v>
-      </c>
-      <c r="H190" s="173" t="str">
-        <v>HasBallParkTransformation</v>
-      </c>
-      <c r="I190" s="218" t="str">
-        <v>False</v>
-      </c>
-      <c r="J190" s="218" t="str">
-        <v>False</v>
-      </c>
-      <c r="K190" s="218" t="str">
-        <v>False</v>
-      </c>
-      <c r="M190"/>
-    </row>
-    <row r="191" spans="3:13" x14ac:dyDescent="0.35">
-      <c r="C191" s="206" t="str">
-        <v>Candidate[0].HasInverse</v>
-      </c>
-      <c r="D191" t="str">
-        <v>True</v>
-      </c>
-      <c r="H191" s="173" t="str">
-        <v>HasInverse</v>
-      </c>
-      <c r="I191" s="218" t="str">
-        <v>True</v>
-      </c>
-      <c r="J191" s="218" t="str">
-        <v>True</v>
-      </c>
-      <c r="K191" s="218" t="str">
-        <v>True</v>
-      </c>
-      <c r="M191"/>
-    </row>
-    <row r="192" spans="3:13" x14ac:dyDescent="0.35">
-      <c r="C192" s="206" t="str">
-        <v>Candidate[0].MethodName</v>
-      </c>
-      <c r="D192" t="str">
-        <v>Coordinate Frame rotation (geog2D domain)</v>
-      </c>
-      <c r="H192" s="173" t="str">
-        <v>MethodName</v>
-      </c>
-      <c r="I192" s="218" t="str">
-        <v>Inverse of Transverse Mercator</v>
-      </c>
-      <c r="J192" s="218" t="str">
-        <v>Coordinate Frame rotation (geog2D domain)</v>
-      </c>
-      <c r="K192" s="218" t="str">
-        <v>Axis Order Reversal (2D)</v>
-      </c>
-      <c r="M192"/>
-    </row>
-    <row r="193" spans="3:13" x14ac:dyDescent="0.35">
-      <c r="C193" s="206" t="str">
-        <v>Candidate[0].Scope</v>
-      </c>
-      <c r="D193" t="str">
-        <v>(null/copy) Approximation for medium and low accuracy applications assuming equality between plate-fixed static and earth-fixed dynamic CRSs, ignoring static/dynamic CRS differences.</v>
-      </c>
-      <c r="H193" s="173" t="str">
-        <v>Scope</v>
-      </c>
-      <c r="I193" s="218" t="str">
-        <v>Topographic mapping (medium scale).</v>
-      </c>
-      <c r="J193" s="218" t="str">
-        <v>(null/copy) Approximation for medium and low accuracy applications assuming equality between plate-fixed static and earth-fixed dynamic CRSs, ignoring static/dynamic CRS differences.</v>
-      </c>
-      <c r="K193" s="218" t="str">
-        <v>&lt;null&gt;</v>
-      </c>
-      <c r="M193"/>
-    </row>
-    <row r="194" spans="3:13" x14ac:dyDescent="0.35">
-      <c r="C194" s="206" t="str">
-        <v>Candidate[0].Remarks</v>
-      </c>
-      <c r="D194" t="str">
-        <v>Parameter values from Albanian 1987 to ETRS89 (1) (code 7833). Assumes ETRS89 and WGS 84 can be considered the same to within the accuracy of the transformation.</v>
-      </c>
-      <c r="H194" s="173" t="str">
-        <v>Remarks</v>
-      </c>
-      <c r="I194" s="218" t="str">
-        <v>Also found with zone truncated from false easting: see 6-degree Gauss-Kruger CM 21E (code 16304).</v>
-      </c>
-      <c r="J194" s="218" t="str">
-        <v>Parameter values from Albanian 1987 to ETRS89 (1) (code 7833). Assumes ETRS89 and WGS 84 can be considered the same to within the accuracy of the transformation.</v>
-      </c>
-      <c r="K194" s="218" t="str">
-        <v>&lt;null&gt;</v>
-      </c>
-      <c r="M194"/>
-    </row>
-    <row r="195" spans="3:13" x14ac:dyDescent="0.35">
-      <c r="C195" s="206" t="str">
-        <v>Candidate[0].GridUsages</v>
-      </c>
-      <c r="D195" t="str">
-        <v/>
-      </c>
-      <c r="H195" s="173" t="str">
-        <v>GridUsages</v>
-      </c>
-      <c r="I195" s="218" t="str">
-        <v>&lt;null&gt;</v>
-      </c>
-      <c r="J195" s="218" t="str">
-        <v>&lt;null&gt;</v>
-      </c>
-      <c r="K195" s="218" t="str">
-        <v>&lt;null&gt;</v>
-      </c>
-      <c r="M195"/>
-    </row>
-    <row r="196" spans="3:13" x14ac:dyDescent="0.35">
-      <c r="C196" s="206" t="str">
-        <v>Candidate[0].Parameters</v>
-      </c>
-      <c r="D196" t="str">
-        <v>UnitCategory=linear; UnitCode=9001; UnitAuthName=EPSG; UnitName=metre; UnitConversionFactor=1; ValueString=-44.183; UnitCategory=linear; UnitCode=9001; UnitAuthName=EPSG; UnitName=metre; UnitConversionFactor=1; ValueString=-0.58; UnitCategory=linear; UnitCode=9001; UnitAuthName=EPSG; UnitName=metre; UnitConversionFactor=1; ValueString=-38.489; UnitCategory=angular; UnitCode=9104; UnitAuthName=EPSG; UnitName=arc-second; UnitConversionFactor=4.84813681109536E-06; ValueString=-2.3867; UnitCategory=angular; UnitCode=9104; UnitAuthName=EPSG; UnitName=arc-second; UnitConversionFactor=4.84813681109536E-06; ValueString=-2.7072; UnitCategory=angular; UnitCode=9104; UnitAuthName=EPSG; UnitName=arc-second; UnitConversionFactor=4.84813681109536E-06; ValueString=3.5196; UnitCategory=scale; UnitCode=9202; UnitAuthName=EPSG; UnitName=parts per million; UnitConversionFactor=1E-06; ValueString=-8.2703</v>
-      </c>
-      <c r="H196" s="173" t="str">
-        <v>Parameters</v>
-      </c>
-      <c r="I196" s="218" t="str">
-        <v>UnitCategory=angular; UnitCode=9102; UnitAuthName=EPSG; UnitName=degree; UnitConversionFactor=0.0174532925199433; Value=0; UnitCategory=angular; UnitCode=9102; UnitAuthName=EPSG; UnitName=degree; UnitConversionFactor=0.0174532925199433; ValueString=21; UnitCategory=scale; UnitCode=9201; UnitAuthName=EPSG; UnitName=unity; UnitConversionFactor=1; ValueString=1; UnitCategory=linear; UnitCode=9001; UnitAuthName=EPSG; UnitName=metre; UnitConversionFactor=1; ValueString=4500000; UnitCategory=linear; UnitCode=9001; UnitAuthName=EPSG; UnitName=metre; UnitConversionFactor=1; Value=0</v>
-      </c>
-      <c r="J196" s="218" t="str">
-        <v>UnitCategory=linear; UnitCode=9001; UnitAuthName=EPSG; UnitName=metre; UnitConversionFactor=1; ValueString=-44.183; UnitCategory=linear; UnitCode=9001; UnitAuthName=EPSG; UnitName=metre; UnitConversionFactor=1; ValueString=-0.58; UnitCategory=linear; UnitCode=9001; UnitAuthName=EPSG; UnitName=metre; UnitConversionFactor=1; ValueString=-38.489; UnitCategory=angular; UnitCode=9104; UnitAuthName=EPSG; UnitName=arc-second; UnitConversionFactor=4.84813681109536E-06; ValueString=-2.3867; UnitCategory=angular; UnitCode=9104; UnitAuthName=EPSG; UnitName=arc-second; UnitConversionFactor=4.84813681109536E-06; ValueString=-2.7072; UnitCategory=angular; UnitCode=9104; UnitAuthName=EPSG; UnitName=arc-second; UnitConversionFactor=4.84813681109536E-06; ValueString=3.5196; UnitCategory=scale; UnitCode=9202; UnitAuthName=EPSG; UnitName=parts per million; UnitConversionFactor=1E-06; ValueString=-8.2703</v>
-      </c>
-      <c r="K196" s="218" t="str">
-        <v>&lt;null&gt;</v>
-      </c>
-      <c r="M196"/>
-    </row>
-    <row r="197" spans="3:13" x14ac:dyDescent="0.35">
-      <c r="C197" s="206" t="str">
-        <v>Candidate[0].SourceCRS</v>
-      </c>
-      <c r="D197" t="str">
-        <v>Albanian 1987</v>
-      </c>
-      <c r="H197" s="173" t="str">
-        <v>SourceCRS</v>
-      </c>
-      <c r="I197" s="218" t="str">
-        <v>Albanian 1987 / Gauss-Kruger zone 4 (with axis order normalized for visualization)</v>
-      </c>
-      <c r="J197" s="218" t="str">
-        <v>Albanian 1987</v>
-      </c>
-      <c r="K197" s="218" t="str">
-        <v>WGS 84</v>
-      </c>
-      <c r="M197"/>
-    </row>
-    <row r="198" spans="3:13" x14ac:dyDescent="0.35">
-      <c r="C198" s="206" t="str">
-        <v>Candidate[0].TargetCRS</v>
-      </c>
-      <c r="D198" t="str">
-        <v>WGS 84</v>
-      </c>
-      <c r="H198" s="173" t="str">
-        <v>TargetCRS</v>
-      </c>
-      <c r="I198" s="218" t="str">
-        <v>Albanian 1987</v>
-      </c>
-      <c r="J198" s="218" t="str">
-        <v>WGS 84</v>
-      </c>
-      <c r="K198" s="218" t="str">
-        <v>WGS 84 (with axis order normalized for visualization)</v>
-      </c>
-      <c r="M198"/>
-    </row>
-    <row r="199" spans="3:13" x14ac:dyDescent="0.35">
-      <c r="C199" s="206" t="str">
-        <v>Candidate[0].Context</v>
-      </c>
-      <c r="D199" t="str">
-        <v>LogLevel=Error; EndpointUrl=https://cdn.proj.org; EnableNetworkConnections=True</v>
-      </c>
-      <c r="H199" s="173" t="str">
-        <v>Context</v>
-      </c>
-      <c r="I199" s="218" t="str">
-        <v>LogLevel=Error; EndpointUrl=https://cdn.proj.org; EnableNetworkConnections=True</v>
-      </c>
-      <c r="J199" s="218" t="str">
-        <v>LogLevel=Error; EndpointUrl=https://cdn.proj.org; EnableNetworkConnections=True</v>
-      </c>
-      <c r="K199" s="218" t="str">
-        <v>LogLevel=Error; EndpointUrl=https://cdn.proj.org; EnableNetworkConnections=True</v>
-      </c>
-      <c r="M199"/>
-    </row>
-    <row r="200" spans="3:13" x14ac:dyDescent="0.35">
-      <c r="C200" s="206" t="str">
-        <v>Candidate[0].UsageArea</v>
-      </c>
-      <c r="D200" t="str">
-        <v>SharpProj.Proj.UsageArea</v>
-      </c>
-      <c r="H200" s="173" t="str">
-        <v>UsageArea</v>
-      </c>
-      <c r="I200" s="218" t="str">
-        <v>UsageArea</v>
-      </c>
-      <c r="J200" s="218" t="str">
-        <v>UsageArea</v>
-      </c>
-      <c r="K200" s="218" t="str">
-        <v>&lt;null&gt;</v>
-      </c>
-      <c r="M200"/>
-    </row>
-    <row r="201" spans="3:13" x14ac:dyDescent="0.35">
-      <c r="C201" s="206" t="str">
-        <v>Candidate[0].UsageArea.Name</v>
-      </c>
-      <c r="D201" t="str">
-        <v>Albania - onshore.</v>
-      </c>
-      <c r="H201" s="173" t="str">
-        <v>UsageArea.Name</v>
-      </c>
-      <c r="I201" s="218" t="str">
-        <v>Between 18°E and 24°E.</v>
-      </c>
-      <c r="J201" s="218" t="str">
-        <v>Albania - onshore.</v>
-      </c>
-      <c r="K201" s="218" t="str">
-        <v>&lt;null&gt;</v>
-      </c>
-      <c r="M201"/>
-    </row>
-    <row r="202" spans="3:13" x14ac:dyDescent="0.35">
-      <c r="C202" s="206" t="str">
-        <v>Candidate[0].UsageArea.WestLongitude</v>
-      </c>
-      <c r="D202" t="str">
-        <v>19.22</v>
-      </c>
-      <c r="H202" s="173" t="str">
-        <v>UsageArea.WestLongitude</v>
-      </c>
-      <c r="I202" s="218" t="str">
-        <v>18</v>
-      </c>
-      <c r="J202" s="218" t="str">
-        <v>19.22</v>
-      </c>
-      <c r="K202" s="218" t="str">
-        <v>&lt;null&gt;</v>
-      </c>
-      <c r="M202"/>
-    </row>
-    <row r="203" spans="3:13" x14ac:dyDescent="0.35">
-      <c r="C203" s="206" t="str">
-        <v>Candidate[0].UsageArea.SouthLatitude</v>
-      </c>
-      <c r="D203" t="str">
-        <v>39.64</v>
-      </c>
-      <c r="H203" s="173" t="str">
-        <v>UsageArea.SouthLatitude</v>
-      </c>
-      <c r="I203" s="218" t="str">
-        <v>-80</v>
-      </c>
-      <c r="J203" s="218" t="str">
-        <v>39.64</v>
-      </c>
-      <c r="K203" s="218" t="str">
-        <v>&lt;null&gt;</v>
-      </c>
-      <c r="M203"/>
-    </row>
-    <row r="204" spans="3:13" x14ac:dyDescent="0.35">
-      <c r="C204" s="206" t="str">
-        <v>Candidate[0].UsageArea.EastLongitude</v>
-      </c>
-      <c r="D204" t="str">
-        <v>21.06</v>
-      </c>
-      <c r="H204" s="173" t="str">
-        <v>UsageArea.EastLongitude</v>
-      </c>
-      <c r="I204" s="218" t="str">
-        <v>24</v>
-      </c>
-      <c r="J204" s="218" t="str">
-        <v>21.06</v>
-      </c>
-      <c r="K204" s="218" t="str">
-        <v>&lt;null&gt;</v>
-      </c>
-      <c r="M204"/>
-    </row>
-    <row r="205" spans="3:13" x14ac:dyDescent="0.35">
-      <c r="C205" s="206" t="str">
-        <v>Candidate[0].UsageArea.NorthLatitude</v>
-      </c>
-      <c r="D205" t="str">
-        <v>42.67</v>
-      </c>
-      <c r="H205" s="173" t="str">
-        <v>UsageArea.NorthLatitude</v>
-      </c>
-      <c r="I205" s="218" t="str">
-        <v>84</v>
-      </c>
-      <c r="J205" s="218" t="str">
-        <v>42.67</v>
-      </c>
-      <c r="K205" s="218" t="str">
-        <v>&lt;null&gt;</v>
-      </c>
-      <c r="M205"/>
-    </row>
-    <row r="206" spans="3:13" x14ac:dyDescent="0.35">
-      <c r="C206" s="206" t="str">
-        <v>Candidate[0].UsageArea.Center</v>
-      </c>
-      <c r="D206" t="str">
-        <v>X=41.155, Y=20.14</v>
-      </c>
-      <c r="H206" s="173" t="str">
-        <v>UsageArea.Center</v>
-      </c>
-      <c r="I206" s="218" t="str">
-        <v>X=4500000, Y=223053.008659147</v>
-      </c>
-      <c r="J206" s="218" t="str">
-        <v>X=41.155, Y=20.14</v>
-      </c>
-      <c r="K206" s="218" t="str">
-        <v>&lt;null&gt;</v>
-      </c>
-      <c r="M206"/>
-    </row>
-    <row r="207" spans="3:13" x14ac:dyDescent="0.35">
-      <c r="C207" s="172" t="str">
-        <v>Candidate[1].Name</v>
-      </c>
-      <c r="D207" t="str">
-        <v>Inverse of 6-degree Gauss-Kruger zone 4</v>
-      </c>
-      <c r="M207"/>
-    </row>
-    <row r="208" spans="3:13" x14ac:dyDescent="0.35">
-      <c r="C208" s="172" t="str">
-        <v>Candidate[1].Type</v>
-      </c>
-      <c r="D208" t="str">
-        <v>Conversion</v>
-      </c>
-      <c r="M208"/>
-    </row>
-    <row r="209" spans="3:13" x14ac:dyDescent="0.35">
-      <c r="C209" s="172" t="str">
-        <v>Candidate[1].Identifier</v>
-      </c>
-      <c r="D209" t="str">
-        <v>INVERSE(EPSG):16204</v>
-      </c>
-      <c r="M209"/>
-    </row>
-    <row r="210" spans="3:13" x14ac:dyDescent="0.35">
-      <c r="C210" s="172" t="str">
-        <v>Candidate[1].Identifiers</v>
-      </c>
-      <c r="D210" t="str">
-        <v>INVERSE(EPSG):16204</v>
-      </c>
-      <c r="M210"/>
-    </row>
-    <row r="211" spans="3:13" x14ac:dyDescent="0.35">
-      <c r="C211" s="172" t="str">
-        <v>Candidate[1].Accuracy</v>
-      </c>
-      <c r="D211" t="str">
-        <v/>
-      </c>
-      <c r="M211"/>
-    </row>
-    <row r="212" spans="3:13" x14ac:dyDescent="0.35">
-      <c r="C212" s="172" t="str">
-        <v>Candidate[1].IsAvailable</v>
-      </c>
-      <c r="D212" t="str">
-        <v>True</v>
-      </c>
-      <c r="M212"/>
-    </row>
-    <row r="213" spans="3:13" x14ac:dyDescent="0.35">
-      <c r="C213" s="172" t="str">
-        <v>Candidate[1].HasBallParkTransformation</v>
-      </c>
-      <c r="D213" t="str">
-        <v>False</v>
-      </c>
-      <c r="M213"/>
-    </row>
-    <row r="214" spans="3:13" x14ac:dyDescent="0.35">
-      <c r="C214" s="172" t="str">
-        <v>Candidate[1].HasInverse</v>
-      </c>
-      <c r="D214" t="str">
-        <v>True</v>
-      </c>
-      <c r="M214"/>
-    </row>
-    <row r="215" spans="3:13" x14ac:dyDescent="0.35">
-      <c r="C215" s="172" t="str">
-        <v>Candidate[1].MethodName</v>
-      </c>
-      <c r="D215" t="str">
-        <v>Inverse of Transverse Mercator</v>
-      </c>
-      <c r="M215"/>
-    </row>
-    <row r="216" spans="3:13" x14ac:dyDescent="0.35">
-      <c r="C216" s="172" t="str">
-        <v>Candidate[1].Scope</v>
-      </c>
-      <c r="D216" t="str">
-        <v>Topographic mapping (medium scale).</v>
-      </c>
-      <c r="M216"/>
-    </row>
-    <row r="217" spans="3:13" x14ac:dyDescent="0.35">
-      <c r="C217" s="172" t="str">
-        <v>Candidate[1].Remarks</v>
-      </c>
-      <c r="D217" t="str">
-        <v>Also found with zone truncated from false easting: see 6-degree Gauss-Kruger CM 21E (code 16304).</v>
-      </c>
-      <c r="M217"/>
-    </row>
-    <row r="218" spans="3:13" x14ac:dyDescent="0.35">
-      <c r="C218" s="172" t="str">
-        <v>Candidate[1].GridUsages</v>
-      </c>
-      <c r="D218" t="str">
-        <v/>
-      </c>
-      <c r="M218"/>
-    </row>
-    <row r="219" spans="3:13" x14ac:dyDescent="0.35">
-      <c r="C219" s="172" t="str">
-        <v>Candidate[1].Parameters</v>
-      </c>
-      <c r="D219" t="str">
-        <v>UnitCategory=angular; UnitCode=9102; UnitAuthName=EPSG; UnitName=degree; UnitConversionFactor=0.0174532925199433; Value=0; UnitCategory=angular; UnitCode=9102; UnitAuthName=EPSG; UnitName=degree; UnitConversionFactor=0.0174532925199433; ValueString=21; UnitCategory=scale; UnitCode=9201; UnitAuthName=EPSG; UnitName=unity; UnitConversionFactor=1; ValueString=1; UnitCategory=linear; UnitCode=9001; UnitAuthName=EPSG; UnitName=metre; UnitConversionFactor=1; ValueString=4500000; UnitCategory=linear; UnitCode=9001; UnitAuthName=EPSG; UnitName=metre; UnitConversionFactor=1; Value=0</v>
-      </c>
-      <c r="M219"/>
-    </row>
-    <row r="220" spans="3:13" x14ac:dyDescent="0.35">
-      <c r="C220" s="172" t="str">
-        <v>Candidate[1].SourceCRS</v>
-      </c>
-      <c r="D220" t="str">
-        <v>Albanian 1987 / Gauss-Kruger zone 4 (with axis order normalized for visualization)</v>
-      </c>
-      <c r="M220"/>
-    </row>
-    <row r="221" spans="3:13" x14ac:dyDescent="0.35">
-      <c r="C221" s="172" t="str">
-        <v>Candidate[1].TargetCRS</v>
-      </c>
-      <c r="D221" t="str">
-        <v>Albanian 1987</v>
-      </c>
-      <c r="M221"/>
-    </row>
-    <row r="222" spans="3:13" x14ac:dyDescent="0.35">
-      <c r="C222" s="172" t="str">
-        <v>Candidate[1].Context</v>
-      </c>
-      <c r="D222" t="str">
-        <v>LogLevel=Error; EndpointUrl=https://cdn.proj.org; EnableNetworkConnections=True</v>
-      </c>
-      <c r="M222"/>
-    </row>
-    <row r="223" spans="3:13" x14ac:dyDescent="0.35">
-      <c r="C223" s="172" t="str">
-        <v>Candidate[1].UsageArea</v>
-      </c>
-      <c r="D223" t="str">
-        <v>SharpProj.Proj.UsageArea</v>
-      </c>
-      <c r="M223"/>
-    </row>
-    <row r="224" spans="3:13" x14ac:dyDescent="0.35">
-      <c r="C224" s="172" t="str">
-        <v>Candidate[1].UsageArea.Name</v>
-      </c>
-      <c r="D224" t="str">
-        <v>Between 18°E and 24°E.</v>
-      </c>
-      <c r="M224"/>
-    </row>
-    <row r="225" spans="3:15" x14ac:dyDescent="0.35">
-      <c r="C225" s="172" t="str">
-        <v>Candidate[1].UsageArea.WestLongitude</v>
-      </c>
-      <c r="D225" t="str">
-        <v>18</v>
-      </c>
-      <c r="M225"/>
-    </row>
-    <row r="226" spans="3:15" x14ac:dyDescent="0.35">
-      <c r="C226" s="172" t="str">
-        <v>Candidate[1].UsageArea.SouthLatitude</v>
-      </c>
-      <c r="D226" t="str">
-        <v>-80</v>
-      </c>
       <c r="M226"/>
+      <c r="O226"/>
     </row>
     <row r="227" spans="3:15" x14ac:dyDescent="0.35">
-      <c r="C227" s="172" t="str">
-        <v>Candidate[1].UsageArea.EastLongitude</v>
-      </c>
-      <c r="D227" t="str">
-        <v>24</v>
-      </c>
       <c r="M227"/>
+      <c r="O227"/>
     </row>
     <row r="228" spans="3:15" x14ac:dyDescent="0.35">
-      <c r="C228" s="172" t="str">
-        <v>Candidate[1].UsageArea.NorthLatitude</v>
-      </c>
-      <c r="D228" t="str">
-        <v>84</v>
-      </c>
       <c r="M228"/>
+      <c r="O228"/>
     </row>
     <row r="229" spans="3:15" x14ac:dyDescent="0.35">
-      <c r="C229" s="172" t="str">
-        <v>Candidate[1].UsageArea.Center</v>
-      </c>
-      <c r="D229" t="str">
-        <v>X=4500000, Y=223053.008659147</v>
-      </c>
       <c r="M229"/>
+      <c r="O229"/>
     </row>
     <row r="230" spans="3:15" x14ac:dyDescent="0.35">
-      <c r="C230" s="206" t="str">
-        <v>Candidate[2].Name</v>
-      </c>
-      <c r="D230" t="str">
-        <v>axis order change (2D)</v>
-      </c>
       <c r="M230"/>
       <c r="O230"/>
     </row>
     <row r="231" spans="3:15" x14ac:dyDescent="0.35">
-      <c r="C231" s="206" t="str">
-        <v>Candidate[2].Type</v>
-      </c>
-      <c r="D231" t="str">
-        <v>Conversion</v>
-      </c>
       <c r="M231"/>
       <c r="O231"/>
     </row>
     <row r="232" spans="3:15" x14ac:dyDescent="0.35">
-      <c r="C232" s="206" t="str">
-        <v>Candidate[2].Identifier</v>
-      </c>
-      <c r="D232" t="str">
-        <v>EPSG:15498</v>
-      </c>
       <c r="M232"/>
       <c r="O232"/>
     </row>
     <row r="233" spans="3:15" x14ac:dyDescent="0.35">
-      <c r="C233" s="206" t="str">
-        <v>Candidate[2].Identifiers</v>
-      </c>
-      <c r="D233" t="str">
-        <v>EPSG:15498</v>
-      </c>
       <c r="M233"/>
       <c r="O233"/>
     </row>
     <row r="234" spans="3:15" x14ac:dyDescent="0.35">
-      <c r="C234" s="206" t="str">
-        <v>Candidate[2].Accuracy</v>
-      </c>
-      <c r="D234" t="str">
-        <v/>
-      </c>
       <c r="M234"/>
       <c r="O234"/>
     </row>
     <row r="235" spans="3:15" x14ac:dyDescent="0.35">
-      <c r="C235" s="206" t="str">
-        <v>Candidate[2].IsAvailable</v>
-      </c>
-      <c r="D235" t="str">
-        <v>True</v>
-      </c>
       <c r="M235"/>
       <c r="O235"/>
     </row>
     <row r="236" spans="3:15" x14ac:dyDescent="0.35">
-      <c r="C236" s="206" t="str">
-        <v>Candidate[2].HasBallParkTransformation</v>
-      </c>
-      <c r="D236" t="str">
-        <v>False</v>
-      </c>
       <c r="M236"/>
       <c r="O236"/>
     </row>
     <row r="237" spans="3:15" x14ac:dyDescent="0.35">
-      <c r="C237" s="206" t="str">
-        <v>Candidate[2].HasInverse</v>
-      </c>
-      <c r="D237" t="str">
-        <v>True</v>
-      </c>
       <c r="M237"/>
       <c r="O237"/>
     </row>
     <row r="238" spans="3:15" x14ac:dyDescent="0.35">
-      <c r="C238" s="206" t="str">
-        <v>Candidate[2].MethodName</v>
-      </c>
-      <c r="D238" t="str">
-        <v>Axis Order Reversal (2D)</v>
-      </c>
       <c r="M238"/>
       <c r="O238"/>
     </row>
     <row r="239" spans="3:15" x14ac:dyDescent="0.35">
-      <c r="C239" s="206" t="str">
-        <v>Candidate[2].Scope</v>
-      </c>
-      <c r="D239" t="str">
-        <v/>
-      </c>
       <c r="M239"/>
       <c r="O239"/>
     </row>
     <row r="240" spans="3:15" x14ac:dyDescent="0.35">
-      <c r="C240" s="206" t="str">
-        <v>Candidate[2].Remarks</v>
-      </c>
-      <c r="D240" t="str">
-        <v/>
-      </c>
       <c r="M240"/>
       <c r="O240"/>
     </row>
-    <row r="241" spans="3:15" x14ac:dyDescent="0.35">
-      <c r="C241" s="206" t="str">
-        <v>Candidate[2].GridUsages</v>
-      </c>
-      <c r="D241" t="str">
-        <v/>
-      </c>
+    <row r="241" spans="13:15" x14ac:dyDescent="0.35">
       <c r="M241"/>
       <c r="O241"/>
     </row>
-    <row r="242" spans="3:15" x14ac:dyDescent="0.35">
-      <c r="C242" s="206" t="str">
-        <v>Candidate[2].Parameters</v>
-      </c>
-      <c r="D242" t="str">
-        <v/>
-      </c>
+    <row r="242" spans="13:15" x14ac:dyDescent="0.35">
       <c r="M242"/>
       <c r="O242"/>
     </row>
-    <row r="243" spans="3:15" x14ac:dyDescent="0.35">
-      <c r="C243" s="206" t="str">
-        <v>Candidate[2].SourceCRS</v>
-      </c>
-      <c r="D243" t="str">
-        <v>WGS 84</v>
-      </c>
+    <row r="243" spans="13:15" x14ac:dyDescent="0.35">
       <c r="M243"/>
       <c r="O243"/>
     </row>
-    <row r="244" spans="3:15" x14ac:dyDescent="0.35">
-      <c r="C244" s="206" t="str">
-        <v>Candidate[2].TargetCRS</v>
-      </c>
-      <c r="D244" t="str">
-        <v>WGS 84 (with axis order normalized for visualization)</v>
-      </c>
+    <row r="244" spans="13:15" x14ac:dyDescent="0.35">
       <c r="M244"/>
       <c r="O244"/>
     </row>
-    <row r="245" spans="3:15" x14ac:dyDescent="0.35">
-      <c r="C245" s="206" t="str">
-        <v>Candidate[2].Context</v>
-      </c>
-      <c r="D245" t="str">
-        <v>LogLevel=Error; EndpointUrl=https://cdn.proj.org; EnableNetworkConnections=True</v>
-      </c>
+    <row r="245" spans="13:15" x14ac:dyDescent="0.35">
       <c r="M245"/>
       <c r="O245"/>
     </row>
-    <row r="246" spans="3:15" x14ac:dyDescent="0.35">
-      <c r="C246" s="206" t="str">
-        <v>Candidate[2].UsageArea</v>
-      </c>
-      <c r="D246" t="str">
-        <v/>
-      </c>
+    <row r="246" spans="13:15" x14ac:dyDescent="0.35">
       <c r="M246"/>
       <c r="O246"/>
     </row>
-    <row r="247" spans="3:15" x14ac:dyDescent="0.35">
+    <row r="247" spans="13:15" x14ac:dyDescent="0.35">
       <c r="M247"/>
       <c r="O247"/>
     </row>
-    <row r="248" spans="3:15" x14ac:dyDescent="0.35">
+    <row r="248" spans="13:15" x14ac:dyDescent="0.35">
       <c r="M248"/>
       <c r="O248"/>
     </row>
-    <row r="249" spans="3:15" x14ac:dyDescent="0.35">
+    <row r="249" spans="13:15" x14ac:dyDescent="0.35">
       <c r="M249"/>
       <c r="O249"/>
     </row>
-    <row r="250" spans="3:15" x14ac:dyDescent="0.35">
+    <row r="250" spans="13:15" x14ac:dyDescent="0.35">
       <c r="M250"/>
       <c r="O250"/>
     </row>
-    <row r="251" spans="3:15" x14ac:dyDescent="0.35">
+    <row r="251" spans="13:15" x14ac:dyDescent="0.35">
       <c r="M251"/>
       <c r="O251"/>
     </row>
-    <row r="252" spans="3:15" x14ac:dyDescent="0.35">
+    <row r="252" spans="13:15" x14ac:dyDescent="0.35">
       <c r="M252"/>
       <c r="O252"/>
     </row>
-    <row r="253" spans="3:15" x14ac:dyDescent="0.35">
+    <row r="253" spans="13:15" x14ac:dyDescent="0.35">
       <c r="M253"/>
       <c r="O253"/>
     </row>
-    <row r="254" spans="3:15" x14ac:dyDescent="0.35">
+    <row r="254" spans="13:15" x14ac:dyDescent="0.35">
       <c r="M254"/>
       <c r="O254"/>
     </row>
-    <row r="255" spans="3:15" x14ac:dyDescent="0.35">
+    <row r="255" spans="13:15" x14ac:dyDescent="0.35">
       <c r="M255"/>
       <c r="O255"/>
     </row>
-    <row r="256" spans="3:15" x14ac:dyDescent="0.35">
+    <row r="256" spans="13:15" x14ac:dyDescent="0.35">
       <c r="M256"/>
       <c r="O256"/>
     </row>
@@ -47835,106 +48287,6 @@
     <row r="286" spans="13:15" x14ac:dyDescent="0.35">
       <c r="M286"/>
       <c r="O286"/>
-    </row>
-    <row r="287" spans="13:15" x14ac:dyDescent="0.35">
-      <c r="M287"/>
-      <c r="O287"/>
-    </row>
-    <row r="288" spans="13:15" x14ac:dyDescent="0.35">
-      <c r="M288"/>
-      <c r="O288"/>
-    </row>
-    <row r="289" spans="13:15" x14ac:dyDescent="0.35">
-      <c r="M289"/>
-      <c r="O289"/>
-    </row>
-    <row r="290" spans="13:15" x14ac:dyDescent="0.35">
-      <c r="M290"/>
-      <c r="O290"/>
-    </row>
-    <row r="291" spans="13:15" x14ac:dyDescent="0.35">
-      <c r="M291"/>
-      <c r="O291"/>
-    </row>
-    <row r="292" spans="13:15" x14ac:dyDescent="0.35">
-      <c r="M292"/>
-      <c r="O292"/>
-    </row>
-    <row r="293" spans="13:15" x14ac:dyDescent="0.35">
-      <c r="M293"/>
-      <c r="O293"/>
-    </row>
-    <row r="294" spans="13:15" x14ac:dyDescent="0.35">
-      <c r="M294"/>
-      <c r="O294"/>
-    </row>
-    <row r="295" spans="13:15" x14ac:dyDescent="0.35">
-      <c r="M295"/>
-      <c r="O295"/>
-    </row>
-    <row r="296" spans="13:15" x14ac:dyDescent="0.35">
-      <c r="M296"/>
-      <c r="O296"/>
-    </row>
-    <row r="297" spans="13:15" x14ac:dyDescent="0.35">
-      <c r="M297"/>
-      <c r="O297"/>
-    </row>
-    <row r="298" spans="13:15" x14ac:dyDescent="0.35">
-      <c r="M298"/>
-      <c r="O298"/>
-    </row>
-    <row r="299" spans="13:15" x14ac:dyDescent="0.35">
-      <c r="M299"/>
-      <c r="O299"/>
-    </row>
-    <row r="300" spans="13:15" x14ac:dyDescent="0.35">
-      <c r="M300"/>
-      <c r="O300"/>
-    </row>
-    <row r="301" spans="13:15" x14ac:dyDescent="0.35">
-      <c r="M301"/>
-      <c r="O301"/>
-    </row>
-    <row r="302" spans="13:15" x14ac:dyDescent="0.35">
-      <c r="M302"/>
-      <c r="O302"/>
-    </row>
-    <row r="303" spans="13:15" x14ac:dyDescent="0.35">
-      <c r="M303"/>
-      <c r="O303"/>
-    </row>
-    <row r="304" spans="13:15" x14ac:dyDescent="0.35">
-      <c r="M304"/>
-      <c r="O304"/>
-    </row>
-    <row r="305" spans="13:15" x14ac:dyDescent="0.35">
-      <c r="M305"/>
-      <c r="O305"/>
-    </row>
-    <row r="306" spans="13:15" x14ac:dyDescent="0.35">
-      <c r="M306"/>
-      <c r="O306"/>
-    </row>
-    <row r="307" spans="13:15" x14ac:dyDescent="0.35">
-      <c r="M307"/>
-      <c r="O307"/>
-    </row>
-    <row r="308" spans="13:15" x14ac:dyDescent="0.35">
-      <c r="M308"/>
-      <c r="O308"/>
-    </row>
-    <row r="309" spans="13:15" x14ac:dyDescent="0.35">
-      <c r="M309"/>
-      <c r="O309"/>
-    </row>
-    <row r="310" spans="13:15" x14ac:dyDescent="0.35">
-      <c r="M310"/>
-      <c r="O310"/>
-    </row>
-    <row r="311" spans="13:15" x14ac:dyDescent="0.35">
-      <c r="M311"/>
-      <c r="O311"/>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>

<commit_message>
Normalized all transforms to have consistent list/steps output
</commit_message>
<xml_diff>
--- a/DegreeTests.xlsx
+++ b/DegreeTests.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Source\VS22\ProjExcel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{766B9A21-4C8C-4160-A61A-707E5903CDEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{733D7FDF-17D6-48A4-847D-39428E023CDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38290" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1214,7 +1214,7 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="13" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="267">
+  <cellXfs count="257">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1795,33 +1795,17 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="15" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="0" fillId="15" borderId="9" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="15" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="15" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="13" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="17" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Comma" xfId="3" builtinId="3"/>
@@ -46965,14 +46949,18 @@
     </row>
     <row r="198" spans="3:20" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C198" s="251" t="str" cm="1">
-        <f t="array" ref="C198:D212">_xll.PE.trf.TransformSteps(D171,D172,C173,"proj")</f>
+        <f t="array" ref="C198:F212">_xll.PE.trf.TransformSteps(D171,D172,C173,"proj")</f>
         <v>Step Number</v>
       </c>
       <c r="D198" s="4">
         <v>0</v>
       </c>
-      <c r="E198" s="215"/>
-      <c r="F198" s="215"/>
+      <c r="E198" s="215">
+        <v>1</v>
+      </c>
+      <c r="F198" s="215">
+        <v>2</v>
+      </c>
       <c r="G198" s="215"/>
       <c r="H198" s="215"/>
       <c r="I198" s="5"/>
@@ -46998,11 +46986,15 @@
       <c r="C199" s="235" t="str">
         <v>Step Identifiers</v>
       </c>
-      <c r="D199" s="178">
-        <v>0</v>
-      </c>
-      <c r="E199" s="172"/>
-      <c r="F199" s="172"/>
+      <c r="D199" s="178" t="str">
+        <v>INVERSE(EPSG)</v>
+      </c>
+      <c r="E199" s="172" t="str">
+        <v>INVERSE(EPSG)</v>
+      </c>
+      <c r="F199" s="172" t="str">
+        <v>EPSG</v>
+      </c>
       <c r="G199" s="172"/>
       <c r="H199" s="172"/>
       <c r="I199" s="179"/>
@@ -47028,10 +47020,14 @@
         <v>Step Name</v>
       </c>
       <c r="D200" s="178" t="str">
-        <v>&lt;choose-coordinate-transform&gt;</v>
-      </c>
-      <c r="E200" s="172"/>
-      <c r="F200" s="172"/>
+        <v>Inverse of Popular Visualisation Pseudo-Mercator</v>
+      </c>
+      <c r="E200" s="172" t="str">
+        <v>Inverse of ED50 to WGS 84 (18)</v>
+      </c>
+      <c r="F200" s="172" t="str">
+        <v>TM 5 NE</v>
+      </c>
       <c r="G200" s="172"/>
       <c r="H200" s="172"/>
       <c r="I200" s="179"/>
@@ -47059,8 +47055,12 @@
       <c r="D201" s="178">
         <v>55</v>
       </c>
-      <c r="E201" s="172"/>
-      <c r="F201" s="172"/>
+      <c r="E201" s="172">
+        <v>55</v>
+      </c>
+      <c r="F201" s="172">
+        <v>55</v>
+      </c>
       <c r="G201" s="172"/>
       <c r="H201" s="172"/>
       <c r="I201" s="179"/>
@@ -47086,10 +47086,14 @@
         <v>UsageArea</v>
       </c>
       <c r="D202" s="178" t="str">
+        <v>World.</v>
+      </c>
+      <c r="E202" s="172" t="str">
         <v>Denmark - offshore North Sea; Ireland - offshore; Netherlands - offshore; United Kingdom - UKCS offshore.</v>
       </c>
-      <c r="E202" s="172"/>
-      <c r="F202" s="172"/>
+      <c r="F202" s="172" t="str">
+        <v>Netherlands - offshore North Sea.</v>
+      </c>
       <c r="G202" s="172"/>
       <c r="H202" s="172"/>
       <c r="I202" s="179"/>
@@ -47115,10 +47119,14 @@
         <v>Scope</v>
       </c>
       <c r="D203" s="178" t="str">
-        <v>Unknown</v>
-      </c>
-      <c r="E203" s="172"/>
-      <c r="F203" s="172"/>
+        <v>Web mapping and visualisation.</v>
+      </c>
+      <c r="E203" s="172" t="str">
+        <v>Oil and gas exploration and production.</v>
+      </c>
+      <c r="F203" s="172" t="str">
+        <v>Oil and gas exploration and production.</v>
+      </c>
       <c r="G203" s="172"/>
       <c r="H203" s="172"/>
       <c r="I203" s="179"/>
@@ -47147,8 +47155,12 @@
       <c r="D204" s="178" t="str">
         <v>None</v>
       </c>
-      <c r="E204" s="172"/>
-      <c r="F204" s="172"/>
+      <c r="E204" s="172" t="str">
+        <v>Recommended CT for UKCS and IrishCS petroleum purposes, known as "Common Offshore". Based on ED50 to WGS 72 (precise ephemeris) 6-nations agreement of 1981 with which precise to broadcast and broadcast to WGS 84 transformations have been concatenated.</v>
+      </c>
+      <c r="F204" s="172" t="str">
+        <v>None</v>
+      </c>
       <c r="G204" s="172"/>
       <c r="H204" s="172"/>
       <c r="I204" s="179"/>
@@ -47175,10 +47187,14 @@
         <v>UsageArea.WestLongitude</v>
       </c>
       <c r="D205" s="178">
+        <v>-180</v>
+      </c>
+      <c r="E205" s="172">
         <v>-16.100000000000001</v>
       </c>
-      <c r="E205" s="172"/>
-      <c r="F205" s="172"/>
+      <c r="F205" s="172">
+        <v>2.5299999999999998</v>
+      </c>
       <c r="G205" s="172"/>
       <c r="H205" s="172"/>
       <c r="I205" s="179"/>
@@ -47188,10 +47204,14 @@
         <v>UsageArea.SouthLatitude</v>
       </c>
       <c r="D206" s="178">
+        <v>180</v>
+      </c>
+      <c r="E206" s="172">
         <v>10.86</v>
       </c>
-      <c r="E206" s="172"/>
-      <c r="F206" s="172"/>
+      <c r="F206" s="172">
+        <v>6.37</v>
+      </c>
       <c r="G206" s="172"/>
       <c r="H206" s="172"/>
       <c r="I206" s="179"/>
@@ -47232,10 +47252,14 @@
         <v>UsageArea.EastLongitude</v>
       </c>
       <c r="D207" s="178">
+        <v>-90</v>
+      </c>
+      <c r="E207" s="172">
         <v>47.42</v>
       </c>
-      <c r="E207" s="172"/>
-      <c r="F207" s="172"/>
+      <c r="F207" s="172">
+        <v>51.44</v>
+      </c>
       <c r="G207" s="172"/>
       <c r="H207" s="172"/>
       <c r="I207" s="179"/>
@@ -47275,10 +47299,14 @@
         <v>UsageArea.NorthLatitude</v>
       </c>
       <c r="D208" s="178">
-        <v>63.89</v>
-      </c>
-      <c r="E208" s="172"/>
-      <c r="F208" s="172"/>
+        <v>0</v>
+      </c>
+      <c r="E208" s="172">
+        <v>0</v>
+      </c>
+      <c r="F208" s="172">
+        <v>0</v>
+      </c>
       <c r="G208" s="172"/>
       <c r="H208" s="172"/>
       <c r="I208" s="179"/>
@@ -47317,11 +47345,15 @@
       <c r="C209" s="235" t="str">
         <v>Nr grids</v>
       </c>
-      <c r="D209" s="178">
-        <v>0</v>
-      </c>
-      <c r="E209" s="172"/>
-      <c r="F209" s="172"/>
+      <c r="D209" s="178" t="str">
+        <v>N.A.</v>
+      </c>
+      <c r="E209" s="172" t="str">
+        <v>N.A.</v>
+      </c>
+      <c r="F209" s="172" t="str">
+        <v>N.A.</v>
+      </c>
       <c r="G209" s="172"/>
       <c r="H209" s="172"/>
       <c r="I209" s="179"/>
@@ -47363,8 +47395,12 @@
       <c r="D210" s="178" t="str">
         <v>N.A.</v>
       </c>
-      <c r="E210" s="172"/>
-      <c r="F210" s="172"/>
+      <c r="E210" s="172" t="str">
+        <v>N.A.</v>
+      </c>
+      <c r="F210" s="172" t="str">
+        <v>N.A.</v>
+      </c>
       <c r="G210" s="172"/>
       <c r="H210" s="172"/>
       <c r="I210" s="179"/>
@@ -47404,10 +47440,14 @@
         <v>2nd grid</v>
       </c>
       <c r="D211" s="178" t="str">
-        <v>N.A.</v>
-      </c>
-      <c r="E211" s="172"/>
-      <c r="F211" s="172"/>
+        <v>+proj=pipeline +step +inv +proj=webmerc +lat_0=0 +lon_0=0 +x_0=0 +y_0=0 +ellps=WGS84 +step +proj=unitconvert +xy_in=rad +xy_out=deg +step +proj=axisswap +order=2,1</v>
+      </c>
+      <c r="E211" s="172" t="str">
+        <v>+proj=pipeline +step +proj=axisswap +order=2,1 +step +proj=unitconvert +xy_in=deg +xy_out=rad +step +proj=push +v_3 +step +proj=cart +ellps=WGS84 +step +inv +proj=helmert +x=-89.5 +y=-93.8 +z=-123.1 +rx=0 +ry=0 +rz=-0.156 +s=1.2 +convention=position_vector +step +inv +proj=cart +ellps=intl +step +proj=pop +v_3 +step +proj=unitconvert +xy_in=rad +xy_out=deg +step +proj=axisswap +order=2,1</v>
+      </c>
+      <c r="F211" s="172" t="str">
+        <v>+proj=pipeline +step +proj=axisswap +order=2,1 +step +proj=unitconvert +xy_in=deg +xy_out=rad +step +proj=tmerc +lat_0=0 +lon_0=5 +k=0.9996 +x_0=500000 +y_0=0 +ellps=intl</v>
+      </c>
       <c r="G211" s="172"/>
       <c r="H211" s="172"/>
       <c r="I211" s="179"/>
@@ -47449,8 +47489,12 @@
       <c r="D212" s="180">
         <v>0</v>
       </c>
-      <c r="E212" s="214"/>
-      <c r="F212" s="214"/>
+      <c r="E212" s="214">
+        <v>0</v>
+      </c>
+      <c r="F212" s="214">
+        <v>0</v>
+      </c>
       <c r="G212" s="214"/>
       <c r="H212" s="214"/>
       <c r="I212" s="181"/>
@@ -47486,15 +47530,7 @@
       </c>
     </row>
     <row r="213" spans="2:20" x14ac:dyDescent="0.35">
-      <c r="L213" s="253"/>
-      <c r="M213" s="253"/>
-      <c r="N213" s="253"/>
-      <c r="O213" s="254"/>
-      <c r="P213" s="253"/>
-      <c r="Q213" s="253"/>
-      <c r="R213" s="253"/>
-      <c r="S213" s="253"/>
-      <c r="T213" s="253"/>
+      <c r="M213"/>
     </row>
     <row r="214" spans="2:20" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="M214"/>
@@ -48385,11 +48421,14 @@
     <row r="242" spans="2:20" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B242"/>
       <c r="C242" s="251" t="str" cm="1">
-        <f t="array" ref="C242:D256">_xll.PE.trf.TransformSteps(D215,D216,C217,"proj")</f>
+        <f t="array" ref="C242:E256">_xll.PE.trf.TransformSteps(D215,D216,C217,"proj")</f>
         <v>Step Number</v>
       </c>
       <c r="D242" s="5">
         <v>0</v>
+      </c>
+      <c r="E242" s="5">
+        <v>1</v>
       </c>
       <c r="F242" t="str">
         <f>D219</f>
@@ -48418,8 +48457,11 @@
       <c r="C243" s="235" t="str">
         <v>Step Identifiers</v>
       </c>
-      <c r="D243" s="179">
-        <v>0</v>
+      <c r="D243" s="179" t="str">
+        <v>INVERSE(EPSG)</v>
+      </c>
+      <c r="E243" s="179" t="str">
+        <v>DERIVED_FROM(EPSG)</v>
       </c>
       <c r="F243" t="str">
         <f>E219</f>
@@ -48448,7 +48490,10 @@
         <v>Step Name</v>
       </c>
       <c r="D244" s="179" t="str">
-        <v>&lt;choose-coordinate-transform&gt;</v>
+        <v>Inverse of Alaska Albers</v>
+      </c>
+      <c r="E244" s="179" t="str">
+        <v>NAD27 to WGS 84 (85)</v>
       </c>
       <c r="F244" t="str">
         <f>F219</f>
@@ -48479,6 +48524,9 @@
       <c r="D245" s="179">
         <v>0</v>
       </c>
+      <c r="E245" s="179">
+        <v>0</v>
+      </c>
       <c r="F245" t="str">
         <f>G219</f>
         <v>Inverse of Alaska Albers + NAD27 to WGS 84 (3) + axis order change (2D)</v>
@@ -48506,6 +48554,9 @@
         <v>UsageArea</v>
       </c>
       <c r="D246" s="179" t="str">
+        <v>United States (USA) - Alaska.</v>
+      </c>
+      <c r="E246" s="179" t="str">
         <v>United States (USA) - Alaska including EEZ.</v>
       </c>
       <c r="F246" t="str">
@@ -48535,7 +48586,10 @@
         <v>Scope</v>
       </c>
       <c r="D247" s="179" t="str">
-        <v>Unknown</v>
+        <v>Topographic mapping (small scale).</v>
+      </c>
+      <c r="E247" s="179" t="str">
+        <v>(null/copy) Approximation for medium and low accuracy applications assuming equality between plate-fixed static and earth-fixed dynamic CRSs, ignoring static/dynamic CRS differences.</v>
       </c>
       <c r="K247" s="198">
         <v>5</v>
@@ -48563,6 +48617,9 @@
       <c r="D248" s="179" t="str">
         <v>None</v>
       </c>
+      <c r="E248" s="179" t="str">
+        <v>Parameter files are from NAD27 to NAD83 (2) (code 1243) assuming that NAD83 is equivalent to WGS 84 within the accuracy of this tfm. Uses NADCON method which expects longitudes positive west; EPSG CRS codes 4267 and 4326 have longitudes positive east.</v>
+      </c>
       <c r="K248" s="198">
         <v>6</v>
       </c>
@@ -48587,6 +48644,9 @@
         <v>UsageArea.WestLongitude</v>
       </c>
       <c r="D249" s="179">
+        <v>172.42</v>
+      </c>
+      <c r="E249" s="179">
         <v>167.65</v>
       </c>
       <c r="K249" s="198">
@@ -48613,6 +48673,9 @@
       <c r="D250" s="179">
         <v>-129.99</v>
       </c>
+      <c r="E250" s="179">
+        <v>-129.99</v>
+      </c>
       <c r="K250" s="198">
         <v>8</v>
       </c>
@@ -48635,6 +48698,9 @@
         <v>UsageArea.EastLongitude</v>
       </c>
       <c r="D251" s="179">
+        <v>51.3</v>
+      </c>
+      <c r="E251" s="179">
         <v>47.88</v>
       </c>
       <c r="K251" s="198">
@@ -48658,7 +48724,10 @@
         <v>UsageArea.NorthLatitude</v>
       </c>
       <c r="D252" s="179">
-        <v>74.709999999999994</v>
+        <v>0</v>
+      </c>
+      <c r="E252" s="179">
+        <v>1</v>
       </c>
       <c r="K252" s="200">
         <v>10</v>
@@ -48680,8 +48749,11 @@
       <c r="C253" s="235" t="str">
         <v>Nr grids</v>
       </c>
-      <c r="D253" s="179">
-        <v>1</v>
+      <c r="D253" s="179" t="str">
+        <v>N.A.</v>
+      </c>
+      <c r="E253" s="179" t="str">
+        <v/>
       </c>
     </row>
     <row r="254" spans="2:20" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -48689,7 +48761,10 @@
         <v>1st grid</v>
       </c>
       <c r="D254" s="179" t="str">
-        <v/>
+        <v>N.A.</v>
+      </c>
+      <c r="E254" s="179" t="str">
+        <v>N.A.</v>
       </c>
       <c r="K254" s="182" t="str" cm="1">
         <f t="array" ref="K254:T264">_xll.PE.trf.ListTransformOptions(D215,D216)</f>
@@ -48728,7 +48803,10 @@
         <v>2nd grid</v>
       </c>
       <c r="D255" s="179" t="str">
-        <v>N.A.</v>
+        <v>+proj=pipeline +step +proj=unitconvert +xy_in=us-ft +xy_out=m +step +inv +proj=aea +lat_0=50 +lon_0=-154 +lat_1=55 +lat_2=65 +x_0=0 +y_0=0 +ellps=clrk66 +step +proj=unitconvert +xy_in=rad +xy_out=deg +step +proj=axisswap +order=2,1</v>
+      </c>
+      <c r="E255" s="179" t="str">
+        <v>+proj=pipeline +step +proj=axisswap +order=2,1 +step +proj=unitconvert +xy_in=deg +xy_out=rad +step +proj=hgridshift +grids=us_noaa_alaska.tif +step +proj=unitconvert +xy_in=rad +xy_out=deg +step +proj=axisswap +order=2,1</v>
       </c>
       <c r="K255" s="244">
         <v>0</v>
@@ -48766,6 +48844,9 @@
         <v>Step ROJ string</v>
       </c>
       <c r="D256" s="181">
+        <v>0</v>
+      </c>
+      <c r="E256" s="181">
         <v>0</v>
       </c>
       <c r="K256" s="198">
@@ -49319,7 +49400,7 @@
     </row>
     <row r="294" spans="3:17" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C294" s="251" t="str" cm="1">
-        <f t="array" ref="C294:E308">_xll.PE.trf.TransformSteps(D267,D268,,"proj")</f>
+        <f t="array" ref="C294:E308">_xll.PE.trf.TransformSteps(D267,D268,C269,"proj")</f>
         <v>Step Number</v>
       </c>
       <c r="D294" s="4">
@@ -49405,10 +49486,10 @@
         <v>Step sccuracy [m]</v>
       </c>
       <c r="D297" s="178">
-        <v>0</v>
+        <v>55</v>
       </c>
       <c r="E297" s="179">
-        <v>0</v>
+        <v>55</v>
       </c>
       <c r="M297"/>
     </row>
@@ -49565,10 +49646,10 @@
         <v>UsageArea.NorthLatitude</v>
       </c>
       <c r="D304" s="178">
-        <v>0</v>
+        <v>84</v>
       </c>
       <c r="E304" s="179">
-        <v>0</v>
+        <v>84</v>
       </c>
       <c r="H304" s="200">
         <v>1</v>
@@ -49605,11 +49686,11 @@
       <c r="C305" s="235" t="str">
         <v>Nr grids</v>
       </c>
-      <c r="D305" s="178" t="str">
-        <v>N.A.</v>
-      </c>
-      <c r="E305" s="179" t="str">
-        <v>N.A.</v>
+      <c r="D305" s="178">
+        <v>0</v>
+      </c>
+      <c r="E305" s="179">
+        <v>0</v>
       </c>
       <c r="M305"/>
       <c r="O305"/>
@@ -49632,23 +49713,23 @@
         <v>2nd grid</v>
       </c>
       <c r="D307" s="178" t="str">
-        <v>+proj=pipeline +step +inv +proj=utm +zone=32 +ellps=GRS80 +step +proj=unitconvert +xy_in=rad +xy_out=deg +step +proj=axisswap +order=2,1</v>
+        <v>N.A.</v>
       </c>
       <c r="E307" s="179" t="str">
-        <v>+proj=pipeline +step +proj=axisswap +order=2,1 +step +proj=unitconvert +xy_in=deg +xy_out=rad +step +proj=utm +zone=33 +ellps=GRS80</v>
+        <v>N.A.</v>
       </c>
       <c r="M307"/>
       <c r="O307"/>
     </row>
     <row r="308" spans="3:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C308" s="236" t="str">
-        <v>Step ROJ string</v>
-      </c>
-      <c r="D308" s="180">
-        <v>0</v>
-      </c>
-      <c r="E308" s="181">
-        <v>0</v>
+        <v>Step PROJ string</v>
+      </c>
+      <c r="D308" s="180" t="str">
+        <v>+proj=pipeline +step +inv +proj=utm +zone=32 +ellps=GRS80 +step +proj=unitconvert +xy_in=rad +xy_out=deg +step +proj=axisswap +order=2,1</v>
+      </c>
+      <c r="E308" s="181" t="str">
+        <v>+proj=pipeline +step +proj=axisswap +order=2,1 +step +proj=unitconvert +xy_in=deg +xy_out=rad +step +proj=utm +zone=33 +ellps=GRS80</v>
       </c>
       <c r="M308"/>
       <c r="O308"/>
@@ -49684,8 +49765,8 @@
     </row>
     <row r="313" spans="3:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C313" s="182" t="str" cm="1">
-        <f t="array" ref="C313">_xll.PE.trf.Options(,,,,,55,,,,,,"Never",,,0,)</f>
-        <v>Authority=EPSG; Area=; Accuracy=55; NoBallparkConversions=False; NoDiscardIfMissing=False; UsePrimaryGridNames=False; UseSuperseded=False; StrictContains=False; IntermediateCrsUsage=Never; BestOnly=False; ForceOver=False; CandidateIndex=0; AllowDeprecatedCrs=False</v>
+        <f t="array" ref="C313">_xll.PE.trf.Options(,,,,,55,,,,,,"Never",,,6,)</f>
+        <v>Authority=EPSG; Area=; Accuracy=55; NoBallparkConversions=False; NoDiscardIfMissing=False; UsePrimaryGridNames=False; UseSuperseded=False; StrictContains=False; IntermediateCrsUsage=Never; BestOnly=False; ForceOver=False; CandidateIndex=6; AllowDeprecatedCrs=False</v>
       </c>
       <c r="D313" s="183"/>
       <c r="E313" s="183"/>
@@ -49702,783 +49783,739 @@
       <c r="P313" s="184"/>
     </row>
     <row r="314" spans="3:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="C314" s="226" t="str" cm="1">
-        <f t="array" ref="C314:M336">_xll.PE.trf.TransformList(D311,D312,,"")</f>
+      <c r="C314" s="223" t="str" cm="1">
+        <f t="array" ref="C314:L336">_xll.PE.trf.TransformList(D311,D312,C313,"")</f>
         <v>Transform Number</v>
       </c>
-      <c r="D314" s="265">
+      <c r="D314" s="4">
         <v>0</v>
       </c>
-      <c r="E314" s="266">
+      <c r="E314" s="215">
         <v>1</v>
       </c>
-      <c r="F314" s="266">
+      <c r="F314" s="215">
         <v>2</v>
       </c>
-      <c r="G314" s="266">
+      <c r="G314" s="215">
         <v>3</v>
       </c>
-      <c r="H314" s="266">
+      <c r="H314" s="215">
         <v>4</v>
       </c>
-      <c r="I314" s="266">
+      <c r="I314" s="215">
         <v>5</v>
       </c>
-      <c r="J314" s="266">
+      <c r="J314" s="215">
         <v>6</v>
       </c>
-      <c r="K314" s="266">
+      <c r="K314" s="215">
         <v>7</v>
       </c>
-      <c r="L314" s="266">
+      <c r="L314" s="5">
         <v>8</v>
       </c>
-      <c r="M314" s="35">
-        <v>9</v>
-      </c>
+      <c r="M314"/>
       <c r="O314"/>
     </row>
     <row r="315" spans="3:16" x14ac:dyDescent="0.35">
       <c r="C315" s="12" t="str">
         <v>Transform Name</v>
       </c>
-      <c r="D315" s="257" t="str">
+      <c r="D315" s="252" t="str">
         <v>Inverse of Alaska Albers + NAD27 to WGS 84 (85) + axis order change (2D)</v>
       </c>
-      <c r="E315" s="252" t="str">
+      <c r="E315" s="256" t="str">
         <v>Inverse of Alaska Albers + NAD27 to WGS 84 (7) + axis order change (2D)</v>
       </c>
-      <c r="F315" s="252" t="str">
+      <c r="F315" s="256" t="str">
         <v>Inverse of Alaska Albers + NAD27 to WGS 84 (33) + axis order change (2D)</v>
       </c>
-      <c r="G315" s="252" t="str">
+      <c r="G315" s="256" t="str">
         <v>Inverse of Alaska Albers + NAD27 to WGS 84 (3) + axis order change (2D)</v>
       </c>
-      <c r="H315" s="252" t="str">
+      <c r="H315" s="256" t="str">
         <v>Inverse of Alaska Albers + NAD27 to WGS 84 (13) + axis order change (2D)</v>
       </c>
-      <c r="I315" s="252" t="str">
+      <c r="I315" s="256" t="str">
         <v>Inverse of Alaska Albers + NAD27 to WGS 84 (14) + axis order change (2D)</v>
       </c>
-      <c r="J315" s="252" t="str">
+      <c r="J315" s="256" t="str">
         <v>Inverse of Alaska Albers + NAD27 to WGS 84 (10) + axis order change (2D)</v>
       </c>
-      <c r="K315" s="252" t="str">
+      <c r="K315" s="256" t="str">
         <v>Inverse of Alaska Albers + NAD27 to WGS 84 (21) + axis order change (2D)</v>
       </c>
-      <c r="L315" s="252" t="str">
+      <c r="L315" s="179" t="str">
         <v>Inverse of Alaska Albers + NAD27 to WGS 84 (22) + axis order change (2D)</v>
       </c>
-      <c r="M315" s="179" t="str">
-        <v>Inverse of Alaska Albers + Ballpark geographic offset from NAD27 to WGS 84 (with axis order normalized for visualization)</v>
-      </c>
+      <c r="M315"/>
       <c r="O315"/>
     </row>
     <row r="316" spans="3:16" x14ac:dyDescent="0.35">
       <c r="C316" s="12" t="str">
         <v>Transform Type</v>
       </c>
-      <c r="D316" s="257" t="str">
+      <c r="D316" s="252" t="str">
         <v>ConcatenatedOperation</v>
       </c>
-      <c r="E316" s="252" t="str">
+      <c r="E316" s="256" t="str">
         <v>ConcatenatedOperation</v>
       </c>
-      <c r="F316" s="252" t="str">
+      <c r="F316" s="256" t="str">
         <v>ConcatenatedOperation</v>
       </c>
-      <c r="G316" s="252" t="str">
+      <c r="G316" s="256" t="str">
         <v>ConcatenatedOperation</v>
       </c>
-      <c r="H316" s="252" t="str">
+      <c r="H316" s="256" t="str">
         <v>ConcatenatedOperation</v>
       </c>
-      <c r="I316" s="252" t="str">
+      <c r="I316" s="256" t="str">
         <v>ConcatenatedOperation</v>
       </c>
-      <c r="J316" s="252" t="str">
+      <c r="J316" s="256" t="str">
         <v>ConcatenatedOperation</v>
       </c>
-      <c r="K316" s="252" t="str">
+      <c r="K316" s="256" t="str">
         <v>ConcatenatedOperation</v>
       </c>
-      <c r="L316" s="252" t="str">
+      <c r="L316" s="179" t="str">
         <v>ConcatenatedOperation</v>
       </c>
-      <c r="M316" s="255" t="str">
-        <v>ConcatenatedOperation</v>
-      </c>
+      <c r="M316"/>
     </row>
     <row r="317" spans="3:16" x14ac:dyDescent="0.35">
       <c r="C317" s="12" t="str">
         <v>Identifier</v>
       </c>
-      <c r="D317" s="257" t="str">
+      <c r="D317" s="252" t="str">
         <v/>
       </c>
-      <c r="E317" s="252" t="str">
+      <c r="E317" s="256" t="str">
         <v/>
       </c>
-      <c r="F317" s="252" t="str">
+      <c r="F317" s="256" t="str">
         <v/>
       </c>
-      <c r="G317" s="252" t="str">
+      <c r="G317" s="256" t="str">
         <v/>
       </c>
-      <c r="H317" s="252" t="str">
+      <c r="H317" s="256" t="str">
         <v/>
       </c>
-      <c r="I317" s="252" t="str">
+      <c r="I317" s="256" t="str">
         <v/>
       </c>
-      <c r="J317" s="252" t="str">
+      <c r="J317" s="256" t="str">
         <v/>
       </c>
-      <c r="K317" s="252" t="str">
+      <c r="K317" s="256" t="str">
         <v/>
       </c>
-      <c r="L317" s="252" t="str">
+      <c r="L317" s="179" t="str">
         <v/>
       </c>
-      <c r="M317" s="255" t="str">
-        <v/>
-      </c>
+      <c r="M317"/>
     </row>
     <row r="318" spans="3:16" x14ac:dyDescent="0.35">
       <c r="C318" s="12" t="str">
         <v>Identifiers</v>
       </c>
-      <c r="D318" s="257" t="str">
+      <c r="D318" s="252" t="str">
         <v/>
       </c>
-      <c r="E318" s="252" t="str">
+      <c r="E318" s="256" t="str">
         <v/>
       </c>
-      <c r="F318" s="252" t="str">
+      <c r="F318" s="256" t="str">
         <v/>
       </c>
-      <c r="G318" s="252" t="str">
+      <c r="G318" s="256" t="str">
         <v/>
       </c>
-      <c r="H318" s="252" t="str">
+      <c r="H318" s="256" t="str">
         <v/>
       </c>
-      <c r="I318" s="252" t="str">
+      <c r="I318" s="256" t="str">
         <v/>
       </c>
-      <c r="J318" s="252" t="str">
+      <c r="J318" s="256" t="str">
         <v/>
       </c>
-      <c r="K318" s="252" t="str">
+      <c r="K318" s="256" t="str">
         <v/>
       </c>
-      <c r="L318" s="252" t="str">
+      <c r="L318" s="179" t="str">
         <v/>
       </c>
-      <c r="M318" s="255" t="str">
-        <v/>
-      </c>
+      <c r="M318"/>
     </row>
     <row r="319" spans="3:16" x14ac:dyDescent="0.35">
       <c r="C319" s="12" t="str">
         <v>Accuracy</v>
       </c>
-      <c r="D319" s="257" t="str">
+      <c r="D319" s="252" t="str">
         <v>5</v>
       </c>
-      <c r="E319" s="252" t="str">
+      <c r="E319" s="256" t="str">
         <v>12</v>
       </c>
-      <c r="F319" s="252" t="str">
+      <c r="F319" s="256" t="str">
         <v>2</v>
       </c>
-      <c r="G319" s="252" t="str">
+      <c r="G319" s="256" t="str">
         <v>20</v>
       </c>
-      <c r="H319" s="252" t="str">
+      <c r="H319" s="256" t="str">
         <v>8</v>
       </c>
-      <c r="I319" s="252" t="str">
+      <c r="I319" s="256" t="str">
         <v>10</v>
       </c>
-      <c r="J319" s="252" t="str">
+      <c r="J319" s="256" t="str">
         <v>13</v>
       </c>
-      <c r="K319" s="252" t="str">
+      <c r="K319" s="256" t="str">
         <v>15</v>
       </c>
-      <c r="L319" s="252" t="str">
+      <c r="L319" s="179" t="str">
         <v>18</v>
       </c>
-      <c r="M319" s="255" t="str">
-        <v/>
-      </c>
+      <c r="M319"/>
     </row>
     <row r="320" spans="3:16" x14ac:dyDescent="0.35">
       <c r="C320" s="12" t="str">
         <v>IsAvailable</v>
       </c>
-      <c r="D320" s="257" t="str">
+      <c r="D320" s="252" t="str">
         <v>True</v>
       </c>
-      <c r="E320" s="252" t="str">
+      <c r="E320" s="256" t="str">
         <v>True</v>
       </c>
-      <c r="F320" s="252" t="str">
+      <c r="F320" s="256" t="str">
         <v>True</v>
       </c>
-      <c r="G320" s="252" t="str">
+      <c r="G320" s="256" t="str">
         <v>True</v>
       </c>
-      <c r="H320" s="252" t="str">
+      <c r="H320" s="256" t="str">
         <v>True</v>
       </c>
-      <c r="I320" s="252" t="str">
+      <c r="I320" s="256" t="str">
         <v>True</v>
       </c>
-      <c r="J320" s="252" t="str">
+      <c r="J320" s="256" t="str">
         <v>True</v>
       </c>
-      <c r="K320" s="252" t="str">
+      <c r="K320" s="256" t="str">
         <v>True</v>
       </c>
-      <c r="L320" s="252" t="str">
+      <c r="L320" s="179" t="str">
         <v>True</v>
       </c>
-      <c r="M320" s="255" t="str">
-        <v>True</v>
-      </c>
+      <c r="M320"/>
     </row>
     <row r="321" spans="3:13" x14ac:dyDescent="0.35">
       <c r="C321" s="12" t="str">
         <v>HasBallParkTransformation</v>
       </c>
-      <c r="D321" s="257" t="str">
+      <c r="D321" s="252" t="str">
         <v>False</v>
       </c>
-      <c r="E321" s="252" t="str">
+      <c r="E321" s="256" t="str">
         <v>False</v>
       </c>
-      <c r="F321" s="252" t="str">
+      <c r="F321" s="256" t="str">
         <v>False</v>
       </c>
-      <c r="G321" s="252" t="str">
+      <c r="G321" s="256" t="str">
         <v>False</v>
       </c>
-      <c r="H321" s="252" t="str">
+      <c r="H321" s="256" t="str">
         <v>False</v>
       </c>
-      <c r="I321" s="252" t="str">
+      <c r="I321" s="256" t="str">
         <v>False</v>
       </c>
-      <c r="J321" s="252" t="str">
+      <c r="J321" s="256" t="str">
         <v>False</v>
       </c>
-      <c r="K321" s="252" t="str">
+      <c r="K321" s="256" t="str">
         <v>False</v>
       </c>
-      <c r="L321" s="252" t="str">
+      <c r="L321" s="179" t="str">
         <v>False</v>
       </c>
-      <c r="M321" s="255" t="str">
-        <v>True</v>
-      </c>
+      <c r="M321"/>
     </row>
     <row r="322" spans="3:13" x14ac:dyDescent="0.35">
       <c r="C322" s="12" t="str">
         <v>HasInverse</v>
       </c>
-      <c r="D322" s="257" t="str">
+      <c r="D322" s="252" t="str">
         <v>True</v>
       </c>
-      <c r="E322" s="252" t="str">
+      <c r="E322" s="256" t="str">
         <v>True</v>
       </c>
-      <c r="F322" s="252" t="str">
+      <c r="F322" s="256" t="str">
         <v>True</v>
       </c>
-      <c r="G322" s="252" t="str">
+      <c r="G322" s="256" t="str">
         <v>True</v>
       </c>
-      <c r="H322" s="252" t="str">
+      <c r="H322" s="256" t="str">
         <v>True</v>
       </c>
-      <c r="I322" s="252" t="str">
+      <c r="I322" s="256" t="str">
         <v>True</v>
       </c>
-      <c r="J322" s="252" t="str">
+      <c r="J322" s="256" t="str">
         <v>True</v>
       </c>
-      <c r="K322" s="252" t="str">
+      <c r="K322" s="256" t="str">
         <v>True</v>
       </c>
-      <c r="L322" s="252" t="str">
+      <c r="L322" s="179" t="str">
         <v>True</v>
       </c>
-      <c r="M322" s="255" t="str">
-        <v>True</v>
-      </c>
+      <c r="M322"/>
     </row>
     <row r="323" spans="3:13" x14ac:dyDescent="0.35">
       <c r="C323" s="12" t="str">
         <v>MethodName</v>
       </c>
-      <c r="D323" s="257" t="str">
+      <c r="D323" s="252" t="str">
         <v/>
       </c>
-      <c r="E323" s="252" t="str">
+      <c r="E323" s="256" t="str">
         <v/>
       </c>
-      <c r="F323" s="252" t="str">
+      <c r="F323" s="256" t="str">
         <v/>
       </c>
-      <c r="G323" s="252" t="str">
+      <c r="G323" s="256" t="str">
         <v/>
       </c>
-      <c r="H323" s="252" t="str">
+      <c r="H323" s="256" t="str">
         <v/>
       </c>
-      <c r="I323" s="252" t="str">
+      <c r="I323" s="256" t="str">
         <v/>
       </c>
-      <c r="J323" s="252" t="str">
+      <c r="J323" s="256" t="str">
         <v/>
       </c>
-      <c r="K323" s="252" t="str">
+      <c r="K323" s="256" t="str">
         <v/>
       </c>
-      <c r="L323" s="252" t="str">
+      <c r="L323" s="179" t="str">
         <v/>
       </c>
-      <c r="M323" s="255" t="str">
-        <v/>
-      </c>
+      <c r="M323"/>
     </row>
     <row r="324" spans="3:13" x14ac:dyDescent="0.35">
       <c r="C324" s="12" t="str">
         <v>Scope</v>
       </c>
-      <c r="D324" s="257" t="str">
+      <c r="D324" s="252" t="str">
         <v/>
       </c>
-      <c r="E324" s="252" t="str">
+      <c r="E324" s="256" t="str">
         <v/>
       </c>
-      <c r="F324" s="252" t="str">
+      <c r="F324" s="256" t="str">
         <v/>
       </c>
-      <c r="G324" s="252" t="str">
+      <c r="G324" s="256" t="str">
         <v/>
       </c>
-      <c r="H324" s="252" t="str">
+      <c r="H324" s="256" t="str">
         <v/>
       </c>
-      <c r="I324" s="252" t="str">
+      <c r="I324" s="256" t="str">
         <v/>
       </c>
-      <c r="J324" s="252" t="str">
+      <c r="J324" s="256" t="str">
         <v/>
       </c>
-      <c r="K324" s="252" t="str">
+      <c r="K324" s="256" t="str">
         <v/>
       </c>
-      <c r="L324" s="252" t="str">
+      <c r="L324" s="179" t="str">
         <v/>
       </c>
-      <c r="M324" s="255" t="str">
-        <v/>
-      </c>
+      <c r="M324"/>
     </row>
     <row r="325" spans="3:13" x14ac:dyDescent="0.35">
       <c r="C325" s="12" t="str">
         <v>Remarks</v>
       </c>
-      <c r="D325" s="257" t="str">
+      <c r="D325" s="252" t="str">
         <v/>
       </c>
-      <c r="E325" s="252" t="str">
+      <c r="E325" s="256" t="str">
         <v/>
       </c>
-      <c r="F325" s="252" t="str">
+      <c r="F325" s="256" t="str">
         <v/>
       </c>
-      <c r="G325" s="252" t="str">
+      <c r="G325" s="256" t="str">
         <v/>
       </c>
-      <c r="H325" s="252" t="str">
+      <c r="H325" s="256" t="str">
         <v/>
       </c>
-      <c r="I325" s="252" t="str">
+      <c r="I325" s="256" t="str">
         <v/>
       </c>
-      <c r="J325" s="252" t="str">
+      <c r="J325" s="256" t="str">
         <v/>
       </c>
-      <c r="K325" s="252" t="str">
+      <c r="K325" s="256" t="str">
         <v/>
       </c>
-      <c r="L325" s="252" t="str">
+      <c r="L325" s="179" t="str">
         <v/>
       </c>
-      <c r="M325" s="255" t="str">
-        <v/>
-      </c>
+      <c r="M325"/>
     </row>
     <row r="326" spans="3:13" x14ac:dyDescent="0.35">
       <c r="C326" s="12" t="str">
         <v>GridUsages</v>
       </c>
-      <c r="D326" s="257" t="str">
+      <c r="D326" s="252" t="str">
         <v/>
       </c>
-      <c r="E326" s="252" t="str">
+      <c r="E326" s="256" t="str">
         <v/>
       </c>
-      <c r="F326" s="252" t="str">
+      <c r="F326" s="256" t="str">
         <v/>
       </c>
-      <c r="G326" s="252" t="str">
+      <c r="G326" s="256" t="str">
         <v/>
       </c>
-      <c r="H326" s="252" t="str">
+      <c r="H326" s="256" t="str">
         <v/>
       </c>
-      <c r="I326" s="252" t="str">
+      <c r="I326" s="256" t="str">
         <v/>
       </c>
-      <c r="J326" s="252" t="str">
+      <c r="J326" s="256" t="str">
         <v/>
       </c>
-      <c r="K326" s="252" t="str">
+      <c r="K326" s="256" t="str">
         <v/>
       </c>
-      <c r="L326" s="252" t="str">
+      <c r="L326" s="179" t="str">
         <v/>
       </c>
-      <c r="M326" s="255" t="str">
-        <v/>
-      </c>
+      <c r="M326"/>
     </row>
     <row r="327" spans="3:13" x14ac:dyDescent="0.35">
       <c r="C327" s="12" t="str">
         <v>Parameters</v>
       </c>
-      <c r="D327" s="257" t="str">
+      <c r="D327" s="252" t="str">
         <v/>
       </c>
-      <c r="E327" s="252" t="str">
+      <c r="E327" s="256" t="str">
         <v/>
       </c>
-      <c r="F327" s="252" t="str">
+      <c r="F327" s="256" t="str">
         <v/>
       </c>
-      <c r="G327" s="252" t="str">
+      <c r="G327" s="256" t="str">
         <v/>
       </c>
-      <c r="H327" s="252" t="str">
+      <c r="H327" s="256" t="str">
         <v/>
       </c>
-      <c r="I327" s="252" t="str">
+      <c r="I327" s="256" t="str">
         <v/>
       </c>
-      <c r="J327" s="252" t="str">
+      <c r="J327" s="256" t="str">
         <v/>
       </c>
-      <c r="K327" s="252" t="str">
+      <c r="K327" s="256" t="str">
         <v/>
       </c>
-      <c r="L327" s="252" t="str">
+      <c r="L327" s="179" t="str">
         <v/>
       </c>
-      <c r="M327" s="255" t="str">
-        <v/>
-      </c>
+      <c r="M327"/>
     </row>
     <row r="328" spans="3:13" x14ac:dyDescent="0.35">
       <c r="C328" s="12" t="str">
         <v>SourceCRS</v>
       </c>
-      <c r="D328" s="257" t="str">
+      <c r="D328" s="252" t="str">
         <v>NAD27 / Alaska Albers</v>
       </c>
-      <c r="E328" s="252" t="str">
+      <c r="E328" s="256" t="str">
         <v>NAD27 / Alaska Albers</v>
       </c>
-      <c r="F328" s="252" t="str">
+      <c r="F328" s="256" t="str">
         <v>NAD27 / Alaska Albers</v>
       </c>
-      <c r="G328" s="252" t="str">
+      <c r="G328" s="256" t="str">
         <v>NAD27 / Alaska Albers</v>
       </c>
-      <c r="H328" s="252" t="str">
+      <c r="H328" s="256" t="str">
         <v>NAD27 / Alaska Albers</v>
       </c>
-      <c r="I328" s="252" t="str">
+      <c r="I328" s="256" t="str">
         <v>NAD27 / Alaska Albers</v>
       </c>
-      <c r="J328" s="252" t="str">
+      <c r="J328" s="256" t="str">
         <v>NAD27 / Alaska Albers</v>
       </c>
-      <c r="K328" s="252" t="str">
+      <c r="K328" s="256" t="str">
         <v>NAD27 / Alaska Albers</v>
       </c>
-      <c r="L328" s="252" t="str">
+      <c r="L328" s="179" t="str">
         <v>NAD27 / Alaska Albers</v>
       </c>
-      <c r="M328" s="255" t="str">
-        <v>NAD27 / Alaska Albers</v>
-      </c>
+      <c r="M328"/>
     </row>
     <row r="329" spans="3:13" x14ac:dyDescent="0.35">
       <c r="C329" s="12" t="str">
         <v>TargetCRS</v>
       </c>
-      <c r="D329" s="257" t="str">
+      <c r="D329" s="252" t="str">
         <v>WGS 84 (with axis order normalized for visualization)</v>
       </c>
-      <c r="E329" s="252" t="str">
+      <c r="E329" s="256" t="str">
         <v>WGS 84 (with axis order normalized for visualization)</v>
       </c>
-      <c r="F329" s="252" t="str">
+      <c r="F329" s="256" t="str">
         <v>WGS 84 (with axis order normalized for visualization)</v>
       </c>
-      <c r="G329" s="252" t="str">
+      <c r="G329" s="256" t="str">
         <v>WGS 84 (with axis order normalized for visualization)</v>
       </c>
-      <c r="H329" s="252" t="str">
+      <c r="H329" s="256" t="str">
         <v>WGS 84 (with axis order normalized for visualization)</v>
       </c>
-      <c r="I329" s="252" t="str">
+      <c r="I329" s="256" t="str">
         <v>WGS 84 (with axis order normalized for visualization)</v>
       </c>
-      <c r="J329" s="252" t="str">
+      <c r="J329" s="256" t="str">
         <v>WGS 84 (with axis order normalized for visualization)</v>
       </c>
-      <c r="K329" s="252" t="str">
+      <c r="K329" s="256" t="str">
         <v>WGS 84 (with axis order normalized for visualization)</v>
       </c>
-      <c r="L329" s="252" t="str">
+      <c r="L329" s="179" t="str">
         <v>WGS 84 (with axis order normalized for visualization)</v>
       </c>
-      <c r="M329" s="255" t="str">
-        <v>WGS 84 (with axis order normalized for visualization)</v>
-      </c>
+      <c r="M329"/>
     </row>
     <row r="330" spans="3:13" x14ac:dyDescent="0.35">
       <c r="C330" s="12" t="str">
         <v>Context</v>
       </c>
-      <c r="D330" s="257" t="str">
+      <c r="D330" s="252" t="str">
         <v>LogLevel=Error; EndpointUrl=https://cdn.proj.org; EnableNetworkConnections=True</v>
       </c>
-      <c r="E330" s="252" t="str">
+      <c r="E330" s="256" t="str">
         <v>LogLevel=Error; EndpointUrl=https://cdn.proj.org; EnableNetworkConnections=True</v>
       </c>
-      <c r="F330" s="252" t="str">
+      <c r="F330" s="256" t="str">
         <v>LogLevel=Error; EndpointUrl=https://cdn.proj.org; EnableNetworkConnections=True</v>
       </c>
-      <c r="G330" s="252" t="str">
+      <c r="G330" s="256" t="str">
         <v>LogLevel=Error; EndpointUrl=https://cdn.proj.org; EnableNetworkConnections=True</v>
       </c>
-      <c r="H330" s="252" t="str">
+      <c r="H330" s="256" t="str">
         <v>LogLevel=Error; EndpointUrl=https://cdn.proj.org; EnableNetworkConnections=True</v>
       </c>
-      <c r="I330" s="252" t="str">
+      <c r="I330" s="256" t="str">
         <v>LogLevel=Error; EndpointUrl=https://cdn.proj.org; EnableNetworkConnections=True</v>
       </c>
-      <c r="J330" s="252" t="str">
+      <c r="J330" s="256" t="str">
         <v>LogLevel=Error; EndpointUrl=https://cdn.proj.org; EnableNetworkConnections=True</v>
       </c>
-      <c r="K330" s="252" t="str">
+      <c r="K330" s="256" t="str">
         <v>LogLevel=Error; EndpointUrl=https://cdn.proj.org; EnableNetworkConnections=True</v>
       </c>
-      <c r="L330" s="252" t="str">
+      <c r="L330" s="179" t="str">
         <v>LogLevel=Error; EndpointUrl=https://cdn.proj.org; EnableNetworkConnections=True</v>
       </c>
-      <c r="M330" s="255" t="str">
-        <v>LogLevel=Error; EndpointUrl=https://cdn.proj.org; EnableNetworkConnections=True</v>
-      </c>
+      <c r="M330"/>
     </row>
     <row r="331" spans="3:13" x14ac:dyDescent="0.35">
       <c r="C331" s="12" t="str">
         <v>UsageArea.Name</v>
       </c>
-      <c r="D331" s="257" t="str">
+      <c r="D331" s="252" t="str">
         <v>United States (USA) - Alaska including EEZ.</v>
       </c>
-      <c r="E331" s="252" t="str">
+      <c r="E331" s="256" t="str">
         <v>United States (USA) - Alaska mainland.</v>
       </c>
-      <c r="F331" s="252" t="str">
+      <c r="F331" s="256" t="str">
         <v>Canada - onshore - Alberta; British Columbia; Manitoba; New Brunswick; Newfoundland and Labrador; Northwest Territories; Nova Scotia; Nunavut; Ontario; Prince Edward Island; Quebec; Saskatchewan; Yukon; offshore east coast west of 44°W and north of 40°N.</v>
       </c>
-      <c r="G331" s="252" t="str">
+      <c r="G331" s="256" t="str">
         <v>Canada - onshore - Alberta; British Columbia; Manitoba; New Brunswick; Newfoundland and Labrador; Northwest Territories; Nova Scotia; Nunavut; Ontario; Prince Edward Island; Quebec; Saskatchewan; Yukon; offshore east coast west of 44°W and north of 40°N.</v>
       </c>
-      <c r="H331" s="252" t="str">
+      <c r="H331" s="256" t="str">
         <v>Canada - Northwest Territories; Nunavut; Saskatchewan.</v>
       </c>
-      <c r="I331" s="252" t="str">
+      <c r="I331" s="256" t="str">
         <v>Canada - Yukon.</v>
       </c>
-      <c r="J331" s="252" t="str">
+      <c r="J331" s="256" t="str">
         <v>Canada - Alberta; British Columbia.</v>
       </c>
-      <c r="K331" s="252" t="str">
+      <c r="K331" s="256" t="str">
         <v>United States (USA) - Alaska - Aleutian Islands onshore east of 180°E.</v>
       </c>
-      <c r="L331" s="252" t="str">
+      <c r="L331" s="179" t="str">
         <v>United States (USA) - Alaska - Aleutian Islands onshore west of 180°W.</v>
       </c>
-      <c r="M331" s="255" t="str">
-        <v>World</v>
-      </c>
+      <c r="M331"/>
     </row>
     <row r="332" spans="3:13" x14ac:dyDescent="0.35">
       <c r="C332" s="12" t="str">
         <v>UsageArea.WestLongitude</v>
       </c>
-      <c r="D332" s="257" t="str">
+      <c r="D332" s="252" t="str">
         <v>167.65</v>
       </c>
-      <c r="E332" s="252" t="str">
+      <c r="E332" s="256" t="str">
         <v>-168.26</v>
       </c>
-      <c r="F332" s="252" t="str">
+      <c r="F332" s="256" t="str">
         <v>-141.01</v>
       </c>
-      <c r="G332" s="252" t="str">
+      <c r="G332" s="256" t="str">
         <v>-141.01</v>
       </c>
-      <c r="H332" s="252" t="str">
+      <c r="H332" s="256" t="str">
         <v>-136.46</v>
       </c>
-      <c r="I332" s="252" t="str">
+      <c r="I332" s="256" t="str">
         <v>-141.01</v>
       </c>
-      <c r="J332" s="252" t="str">
+      <c r="J332" s="256" t="str">
         <v>-139.04</v>
       </c>
-      <c r="K332" s="252" t="str">
+      <c r="K332" s="256" t="str">
         <v>-178.3</v>
       </c>
-      <c r="L332" s="252" t="str">
+      <c r="L332" s="179" t="str">
         <v>172.42</v>
       </c>
-      <c r="M332" s="255" t="str">
-        <v>-180</v>
-      </c>
+      <c r="M332"/>
     </row>
     <row r="333" spans="3:13" x14ac:dyDescent="0.35">
       <c r="C333" s="12" t="str">
         <v>UsageArea.SouthLatitude</v>
       </c>
-      <c r="D333" s="257" t="str">
+      <c r="D333" s="252" t="str">
         <v>47.88</v>
       </c>
-      <c r="E333" s="252" t="str">
+      <c r="E333" s="256" t="str">
         <v>54.34</v>
       </c>
-      <c r="F333" s="252" t="str">
+      <c r="F333" s="256" t="str">
         <v>40</v>
       </c>
-      <c r="G333" s="252" t="str">
+      <c r="G333" s="256" t="str">
         <v>40</v>
       </c>
-      <c r="H333" s="252" t="str">
+      <c r="H333" s="256" t="str">
         <v>49</v>
       </c>
-      <c r="I333" s="252" t="str">
+      <c r="I333" s="256" t="str">
         <v>59.99</v>
       </c>
-      <c r="J333" s="252" t="str">
+      <c r="J333" s="256" t="str">
         <v>48.25</v>
       </c>
-      <c r="K333" s="252" t="str">
+      <c r="K333" s="256" t="str">
         <v>51.54</v>
       </c>
-      <c r="L333" s="252" t="str">
+      <c r="L333" s="179" t="str">
         <v>51.3</v>
       </c>
-      <c r="M333" s="255" t="str">
-        <v>-90</v>
-      </c>
+      <c r="M333"/>
     </row>
     <row r="334" spans="3:13" x14ac:dyDescent="0.35">
       <c r="C334" s="12" t="str">
         <v>UsageArea.EastLongitude</v>
       </c>
-      <c r="D334" s="257" t="str">
+      <c r="D334" s="252" t="str">
         <v>-129.99</v>
       </c>
-      <c r="E334" s="252" t="str">
+      <c r="E334" s="256" t="str">
         <v>-129.99</v>
       </c>
-      <c r="F334" s="252" t="str">
+      <c r="F334" s="256" t="str">
         <v>-44</v>
       </c>
-      <c r="G334" s="252" t="str">
+      <c r="G334" s="256" t="str">
         <v>-44</v>
       </c>
-      <c r="H334" s="252" t="str">
+      <c r="H334" s="256" t="str">
         <v>-60.72</v>
       </c>
-      <c r="I334" s="252" t="str">
+      <c r="I334" s="256" t="str">
         <v>-123.91</v>
       </c>
-      <c r="J334" s="252" t="str">
+      <c r="J334" s="256" t="str">
         <v>-109.98</v>
       </c>
-      <c r="K334" s="252" t="str">
+      <c r="K334" s="256" t="str">
         <v>-164.84</v>
       </c>
-      <c r="L334" s="252" t="str">
+      <c r="L334" s="179" t="str">
         <v>179.86</v>
       </c>
-      <c r="M334" s="255" t="str">
-        <v>180</v>
-      </c>
+      <c r="M334"/>
     </row>
     <row r="335" spans="3:13" x14ac:dyDescent="0.35">
       <c r="C335" s="12" t="str">
         <v>UsageArea.NorthLatitude</v>
       </c>
-      <c r="D335" s="257" t="str">
+      <c r="D335" s="252" t="str">
         <v>74.71</v>
       </c>
-      <c r="E335" s="252" t="str">
+      <c r="E335" s="256" t="str">
         <v>71.4</v>
       </c>
-      <c r="F335" s="252" t="str">
+      <c r="F335" s="256" t="str">
         <v>83.17</v>
       </c>
-      <c r="G335" s="252" t="str">
+      <c r="G335" s="256" t="str">
         <v>83.17</v>
       </c>
-      <c r="H335" s="252" t="str">
+      <c r="H335" s="256" t="str">
         <v>83.17</v>
       </c>
-      <c r="I335" s="252" t="str">
+      <c r="I335" s="256" t="str">
         <v>69.7</v>
       </c>
-      <c r="J335" s="252" t="str">
+      <c r="J335" s="256" t="str">
         <v>60.01</v>
       </c>
-      <c r="K335" s="252" t="str">
+      <c r="K335" s="256" t="str">
         <v>54.34</v>
       </c>
-      <c r="L335" s="252" t="str">
+      <c r="L335" s="179" t="str">
         <v>53.07</v>
       </c>
-      <c r="M335" s="255" t="str">
-        <v>90</v>
-      </c>
+      <c r="M335"/>
     </row>
     <row r="336" spans="3:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C336" s="13" t="str">
         <v>UsageArea.Center</v>
       </c>
-      <c r="D336" s="258" t="str">
+      <c r="D336" s="253" t="str">
         <v>18.83, 61.295</v>
       </c>
       <c r="E336" s="214" t="str">
@@ -50502,149 +50539,226 @@
       <c r="K336" s="214" t="str">
         <v>-171.57, 52.94</v>
       </c>
-      <c r="L336" s="214" t="str">
+      <c r="L336" s="181" t="str">
         <v>176.14, 52.185</v>
       </c>
-      <c r="M336" s="256" t="str">
-        <v>0, 0</v>
-      </c>
-    </row>
-    <row r="337" spans="3:5" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="338" spans="3:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="M336"/>
+    </row>
+    <row r="337" spans="3:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="M337"/>
+    </row>
+    <row r="338" spans="3:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C338" s="251" t="str" cm="1">
-        <f t="array" ref="C338:D352">_xll.PE.trf.TransformSteps(D311,D312,C313,"proj")</f>
+        <f t="array" ref="C338:F352">_xll.PE.trf.TransformSteps(D311,D312,C313,"proj")</f>
         <v>Step Number</v>
       </c>
       <c r="D338" s="4">
         <v>0</v>
       </c>
-      <c r="E338" s="5"/>
-    </row>
-    <row r="339" spans="3:5" x14ac:dyDescent="0.35">
+      <c r="E338" s="215">
+        <v>1</v>
+      </c>
+      <c r="F338" s="5">
+        <v>2</v>
+      </c>
+      <c r="M338"/>
+    </row>
+    <row r="339" spans="3:13" x14ac:dyDescent="0.35">
       <c r="C339" s="235" t="str">
         <v>Step Identifiers</v>
       </c>
-      <c r="D339" s="178">
-        <v>0</v>
-      </c>
-      <c r="E339" s="179"/>
-    </row>
-    <row r="340" spans="3:5" x14ac:dyDescent="0.35">
+      <c r="D339" s="178" t="str">
+        <v>INVERSE(EPSG)</v>
+      </c>
+      <c r="E339" s="256" t="str">
+        <v>DERIVED_FROM(EPSG)</v>
+      </c>
+      <c r="F339" s="179" t="str">
+        <v>EPSG</v>
+      </c>
+      <c r="M339"/>
+    </row>
+    <row r="340" spans="3:13" x14ac:dyDescent="0.35">
       <c r="C340" s="235" t="str">
         <v>Step Name</v>
       </c>
       <c r="D340" s="178" t="str">
-        <v>&lt;choose-coordinate-transform&gt;</v>
-      </c>
-      <c r="E340" s="179"/>
-    </row>
-    <row r="341" spans="3:5" x14ac:dyDescent="0.35">
+        <v>Inverse of Alaska Albers</v>
+      </c>
+      <c r="E340" s="256" t="str">
+        <v>NAD27 to WGS 84 (10)</v>
+      </c>
+      <c r="F340" s="179" t="str">
+        <v>axis order change (2D)</v>
+      </c>
+    </row>
+    <row r="341" spans="3:13" x14ac:dyDescent="0.35">
       <c r="C341" s="235" t="str">
         <v>Step sccuracy [m]</v>
       </c>
       <c r="D341" s="178">
         <v>55</v>
       </c>
-      <c r="E341" s="179"/>
-    </row>
-    <row r="342" spans="3:5" x14ac:dyDescent="0.35">
+      <c r="E341" s="256">
+        <v>55</v>
+      </c>
+      <c r="F341" s="179">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="342" spans="3:13" x14ac:dyDescent="0.35">
       <c r="C342" s="235" t="str">
         <v>UsageArea</v>
       </c>
       <c r="D342" s="178" t="str">
-        <v>United States (USA) - Alaska including EEZ.</v>
-      </c>
-      <c r="E342" s="179"/>
-    </row>
-    <row r="343" spans="3:5" x14ac:dyDescent="0.35">
+        <v>Unknown</v>
+      </c>
+      <c r="E342" s="256" t="str">
+        <v>Canada - Alberta; British Columbia.</v>
+      </c>
+      <c r="F342" s="179">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="343" spans="3:13" x14ac:dyDescent="0.35">
       <c r="C343" s="235" t="str">
         <v>Scope</v>
       </c>
       <c r="D343" s="178" t="str">
+        <v>Topographic mapping (small scale).</v>
+      </c>
+      <c r="E343" s="256" t="str">
+        <v>Military survey.</v>
+      </c>
+      <c r="F343" s="179" t="str">
         <v>Unknown</v>
       </c>
-      <c r="E343" s="179"/>
-    </row>
-    <row r="344" spans="3:5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="344" spans="3:13" x14ac:dyDescent="0.35">
       <c r="C344" s="235" t="str">
         <v>Remarks</v>
       </c>
       <c r="D344" s="178" t="str">
         <v>None</v>
       </c>
-      <c r="E344" s="179"/>
-    </row>
-    <row r="345" spans="3:5" x14ac:dyDescent="0.35">
+      <c r="E344" s="256" t="str">
+        <v>Derived at 25 stations. Accuracy 8m, 8m and 6m in X, Y and Z axes.</v>
+      </c>
+      <c r="F344" s="179" t="str">
+        <v>None</v>
+      </c>
+    </row>
+    <row r="345" spans="3:13" x14ac:dyDescent="0.35">
       <c r="C345" s="235" t="str">
         <v>UsageArea.WestLongitude</v>
       </c>
       <c r="D345" s="178">
-        <v>167.65</v>
-      </c>
-      <c r="E345" s="179"/>
-    </row>
-    <row r="346" spans="3:5" x14ac:dyDescent="0.35">
+        <v>-1000</v>
+      </c>
+      <c r="E345" s="256">
+        <v>-139.04</v>
+      </c>
+      <c r="F345" s="179">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="346" spans="3:13" x14ac:dyDescent="0.35">
       <c r="C346" s="235" t="str">
         <v>UsageArea.SouthLatitude</v>
       </c>
       <c r="D346" s="178">
-        <v>-129.99</v>
-      </c>
-      <c r="E346" s="179"/>
-    </row>
-    <row r="347" spans="3:5" x14ac:dyDescent="0.35">
+        <v>-1000</v>
+      </c>
+      <c r="E346" s="256">
+        <v>-109.98</v>
+      </c>
+      <c r="F346" s="179">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="347" spans="3:13" x14ac:dyDescent="0.35">
       <c r="C347" s="235" t="str">
         <v>UsageArea.EastLongitude</v>
       </c>
       <c r="D347" s="178">
-        <v>47.88</v>
-      </c>
-      <c r="E347" s="179"/>
-    </row>
-    <row r="348" spans="3:5" x14ac:dyDescent="0.35">
+        <v>-1000</v>
+      </c>
+      <c r="E347" s="256">
+        <v>48.25</v>
+      </c>
+      <c r="F347" s="179">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="348" spans="3:13" x14ac:dyDescent="0.35">
       <c r="C348" s="235" t="str">
         <v>UsageArea.NorthLatitude</v>
       </c>
       <c r="D348" s="178">
-        <v>74.709999999999994</v>
-      </c>
-      <c r="E348" s="179"/>
-    </row>
-    <row r="349" spans="3:5" x14ac:dyDescent="0.35">
+        <v>-1000</v>
+      </c>
+      <c r="E348" s="256">
+        <v>60.01</v>
+      </c>
+      <c r="F348" s="179">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="349" spans="3:13" x14ac:dyDescent="0.35">
       <c r="C349" s="235" t="str">
         <v>Nr grids</v>
       </c>
       <c r="D349" s="178">
-        <v>1</v>
-      </c>
-      <c r="E349" s="179"/>
-    </row>
-    <row r="350" spans="3:5" x14ac:dyDescent="0.35">
+        <v>0</v>
+      </c>
+      <c r="E349" s="256">
+        <v>0</v>
+      </c>
+      <c r="F349" s="179">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="350" spans="3:13" x14ac:dyDescent="0.35">
       <c r="C350" s="235" t="str">
         <v>1st grid</v>
       </c>
       <c r="D350" s="178" t="str">
-        <v/>
-      </c>
-      <c r="E350" s="179"/>
-    </row>
-    <row r="351" spans="3:5" x14ac:dyDescent="0.35">
+        <v>N.A.</v>
+      </c>
+      <c r="E350" s="256" t="str">
+        <v>N.A.</v>
+      </c>
+      <c r="F350" s="179" t="str">
+        <v>N.A.</v>
+      </c>
+    </row>
+    <row r="351" spans="3:13" x14ac:dyDescent="0.35">
       <c r="C351" s="235" t="str">
         <v>2nd grid</v>
       </c>
       <c r="D351" s="178" t="str">
         <v>N.A.</v>
       </c>
-      <c r="E351" s="179"/>
-    </row>
-    <row r="352" spans="3:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="E351" s="256" t="str">
+        <v>N.A.</v>
+      </c>
+      <c r="F351" s="179" t="str">
+        <v>N.A.</v>
+      </c>
+    </row>
+    <row r="352" spans="3:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C352" s="236" t="str">
-        <v>Step ROJ string</v>
-      </c>
-      <c r="D352" s="180">
-        <v>0</v>
-      </c>
-      <c r="E352" s="181"/>
+        <v>Step PROJ string</v>
+      </c>
+      <c r="D352" s="180" t="str">
+        <v>+proj=pipeline +step +proj=unitconvert +xy_in=us-ft +xy_out=m +step +inv +proj=aea +lat_0=50 +lon_0=-154 +lat_1=55 +lat_2=65 +x_0=0 +y_0=0 +ellps=clrk66 +step +proj=unitconvert +xy_in=rad +xy_out=deg +step +proj=axisswap +order=2,1</v>
+      </c>
+      <c r="E352" s="214" t="str">
+        <v>+proj=pipeline +step +proj=axisswap +order=2,1 +step +proj=unitconvert +xy_in=deg +xy_out=rad +step +proj=push +v_3 +step +proj=cart +ellps=clrk66 +step +proj=helmert +x=-7 +y=162 +z=188 +step +inv +proj=cart +ellps=WGS84 +step +proj=pop +v_3 +step +proj=unitconvert +xy_in=rad +xy_out=deg +step +proj=axisswap +order=2,1</v>
+      </c>
+      <c r="F352" s="181" t="str">
+        <v>+proj=axisswap +order=2,1</v>
+      </c>
     </row>
     <row r="354" spans="3:16" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="355" spans="3:16" x14ac:dyDescent="0.35">
@@ -50669,8 +50783,8 @@
     </row>
     <row r="357" spans="3:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C357" s="182" t="str" cm="1">
-        <f t="array" ref="C357">_xll.PE.trf.Options(,,,,,55,,,,,,"Never",,,0,)</f>
-        <v>Authority=EPSG; Area=; Accuracy=55; NoBallparkConversions=False; NoDiscardIfMissing=False; UsePrimaryGridNames=False; UseSuperseded=False; StrictContains=False; IntermediateCrsUsage=Never; BestOnly=False; ForceOver=False; CandidateIndex=0; AllowDeprecatedCrs=False</v>
+        <f t="array" ref="C357">_xll.PE.trf.Options(,,,,,55,,,,,,"Never",,,1,)</f>
+        <v>Authority=EPSG; Area=; Accuracy=55; NoBallparkConversions=False; NoDiscardIfMissing=False; UsePrimaryGridNames=False; UseSuperseded=False; StrictContains=False; IntermediateCrsUsage=Never; BestOnly=False; ForceOver=False; CandidateIndex=1; AllowDeprecatedCrs=False</v>
       </c>
       <c r="D357" s="183"/>
       <c r="E357" s="183"/>
@@ -50688,17 +50802,14 @@
     </row>
     <row r="358" spans="3:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C358" s="223" t="str" cm="1">
-        <f t="array" ref="C358:F380">_xll.PE.trf.TransformList(D355,D356,,"")</f>
+        <f t="array" ref="C358:E380">_xll.PE.trf.TransformList(D355,D356,C357,"")</f>
         <v>Transform Number</v>
       </c>
-      <c r="D358" s="259">
+      <c r="D358" s="4">
         <v>0</v>
       </c>
-      <c r="E358" s="260">
+      <c r="E358" s="5">
         <v>1</v>
-      </c>
-      <c r="F358" s="261">
-        <v>2</v>
       </c>
       <c r="M358"/>
       <c r="O358"/>
@@ -50707,14 +50818,11 @@
       <c r="C359" s="12" t="str">
         <v>Transform Name</v>
       </c>
-      <c r="D359" s="257" t="str">
+      <c r="D359" s="252" t="str">
         <v>Inverse of RD New + Amersfoort to ETRS89 (9) + Belgian Lambert 2008</v>
       </c>
-      <c r="E359" s="252" t="str">
+      <c r="E359" s="179" t="str">
         <v>Inverse of RD New + Amersfoort to ETRS89 (8) + Belgian Lambert 2008</v>
-      </c>
-      <c r="F359" s="179" t="str">
-        <v>Inverse of RD New + Ballpark geographic offset from Amersfoort to ETRS89 + Belgian Lambert 2008</v>
       </c>
       <c r="M359"/>
       <c r="O359"/>
@@ -50723,13 +50831,10 @@
       <c r="C360" s="12" t="str">
         <v>Transform Type</v>
       </c>
-      <c r="D360" s="257" t="str">
+      <c r="D360" s="252" t="str">
         <v>ConcatenatedOperation</v>
       </c>
-      <c r="E360" s="252" t="str">
-        <v>ConcatenatedOperation</v>
-      </c>
-      <c r="F360" s="179" t="str">
+      <c r="E360" s="179" t="str">
         <v>ConcatenatedOperation</v>
       </c>
       <c r="M360"/>
@@ -50738,13 +50843,10 @@
       <c r="C361" s="12" t="str">
         <v>Identifier</v>
       </c>
-      <c r="D361" s="257" t="str">
+      <c r="D361" s="252" t="str">
         <v/>
       </c>
-      <c r="E361" s="252" t="str">
-        <v/>
-      </c>
-      <c r="F361" s="179" t="str">
+      <c r="E361" s="179" t="str">
         <v/>
       </c>
       <c r="M361"/>
@@ -50753,13 +50855,10 @@
       <c r="C362" s="12" t="str">
         <v>Identifiers</v>
       </c>
-      <c r="D362" s="257" t="str">
+      <c r="D362" s="252" t="str">
         <v/>
       </c>
-      <c r="E362" s="252" t="str">
-        <v/>
-      </c>
-      <c r="F362" s="179" t="str">
+      <c r="E362" s="179" t="str">
         <v/>
       </c>
       <c r="M362"/>
@@ -50768,14 +50867,11 @@
       <c r="C363" s="12" t="str">
         <v>Accuracy</v>
       </c>
-      <c r="D363" s="257" t="str">
+      <c r="D363" s="252" t="str">
         <v>0</v>
       </c>
-      <c r="E363" s="252" t="str">
+      <c r="E363" s="179" t="str">
         <v>0.25</v>
-      </c>
-      <c r="F363" s="179" t="str">
-        <v/>
       </c>
       <c r="M363"/>
     </row>
@@ -50783,13 +50879,10 @@
       <c r="C364" s="12" t="str">
         <v>IsAvailable</v>
       </c>
-      <c r="D364" s="257" t="str">
+      <c r="D364" s="252" t="str">
         <v>True</v>
       </c>
-      <c r="E364" s="252" t="str">
-        <v>True</v>
-      </c>
-      <c r="F364" s="179" t="str">
+      <c r="E364" s="179" t="str">
         <v>True</v>
       </c>
       <c r="M364"/>
@@ -50798,14 +50891,11 @@
       <c r="C365" s="12" t="str">
         <v>HasBallParkTransformation</v>
       </c>
-      <c r="D365" s="257" t="str">
+      <c r="D365" s="252" t="str">
         <v>False</v>
       </c>
-      <c r="E365" s="252" t="str">
+      <c r="E365" s="179" t="str">
         <v>False</v>
-      </c>
-      <c r="F365" s="179" t="str">
-        <v>True</v>
       </c>
       <c r="M365"/>
     </row>
@@ -50813,13 +50903,10 @@
       <c r="C366" s="12" t="str">
         <v>HasInverse</v>
       </c>
-      <c r="D366" s="257" t="str">
+      <c r="D366" s="252" t="str">
         <v>True</v>
       </c>
-      <c r="E366" s="252" t="str">
-        <v>True</v>
-      </c>
-      <c r="F366" s="179" t="str">
+      <c r="E366" s="179" t="str">
         <v>True</v>
       </c>
       <c r="M366"/>
@@ -50828,13 +50915,10 @@
       <c r="C367" s="12" t="str">
         <v>MethodName</v>
       </c>
-      <c r="D367" s="257" t="str">
+      <c r="D367" s="252" t="str">
         <v/>
       </c>
-      <c r="E367" s="252" t="str">
-        <v/>
-      </c>
-      <c r="F367" s="179" t="str">
+      <c r="E367" s="179" t="str">
         <v/>
       </c>
       <c r="M367"/>
@@ -50843,13 +50927,10 @@
       <c r="C368" s="12" t="str">
         <v>Scope</v>
       </c>
-      <c r="D368" s="257" t="str">
+      <c r="D368" s="252" t="str">
         <v/>
       </c>
-      <c r="E368" s="252" t="str">
-        <v/>
-      </c>
-      <c r="F368" s="179" t="str">
+      <c r="E368" s="179" t="str">
         <v/>
       </c>
       <c r="M368"/>
@@ -50858,13 +50939,10 @@
       <c r="C369" s="12" t="str">
         <v>Remarks</v>
       </c>
-      <c r="D369" s="257" t="str">
+      <c r="D369" s="252" t="str">
         <v/>
       </c>
-      <c r="E369" s="252" t="str">
-        <v/>
-      </c>
-      <c r="F369" s="179" t="str">
+      <c r="E369" s="179" t="str">
         <v/>
       </c>
       <c r="M369"/>
@@ -50873,13 +50951,10 @@
       <c r="C370" s="12" t="str">
         <v>GridUsages</v>
       </c>
-      <c r="D370" s="257" t="str">
+      <c r="D370" s="252" t="str">
         <v/>
       </c>
-      <c r="E370" s="252" t="str">
-        <v/>
-      </c>
-      <c r="F370" s="179" t="str">
+      <c r="E370" s="179" t="str">
         <v/>
       </c>
       <c r="M370"/>
@@ -50888,13 +50963,10 @@
       <c r="C371" s="12" t="str">
         <v>Parameters</v>
       </c>
-      <c r="D371" s="257" t="str">
+      <c r="D371" s="252" t="str">
         <v/>
       </c>
-      <c r="E371" s="252" t="str">
-        <v/>
-      </c>
-      <c r="F371" s="179" t="str">
+      <c r="E371" s="179" t="str">
         <v/>
       </c>
       <c r="M371"/>
@@ -50903,13 +50975,10 @@
       <c r="C372" s="12" t="str">
         <v>SourceCRS</v>
       </c>
-      <c r="D372" s="257" t="str">
+      <c r="D372" s="252" t="str">
         <v>Amersfoort / RD New</v>
       </c>
-      <c r="E372" s="252" t="str">
-        <v>Amersfoort / RD New</v>
-      </c>
-      <c r="F372" s="179" t="str">
+      <c r="E372" s="179" t="str">
         <v>Amersfoort / RD New</v>
       </c>
       <c r="M372"/>
@@ -50918,13 +50987,10 @@
       <c r="C373" s="12" t="str">
         <v>TargetCRS</v>
       </c>
-      <c r="D373" s="257" t="str">
+      <c r="D373" s="252" t="str">
         <v>ETRS89 / Belgian Lambert 2008</v>
       </c>
-      <c r="E373" s="252" t="str">
-        <v>ETRS89 / Belgian Lambert 2008</v>
-      </c>
-      <c r="F373" s="179" t="str">
+      <c r="E373" s="179" t="str">
         <v>ETRS89 / Belgian Lambert 2008</v>
       </c>
       <c r="M373"/>
@@ -50933,13 +50999,10 @@
       <c r="C374" s="12" t="str">
         <v>Context</v>
       </c>
-      <c r="D374" s="257" t="str">
+      <c r="D374" s="252" t="str">
         <v>LogLevel=Error; EndpointUrl=https://cdn.proj.org; EnableNetworkConnections=True</v>
       </c>
-      <c r="E374" s="252" t="str">
-        <v>LogLevel=Error; EndpointUrl=https://cdn.proj.org; EnableNetworkConnections=True</v>
-      </c>
-      <c r="F374" s="179" t="str">
+      <c r="E374" s="179" t="str">
         <v>LogLevel=Error; EndpointUrl=https://cdn.proj.org; EnableNetworkConnections=True</v>
       </c>
       <c r="M374"/>
@@ -50948,14 +51011,11 @@
       <c r="C375" s="12" t="str">
         <v>UsageArea.Name</v>
       </c>
-      <c r="D375" s="257" t="str">
+      <c r="D375" s="252" t="str">
         <v>Netherlands - onshore, including Waddenzee, Dutch Wadden Islands and 12-mile offshore coastal zone.</v>
       </c>
-      <c r="E375" s="252" t="str">
+      <c r="E375" s="179" t="str">
         <v>Netherlands - onshore, including Waddenzee, Dutch Wadden Islands and 12-mile offshore coastal zone.</v>
-      </c>
-      <c r="F375" s="179" t="str">
-        <v>World</v>
       </c>
       <c r="M375"/>
     </row>
@@ -50963,14 +51023,11 @@
       <c r="C376" s="12" t="str">
         <v>UsageArea.WestLongitude</v>
       </c>
-      <c r="D376" s="257" t="str">
+      <c r="D376" s="252" t="str">
         <v>3.2</v>
       </c>
-      <c r="E376" s="252" t="str">
+      <c r="E376" s="179" t="str">
         <v>3.2</v>
-      </c>
-      <c r="F376" s="179" t="str">
-        <v>-180</v>
       </c>
       <c r="M376"/>
     </row>
@@ -50978,14 +51035,11 @@
       <c r="C377" s="12" t="str">
         <v>UsageArea.SouthLatitude</v>
       </c>
-      <c r="D377" s="257" t="str">
+      <c r="D377" s="252" t="str">
         <v>50.75</v>
       </c>
-      <c r="E377" s="252" t="str">
+      <c r="E377" s="179" t="str">
         <v>50.75</v>
-      </c>
-      <c r="F377" s="179" t="str">
-        <v>-90</v>
       </c>
       <c r="M377"/>
     </row>
@@ -50993,14 +51047,11 @@
       <c r="C378" s="12" t="str">
         <v>UsageArea.EastLongitude</v>
       </c>
-      <c r="D378" s="257" t="str">
+      <c r="D378" s="252" t="str">
         <v>7.22</v>
       </c>
-      <c r="E378" s="252" t="str">
+      <c r="E378" s="179" t="str">
         <v>7.22</v>
-      </c>
-      <c r="F378" s="179" t="str">
-        <v>180</v>
       </c>
       <c r="M378"/>
     </row>
@@ -51008,14 +51059,11 @@
       <c r="C379" s="12" t="str">
         <v>UsageArea.NorthLatitude</v>
       </c>
-      <c r="D379" s="257" t="str">
+      <c r="D379" s="252" t="str">
         <v>53.7</v>
       </c>
-      <c r="E379" s="252" t="str">
+      <c r="E379" s="179" t="str">
         <v>53.7</v>
-      </c>
-      <c r="F379" s="179" t="str">
-        <v>90</v>
       </c>
       <c r="M379"/>
     </row>
@@ -51023,14 +51071,11 @@
       <c r="C380" s="13" t="str">
         <v>UsageArea.Center</v>
       </c>
-      <c r="D380" s="258" t="str">
+      <c r="D380" s="253" t="str">
         <v>5.21, 52.225</v>
       </c>
-      <c r="E380" s="214" t="str">
+      <c r="E380" s="181" t="str">
         <v>5.21, 52.225</v>
-      </c>
-      <c r="F380" s="181" t="str">
-        <v>0, 0</v>
       </c>
       <c r="M380"/>
     </row>
@@ -51039,11 +51084,17 @@
     </row>
     <row r="382" spans="3:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C382" s="251" t="str" cm="1">
-        <f t="array" ref="C382:D396">_xll.PE.trf.TransformSteps(D355,D356,C357,"proj")</f>
+        <f t="array" ref="C382:F396">_xll.PE.trf.TransformSteps(D355,D356,C357,"proj")</f>
         <v>Step Number</v>
       </c>
-      <c r="D382" s="21">
+      <c r="D382" s="4">
         <v>0</v>
+      </c>
+      <c r="E382" s="215">
+        <v>1</v>
+      </c>
+      <c r="F382" s="5">
+        <v>2</v>
       </c>
       <c r="H382" s="182" t="str" cm="1">
         <f t="array" ref="H382:L385">_xll.PE.xfm.ListTransformPipelines(D355,D356)</f>
@@ -51066,8 +51117,14 @@
       <c r="C383" s="235" t="str">
         <v>Step Identifiers</v>
       </c>
-      <c r="D383" s="262">
-        <v>0</v>
+      <c r="D383" s="254" t="str">
+        <v>INVERSE(EPSG)</v>
+      </c>
+      <c r="E383" s="255" t="str">
+        <v>EPSG</v>
+      </c>
+      <c r="F383" s="177" t="str">
+        <v>EPSG</v>
       </c>
       <c r="H383" s="244">
         <v>1</v>
@@ -51089,8 +51146,14 @@
       <c r="C384" s="235" t="str">
         <v>Step Name</v>
       </c>
-      <c r="D384" s="262" t="str">
-        <v>&lt;choose-coordinate-transform&gt;</v>
+      <c r="D384" s="252" t="str">
+        <v>Inverse of RD New</v>
+      </c>
+      <c r="E384" s="172" t="str">
+        <v>Amersfoort to ETRS89 (8)</v>
+      </c>
+      <c r="F384" s="179" t="str">
+        <v>Belgian Lambert 2008</v>
       </c>
       <c r="H384" s="200">
         <v>2</v>
@@ -51112,7 +51175,13 @@
       <c r="C385" s="235" t="str">
         <v>Step sccuracy [m]</v>
       </c>
-      <c r="D385" s="262">
+      <c r="D385" s="252">
+        <v>55</v>
+      </c>
+      <c r="E385" s="172">
+        <v>55</v>
+      </c>
+      <c r="F385" s="179">
         <v>55</v>
       </c>
       <c r="H385">
@@ -51135,40 +51204,70 @@
       <c r="C386" s="235" t="str">
         <v>UsageArea</v>
       </c>
-      <c r="D386" s="262" t="str">
+      <c r="D386" s="252" t="str">
         <v>Netherlands - onshore, including Waddenzee, Dutch Wadden Islands and 12-mile offshore coastal zone.</v>
+      </c>
+      <c r="E386" s="172" t="str">
+        <v>Netherlands - onshore, including Waddenzee, Dutch Wadden Islands and 12-mile offshore coastal zone.</v>
+      </c>
+      <c r="F386" s="179" t="str">
+        <v>Belgium - onshore.</v>
       </c>
     </row>
     <row r="387" spans="3:17" x14ac:dyDescent="0.35">
       <c r="C387" s="235" t="str">
         <v>Scope</v>
       </c>
-      <c r="D387" s="262" t="str">
-        <v>Unknown</v>
+      <c r="D387" s="252" t="str">
+        <v>Engineering survey, topographic mapping.</v>
+      </c>
+      <c r="E387" s="172" t="str">
+        <v>Transformation of coordinates at 0.25m level of accuracy.</v>
+      </c>
+      <c r="F387" s="179" t="str">
+        <v>Engineering survey, topographic mapping.</v>
       </c>
     </row>
     <row r="388" spans="3:17" x14ac:dyDescent="0.35">
       <c r="C388" s="235" t="str">
         <v>Remarks</v>
       </c>
-      <c r="D388" s="262" t="str">
+      <c r="D388" s="252" t="str">
         <v>None</v>
+      </c>
+      <c r="E388" s="172" t="str">
+        <v>Replaces Amersfoort to ETRS89 (5) and (6) (tfm codes 4830 and 4831). Derived using ETRF2000. In official transformation used with an ellipsoidal height of 0m in Amersfoort or 43m in ETRS89 and with an additional correction grid (up to 0.25m).</v>
+      </c>
+      <c r="F388" s="179" t="str">
+        <v>Replaces Lambert 2005.</v>
       </c>
     </row>
     <row r="389" spans="3:17" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C389" s="235" t="str">
         <v>UsageArea.WestLongitude</v>
       </c>
-      <c r="D389" s="262">
+      <c r="D389" s="252">
         <v>3.2</v>
+      </c>
+      <c r="E389" s="172">
+        <v>3.2</v>
+      </c>
+      <c r="F389" s="179">
+        <v>2.5</v>
       </c>
     </row>
     <row r="390" spans="3:17" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C390" s="235" t="str">
         <v>UsageArea.SouthLatitude</v>
       </c>
-      <c r="D390" s="262">
+      <c r="D390" s="252">
         <v>7.22</v>
+      </c>
+      <c r="E390" s="172">
+        <v>7.22</v>
+      </c>
+      <c r="F390" s="179">
+        <v>6.4</v>
       </c>
       <c r="H390" s="182" t="str" cm="1">
         <f t="array" ref="H390:Q393">_xll.PE.trf.ListTransformOptions(D355,D356)</f>
@@ -51206,8 +51305,14 @@
       <c r="C391" s="235" t="str">
         <v>UsageArea.EastLongitude</v>
       </c>
-      <c r="D391" s="262">
+      <c r="D391" s="252">
         <v>50.75</v>
+      </c>
+      <c r="E391" s="172">
+        <v>50.75</v>
+      </c>
+      <c r="F391" s="179">
+        <v>49.5</v>
       </c>
       <c r="H391" s="244">
         <v>0</v>
@@ -51244,34 +51349,40 @@
       <c r="C392" s="235" t="str">
         <v>UsageArea.NorthLatitude</v>
       </c>
-      <c r="D392" s="262">
-        <v>53.7</v>
+      <c r="D392" s="252">
+        <v>0</v>
+      </c>
+      <c r="E392" s="172">
+        <v>0</v>
+      </c>
+      <c r="F392" s="179">
+        <v>0</v>
       </c>
       <c r="H392" s="198">
         <v>1</v>
       </c>
-      <c r="I392" s="253" t="str">
+      <c r="I392" t="str">
         <v>No</v>
       </c>
-      <c r="J392" s="253" t="str">
+      <c r="J392" t="str">
         <v>Inverse of RD New + Amersfoort to ETRS89 (8) + Belgian Lambert 2008</v>
       </c>
-      <c r="K392" s="253" t="str">
+      <c r="K392" t="str">
         <v>ConcatenatedOperation</v>
       </c>
-      <c r="L392" s="253">
+      <c r="L392">
         <v>0.25</v>
       </c>
-      <c r="M392" s="253" t="b">
+      <c r="M392" t="b">
         <v>1</v>
       </c>
-      <c r="N392" s="253" t="b">
+      <c r="N392" t="b">
         <v>0</v>
       </c>
-      <c r="O392" s="253" t="str">
+      <c r="O392" t="str">
         <v>Netherlands - onshore, including Waddenzee, Dutch Wadden Islands and 12-mile offshore coastal zone.</v>
       </c>
-      <c r="P392" s="264" t="str">
+      <c r="P392" s="237" t="str">
         <v>Available; Non-ballpark; Accuracy=0.25; Has usage area</v>
       </c>
       <c r="Q392" s="238" t="str">
@@ -51282,8 +51393,14 @@
       <c r="C393" s="235" t="str">
         <v>Nr grids</v>
       </c>
-      <c r="D393" s="262">
-        <v>1</v>
+      <c r="D393" s="252" t="str">
+        <v>N.A.</v>
+      </c>
+      <c r="E393" s="172" t="str">
+        <v>N.A.</v>
+      </c>
+      <c r="F393" s="179" t="str">
+        <v>N.A.</v>
       </c>
       <c r="H393" s="200">
         <v>2</v>
@@ -51320,23 +51437,41 @@
       <c r="C394" s="235" t="str">
         <v>1st grid</v>
       </c>
-      <c r="D394" s="262" t="str">
-        <v/>
+      <c r="D394" s="252" t="str">
+        <v>N.A.</v>
+      </c>
+      <c r="E394" s="172" t="str">
+        <v>N.A.</v>
+      </c>
+      <c r="F394" s="179" t="str">
+        <v>N.A.</v>
       </c>
     </row>
     <row r="395" spans="3:17" x14ac:dyDescent="0.35">
       <c r="C395" s="235" t="str">
         <v>2nd grid</v>
       </c>
-      <c r="D395" s="262" t="str">
-        <v>N.A.</v>
+      <c r="D395" s="252" t="str">
+        <v>+proj=pipeline +step +inv +proj=sterea +lat_0=52.1561605555556 +lon_0=5.38763888888889 +k=0.9999079 +x_0=155000 +y_0=463000 +ellps=bessel +step +proj=unitconvert +xy_in=rad +xy_out=deg +step +proj=axisswap +order=2,1</v>
+      </c>
+      <c r="E395" s="172" t="str">
+        <v>+proj=pipeline +step +proj=axisswap +order=2,1 +step +proj=unitconvert +xy_in=deg +xy_out=rad +step +proj=push +v_3 +step +proj=cart +ellps=bessel +step +proj=helmert +x=565.7381 +y=50.4018 +z=465.2904 +rx=0.395025981036064 +ry=-0.330772431242031 +rz=1.87607329462821 +s=4.07244 +convention=coordinate_frame +step +inv +proj=cart +ellps=GRS80 +step +proj=pop +v_3 +step +proj=unitconvert +xy_in=rad +xy_out=deg +step +proj=axisswap +order=2,1</v>
+      </c>
+      <c r="F395" s="179" t="str">
+        <v>+proj=pipeline +step +proj=axisswap +order=2,1 +step +proj=unitconvert +xy_in=deg +xy_out=rad +step +proj=lcc +lat_0=50.797815 +lon_0=4.35921583333333 +lat_1=49.8333333333333 +lat_2=51.1666666666667 +x_0=649328 +y_0=665262 +ellps=GRS80</v>
       </c>
     </row>
     <row r="396" spans="3:17" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C396" s="236" t="str">
         <v>Step ROJ string</v>
       </c>
-      <c r="D396" s="263">
+      <c r="D396" s="253">
+        <v>0</v>
+      </c>
+      <c r="E396" s="214">
+        <v>0</v>
+      </c>
+      <c r="F396" s="181">
         <v>0</v>
       </c>
     </row>

</xml_diff>